<commit_message>
Separate the two enforcement questions in the design document, and add memory.
Section 3's last column becomes grant list granularity, section 4's stays
the control enforcement question, and each says what the other is not.
Ask what the agent remembers between runs, and how a prompt-enforced
control is itself controlled. Move the classification field below the test
so the answer is read off the floors. Say that a new model version changes
the sign-off record, not this document. Widen the tables and update the
workbook to match.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1 Agent Design" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2 Classification" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2a Floor Anchors" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="3 Platform &amp; Sign-off" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="4 Monitoring" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="5 Audit &amp; Assurance" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="6 Reference" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Agent Design" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Classification" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2a Floor Anchors" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Platform &amp; Sign-off" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Monitoring" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Audit &amp; Assurance" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Reference" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'1 Agent Design'!$1:$2</definedName>
@@ -409,7 +409,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -424,14 +424,14 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
       </blipFill>
       <spPr>
-        <a:prstGeom prst="rect"/>
-        <a:ln>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
@@ -974,7 +974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G83"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>Where the limit is enforced</t>
+          <t>Grant list granularity</t>
         </is>
       </c>
       <c r="G34" s="15" t="n"/>
@@ -1430,20 +1430,20 @@
     <row r="44" ht="64" customHeight="1">
       <c r="A44" s="10" t="inlineStr">
         <is>
+          <t>What the agent remembers between runs. Conversation history, retrieved documents, learned preferences, or a store it writes to itself. Say who that memory is scoped to — one user, one account, or everybody — and how long it is kept. Write "nothing" if every run starts clean.</t>
+        </is>
+      </c>
+      <c r="B44" s="10" t="n"/>
+      <c r="C44" s="35" t="n"/>
+      <c r="D44" s="35" t="n"/>
+      <c r="E44" s="35" t="n"/>
+      <c r="F44" s="35" t="n"/>
+      <c r="G44" s="35" t="n"/>
+    </row>
+    <row r="45" ht="64" customHeight="1">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
           <t>Other agents it calls, and agents that call it. Name the agent, not the tools behind it. Say whose authority an incoming call runs under, and what this agent does when it cannot tell.</t>
-        </is>
-      </c>
-      <c r="B44" s="15" t="n"/>
-      <c r="C44" s="35" t="n"/>
-      <c r="D44" s="36" t="n"/>
-      <c r="E44" s="36" t="n"/>
-      <c r="F44" s="36" t="n"/>
-      <c r="G44" s="34" t="n"/>
-    </row>
-    <row r="45" ht="56" customHeight="1">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>What the agent must never reach</t>
         </is>
       </c>
       <c r="B45" s="15" t="n"/>
@@ -1453,78 +1453,82 @@
       <c r="F45" s="36" t="n"/>
       <c r="G45" s="34" t="n"/>
     </row>
-    <row r="46" ht="13" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
+    <row r="46" ht="56" customHeight="1">
+      <c r="A46" s="10" t="inlineStr">
+        <is>
+          <t>What the agent must never reach</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="n"/>
+      <c r="C46" s="35" t="n"/>
+      <c r="D46" s="36" t="n"/>
+      <c r="E46" s="36" t="n"/>
+      <c r="F46" s="36" t="n"/>
+      <c r="G46" s="34" t="n"/>
+    </row>
+    <row r="47" ht="13" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>Even though its credentials or its host could technically get there. Say where that refusal is enforced.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="56" customHeight="1">
-      <c r="A47" s="10" t="inlineStr">
+    <row r="48" ht="56" customHeight="1">
+      <c r="A48" s="10" t="inlineStr">
         <is>
           <t>Value ceiling</t>
         </is>
       </c>
-      <c r="B47" s="15" t="n"/>
-      <c r="C47" s="35" t="n"/>
-      <c r="D47" s="36" t="n"/>
-      <c r="E47" s="36" t="n"/>
-      <c r="F47" s="36" t="n"/>
-      <c r="G47" s="34" t="n"/>
-    </row>
-    <row r="48" ht="13" customHeight="1">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="B48" s="15" t="n"/>
+      <c r="C48" s="35" t="n"/>
+      <c r="D48" s="36" t="n"/>
+      <c r="E48" s="36" t="n"/>
+      <c r="F48" s="36" t="n"/>
+      <c r="G48" s="34" t="n"/>
+    </row>
+    <row r="49" ht="13" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
         <is>
           <t>The most money or value the agent can move in one action, and in one day. Write "none" if there is no ceiling, and expect the Classification sheet to charge you for it.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="26" customHeight="1">
-      <c r="A49" s="32" t="n"/>
-      <c r="B49" s="32" t="n"/>
-      <c r="C49" s="32" t="n"/>
-      <c r="D49" s="32" t="n"/>
-      <c r="E49" s="32" t="n"/>
-      <c r="F49" s="32" t="n"/>
-      <c r="G49" s="32" t="n"/>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="9" t="inlineStr">
+    <row r="50" ht="26" customHeight="1">
+      <c r="A50" s="32" t="n"/>
+      <c r="B50" s="32" t="n"/>
+      <c r="C50" s="32" t="n"/>
+      <c r="D50" s="32" t="n"/>
+      <c r="E50" s="32" t="n"/>
+      <c r="F50" s="32" t="n"/>
+      <c r="G50" s="32" t="n"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="9" t="inlineStr">
         <is>
           <t>4.  What it decides alone</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="14" t="inlineStr">
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="14" t="inlineStr">
         <is>
           <t>Action or decision</t>
         </is>
       </c>
-      <c r="B51" s="14" t="inlineStr">
+      <c r="B52" s="14" t="inlineStr">
         <is>
           <t>Alone, never, or needs approval</t>
         </is>
       </c>
-      <c r="C51" s="14" t="inlineStr">
-        <is>
-          <t>Where that is enforced</t>
-        </is>
-      </c>
-      <c r="D51" s="16" t="n"/>
-      <c r="E51" s="16" t="n"/>
-      <c r="F51" s="16" t="n"/>
-      <c r="G51" s="15" t="n"/>
-    </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="35" t="n"/>
-      <c r="B52" s="35" t="n"/>
-      <c r="C52" s="35" t="n"/>
-      <c r="D52" s="36" t="n"/>
-      <c r="E52" s="36" t="n"/>
-      <c r="F52" s="36" t="n"/>
-      <c r="G52" s="34" t="n"/>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>Where the control is enforced</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="n"/>
+      <c r="E52" s="16" t="n"/>
+      <c r="F52" s="16" t="n"/>
+      <c r="G52" s="15" t="n"/>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="35" t="n"/>
@@ -1589,53 +1593,55 @@
       <c r="F59" s="36" t="n"/>
       <c r="G59" s="34" t="n"/>
     </row>
-    <row r="60" ht="14" customHeight="1">
-      <c r="A60" s="13" t="inlineStr">
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="35" t="n"/>
+      <c r="B60" s="35" t="n"/>
+      <c r="C60" s="35" t="n"/>
+      <c r="D60" s="36" t="n"/>
+      <c r="E60" s="36" t="n"/>
+      <c r="F60" s="36" t="n"/>
+      <c r="G60" s="34" t="n"/>
+    </row>
+    <row r="61" ht="14" customHeight="1">
+      <c r="A61" s="13" t="inlineStr">
         <is>
           <t>Enforcement is one of four answers: in the prompt, in the tool layer, in the platform, or nowhere. "In the prompt" counts, and it is the weakest of the four.</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="26" customHeight="1">
-      <c r="A61" s="32" t="n"/>
-      <c r="B61" s="32" t="n"/>
-      <c r="C61" s="32" t="n"/>
-      <c r="D61" s="32" t="n"/>
-      <c r="E61" s="32" t="n"/>
-      <c r="F61" s="32" t="n"/>
-      <c r="G61" s="32" t="n"/>
-    </row>
-    <row r="62" ht="22" customHeight="1">
-      <c r="A62" s="9" t="inlineStr">
+    <row r="62" ht="64" customHeight="1">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>If any row above says "In the prompt", say how the prompt is controlled. Where it lives, who can change it, and whether a change is reviewed before it reaches production. A control written into a prompt that anybody can edit is not a weak control, it is a removable one, and nothing in section 7 will show you that it went.</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="n"/>
+      <c r="C62" s="35" t="n"/>
+      <c r="D62" s="35" t="n"/>
+      <c r="E62" s="35" t="n"/>
+      <c r="F62" s="35" t="n"/>
+      <c r="G62" s="35" t="n"/>
+    </row>
+    <row r="63" ht="26" customHeight="1">
+      <c r="A63" s="32" t="n"/>
+      <c r="B63" s="32" t="n"/>
+      <c r="C63" s="32" t="n"/>
+      <c r="D63" s="32" t="n"/>
+      <c r="E63" s="32" t="n"/>
+      <c r="F63" s="32" t="n"/>
+      <c r="G63" s="32" t="n"/>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="9" t="inlineStr">
         <is>
           <t>5.  Escalation and override</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="56" customHeight="1">
-      <c r="A63" s="10" t="inlineStr">
-        <is>
-          <t>How the agent hands work to a person</t>
-        </is>
-      </c>
-      <c r="B63" s="15" t="n"/>
-      <c r="C63" s="35" t="n"/>
-      <c r="D63" s="36" t="n"/>
-      <c r="E63" s="36" t="n"/>
-      <c r="F63" s="36" t="n"/>
-      <c r="G63" s="34" t="n"/>
-    </row>
-    <row r="64" ht="13" customHeight="1">
-      <c r="A64" s="13" t="inlineStr">
-        <is>
-          <t>What triggers it, who receives it, in which channel, and what happens if nobody answers.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="56" customHeight="1">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>How a person stops the agent</t>
+          <t>How the agent hands work to a person</t>
         </is>
       </c>
       <c r="B65" s="15" t="n"/>
@@ -1648,14 +1654,14 @@
     <row r="66" ht="13" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
-          <t>The specific action, who can take it, and how long it takes to have effect. Include how a run already in progress is stopped.</t>
+          <t>What triggers it, who receives it, in which channel, and what happens if nobody answers.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="56" customHeight="1">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>How a person reverses what it already did</t>
+          <t>How a person stops the agent</t>
         </is>
       </c>
       <c r="B67" s="15" t="n"/>
@@ -1668,14 +1674,14 @@
     <row r="68" ht="13" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
-          <t>Per row of section 3 where the answer differs.</t>
+          <t>The specific action, who can take it, and how long it takes to have effect. Include how a run already in progress is stopped.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="56" customHeight="1">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>Who is told when it fails</t>
+          <t>How a person reverses what it already did</t>
         </is>
       </c>
       <c r="B69" s="15" t="n"/>
@@ -1688,79 +1694,81 @@
     <row r="70" ht="13" customHeight="1">
       <c r="A70" s="13" t="inlineStr">
         <is>
+          <t>Per row of section 3 where the answer differs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="56" customHeight="1">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>Who is told when it fails</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="n"/>
+      <c r="C71" s="35" t="n"/>
+      <c r="D71" s="36" t="n"/>
+      <c r="E71" s="36" t="n"/>
+      <c r="F71" s="36" t="n"/>
+      <c r="G71" s="34" t="n"/>
+    </row>
+    <row r="72" ht="13" customHeight="1">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
           <t>The person, the channel, and the time within which they are told.</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="26" customHeight="1">
-      <c r="A71" s="32" t="n"/>
-      <c r="B71" s="32" t="n"/>
-      <c r="C71" s="32" t="n"/>
-      <c r="D71" s="32" t="n"/>
-      <c r="E71" s="32" t="n"/>
-      <c r="F71" s="32" t="n"/>
-      <c r="G71" s="32" t="n"/>
-    </row>
-    <row r="72" ht="22" customHeight="1">
-      <c r="A72" s="9" t="inlineStr">
+    <row r="73" ht="26" customHeight="1">
+      <c r="A73" s="32" t="n"/>
+      <c r="B73" s="32" t="n"/>
+      <c r="C73" s="32" t="n"/>
+      <c r="D73" s="32" t="n"/>
+      <c r="E73" s="32" t="n"/>
+      <c r="F73" s="32" t="n"/>
+      <c r="G73" s="32" t="n"/>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="9" t="inlineStr">
         <is>
           <t>6.  Classification and the Classification Test  →  see the Classification sheet</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="22" customHeight="1">
-      <c r="A73" s="9" t="inlineStr">
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="9" t="inlineStr">
         <is>
           <t>7.  Revision history</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="20" customHeight="1">
-      <c r="A74" s="14" t="inlineStr">
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B74" s="14" t="inlineStr">
+      <c r="B76" s="14" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="C74" s="14" t="inlineStr">
+      <c r="C76" s="14" t="inlineStr">
         <is>
           <t>What changed</t>
         </is>
       </c>
-      <c r="D74" s="14" t="inlineStr">
+      <c r="D76" s="14" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="E74" s="14" t="inlineStr">
+      <c r="E76" s="14" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="F74" s="15" t="n"/>
-      <c r="G74" s="14" t="n"/>
-    </row>
-    <row r="75" ht="26" customHeight="1">
-      <c r="A75" s="35" t="n"/>
-      <c r="B75" s="35" t="n"/>
-      <c r="C75" s="35" t="n"/>
-      <c r="D75" s="35" t="n"/>
-      <c r="E75" s="35" t="n"/>
-      <c r="F75" s="34" t="n"/>
-      <c r="G75" s="35" t="n"/>
-    </row>
-    <row r="76" ht="26" customHeight="1">
-      <c r="A76" s="35" t="n"/>
-      <c r="B76" s="35" t="n"/>
-      <c r="C76" s="35" t="n"/>
-      <c r="D76" s="35" t="n"/>
-      <c r="E76" s="35" t="n"/>
-      <c r="F76" s="34" t="n"/>
-      <c r="G76" s="35" t="n"/>
+      <c r="F76" s="15" t="n"/>
+      <c r="G76" s="14" t="n"/>
     </row>
     <row r="77" ht="26" customHeight="1">
       <c r="A77" s="35" t="n"/>
@@ -1816,19 +1824,36 @@
       <c r="F82" s="34" t="n"/>
       <c r="G82" s="35" t="n"/>
     </row>
-    <row r="83">
-      <c r="A83" s="13" t="inlineStr">
-        <is>
-          <t>One more tool, a widened scope, or a new audience all produce a row. A new model version changes the Platform and Sign-off Record instead, not this document.</t>
+    <row r="83" ht="26" customHeight="1">
+      <c r="A83" s="35" t="n"/>
+      <c r="B83" s="35" t="n"/>
+      <c r="C83" s="35" t="n"/>
+      <c r="D83" s="35" t="n"/>
+      <c r="E83" s="35" t="n"/>
+      <c r="F83" s="34" t="n"/>
+      <c r="G83" s="35" t="n"/>
+    </row>
+    <row r="84" ht="26" customHeight="1">
+      <c r="A84" s="35" t="n"/>
+      <c r="B84" s="35" t="n"/>
+      <c r="C84" s="35" t="n"/>
+      <c r="D84" s="35" t="n"/>
+      <c r="E84" s="35" t="n"/>
+      <c r="F84" s="34" t="n"/>
+      <c r="G84" s="35" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="13" t="inlineStr">
+        <is>
+          <t>One more tool, a widened scope, or a new audience all produce a row. So do stage 4 and stage 5 findings: an eval that catches drift, an audit finding against your classification criteria, or a monitor reporting a tool call outside section 3. A new model version does not; that changes the Platform and Sign-off Record instead. Retiring the agent produces the last row: set Status above to retired, date it, and fill in section E of the Audit &amp; Assurance sheet.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="96">
+  <mergeCells count="100">
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="C58:G58"/>
-    <mergeCell ref="A62:G62"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="C45:G45"/>
     <mergeCell ref="A19:G19"/>
@@ -1836,38 +1861,42 @@
     <mergeCell ref="E79:F79"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C65:G65"/>
-    <mergeCell ref="C47:G47"/>
-    <mergeCell ref="A48:G48"/>
     <mergeCell ref="C44:G44"/>
+    <mergeCell ref="C60:G60"/>
+    <mergeCell ref="C71:G71"/>
     <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="A62:B62"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C57:G57"/>
-    <mergeCell ref="E75:F75"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="C18:G18"/>
     <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A48:B48"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="F34:G34"/>
     <mergeCell ref="A45:B45"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="C20:G20"/>
-    <mergeCell ref="A83:G83"/>
+    <mergeCell ref="A46:B46"/>
     <mergeCell ref="F42:G42"/>
     <mergeCell ref="C22:G22"/>
+    <mergeCell ref="A49:G49"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="C59:G59"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="C12:G12"/>
-    <mergeCell ref="C51:G51"/>
+    <mergeCell ref="C46:G46"/>
+    <mergeCell ref="A71:B71"/>
     <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C48:G48"/>
+    <mergeCell ref="A75:G75"/>
     <mergeCell ref="F39:G39"/>
     <mergeCell ref="E76:F76"/>
-    <mergeCell ref="A63:B63"/>
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="E83:F83"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="C26:G26"/>
     <mergeCell ref="A69:B69"/>
@@ -1875,7 +1904,7 @@
     <mergeCell ref="C16:G16"/>
     <mergeCell ref="F36:G36"/>
     <mergeCell ref="C55:G55"/>
-    <mergeCell ref="A60:G60"/>
+    <mergeCell ref="E84:F84"/>
     <mergeCell ref="E78:F78"/>
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="A12:B12"/>
@@ -1887,13 +1916,14 @@
     <mergeCell ref="C52:G52"/>
     <mergeCell ref="A66:G66"/>
     <mergeCell ref="C67:G67"/>
-    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="E81:F81"/>
     <mergeCell ref="C28:G28"/>
-    <mergeCell ref="E81:F81"/>
     <mergeCell ref="A67:B67"/>
     <mergeCell ref="C69:G69"/>
+    <mergeCell ref="A47:G47"/>
     <mergeCell ref="C30:G30"/>
     <mergeCell ref="C6:G6"/>
+    <mergeCell ref="C62:G62"/>
     <mergeCell ref="A72:G72"/>
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="F40:G40"/>
@@ -1903,25 +1933,25 @@
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="C54:G54"/>
-    <mergeCell ref="C63:G63"/>
+    <mergeCell ref="A64:G64"/>
     <mergeCell ref="A15:G15"/>
-    <mergeCell ref="A64:G64"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A73:G73"/>
     <mergeCell ref="F41:G41"/>
-    <mergeCell ref="E74:F74"/>
+    <mergeCell ref="A51:G51"/>
     <mergeCell ref="F35:G35"/>
     <mergeCell ref="C56:G56"/>
+    <mergeCell ref="A61:G61"/>
     <mergeCell ref="A70:G70"/>
     <mergeCell ref="F38:G38"/>
-    <mergeCell ref="A47:B47"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="F37:G37"/>
+    <mergeCell ref="A74:G74"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="C53:G53"/>
     <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A85:G85"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation sqref="C35:C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1930,10 +1960,10 @@
     <dataValidation sqref="F35:F42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Tool level,Data level,Not enforceable here"</formula1>
     </dataValidation>
-    <dataValidation sqref="B52:B59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B53:B60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"May do alone,May never do,Needs a person to approve"</formula1>
     </dataValidation>
-    <dataValidation sqref="C52:C59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C53:C60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"In the platform,In the tool layer,In the prompt,Nowhere"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2367,7 +2397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2701,12 +2731,20 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>These anchors are a copy. The authoritative version is part 2 of your Risk Classifications standard. If that has been revised and this sheet has not, use theirs, and rewrite this sheet to match.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="4">
-    <mergeCell ref="A17:F17"/>
+  <mergeCells count="5">
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Align the classification tables with the test, and give the level gap a home.
Add the four test questions the classification tables were missing, so the
starter tables and the anchors cover the same eight. Rename the trigger row
to say what it does, and require classifications to be strictly ordered so
the highest-floor rule can resolve. Make question 4 judge the shape of a
spending control rather than name an amount, since the amount is per agent.
Add the level gap block to section C of the sign-off record, including the
count of consecutive sign-offs that accepted the same gap. Update the
workbook to match.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -1433,12 +1433,12 @@
           <t>What the agent remembers between runs. Conversation history, retrieved documents, learned preferences, or a store it writes to itself. Say who that memory is scoped to — one user, one account, or everybody — and how long it is kept. Write "nothing" if every run starts clean.</t>
         </is>
       </c>
-      <c r="B44" s="10" t="n"/>
+      <c r="B44" s="15" t="n"/>
       <c r="C44" s="35" t="n"/>
-      <c r="D44" s="35" t="n"/>
-      <c r="E44" s="35" t="n"/>
-      <c r="F44" s="35" t="n"/>
-      <c r="G44" s="35" t="n"/>
+      <c r="D44" s="36" t="n"/>
+      <c r="E44" s="36" t="n"/>
+      <c r="F44" s="36" t="n"/>
+      <c r="G44" s="34" t="n"/>
     </row>
     <row r="45" ht="64" customHeight="1">
       <c r="A45" s="10" t="inlineStr">
@@ -1615,12 +1615,12 @@
           <t>If any row above says "In the prompt", say how the prompt is controlled. Where it lives, who can change it, and whether a change is reviewed before it reaches production. A control written into a prompt that anybody can edit is not a weak control, it is a removable one, and nothing in section 7 will show you that it went.</t>
         </is>
       </c>
-      <c r="B62" s="10" t="n"/>
+      <c r="B62" s="15" t="n"/>
       <c r="C62" s="35" t="n"/>
-      <c r="D62" s="35" t="n"/>
-      <c r="E62" s="35" t="n"/>
-      <c r="F62" s="35" t="n"/>
-      <c r="G62" s="35" t="n"/>
+      <c r="D62" s="36" t="n"/>
+      <c r="E62" s="36" t="n"/>
+      <c r="F62" s="36" t="n"/>
+      <c r="G62" s="34" t="n"/>
     </row>
     <row r="63" ht="26" customHeight="1">
       <c r="A63" s="32" t="n"/>
@@ -2582,12 +2582,12 @@
       </c>
       <c r="D11" s="35" t="inlineStr">
         <is>
-          <t>Within a ceiling a manager can approve as ordinary spend.</t>
+          <t>It moves money or value within a ceiling that covers both one action and one day, recorded in its design document.</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Above that ceiling, or the ceiling is per action with no daily limit.</t>
+          <t>The ceiling covers one action but not one day, or nothing approves the actions that reach it.</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
@@ -2727,7 +2727,7 @@
     <row r="17" ht="44" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Question 4 needs your own two numbers, per action and per day. Put them here and in your Risk Classifications standard, so the same numbers govern every agent. Question 7 is the one row where the anchors describe supervision instead of damage: it is what turns the other seven into risk.</t>
+          <t>Question 4 sets no amount, and this pack names none. What a given agent may move is the value ceiling in section 3 of its Agent Design sheet, accepted by whoever signs it off. The anchors judge the shape of the control instead: whether a ceiling exists, whether it covers a day as well as an action, and whether the platform enforces it or the agent is trusted to observe it. Question 7 is the one row where the anchors describe supervision instead of damage: it is what turns the other seven into risk.</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3302,123 +3302,151 @@
       <c r="E52" s="36" t="n"/>
       <c r="F52" s="34" t="n"/>
     </row>
-    <row r="53" ht="26" customHeight="1">
-      <c r="A53" s="32" t="n"/>
-      <c r="B53" s="32" t="n"/>
-      <c r="C53" s="32" t="n"/>
-      <c r="D53" s="32" t="n"/>
-      <c r="E53" s="32" t="n"/>
-      <c r="F53" s="32" t="n"/>
-    </row>
-    <row r="54" ht="26" customHeight="1">
-      <c r="A54" s="24" t="inlineStr">
-        <is>
-          <t>The sign-off is against the two versions named above. When live behavior stops matching the description it was granted against, it is void until somebody looks again.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="32" t="n"/>
-      <c r="B55" s="32" t="n"/>
-      <c r="C55" s="32" t="n"/>
-      <c r="D55" s="32" t="n"/>
-      <c r="E55" s="32" t="n"/>
-      <c r="F55" s="32" t="n"/>
-    </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="9" t="inlineStr">
-        <is>
-          <t>D.  Revision history</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="28" customHeight="1">
-      <c r="A57" s="14" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B57" s="14" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
-      <c r="C57" s="14" t="inlineStr">
-        <is>
-          <t>What changed</t>
-        </is>
-      </c>
-      <c r="D57" s="14" t="inlineStr">
-        <is>
-          <t>Why</t>
-        </is>
-      </c>
-      <c r="E57" s="14" t="inlineStr">
-        <is>
-          <t>Who</t>
-        </is>
-      </c>
-      <c r="F57" s="14" t="inlineStr">
-        <is>
-          <t>Did it need a new sign-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="26" customHeight="1">
-      <c r="A58" s="35" t="n"/>
-      <c r="B58" s="35" t="n"/>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="24" t="inlineStr">
+        <is>
+          <t>THE LEVEL GAP.  The agent's classification names a platform control level and a monitoring level that an agent in it requires. Where the level applied is lower, the gap is accepted here, by name, or it is not accepted at all.</t>
+        </is>
+      </c>
+      <c r="B53" s="24" t="n"/>
+      <c r="C53" s="24" t="n"/>
+      <c r="D53" s="24" t="n"/>
+      <c r="E53" s="24" t="n"/>
+      <c r="F53" s="24" t="n"/>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>Platform control level the classification requires, and the level applied</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="n"/>
+      <c r="C54" s="35" t="n"/>
+      <c r="D54" s="35" t="n"/>
+      <c r="E54" s="35" t="n"/>
+      <c r="F54" s="35" t="n"/>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>Monitoring level the classification requires, and the level applied</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="n"/>
+      <c r="C55" s="35" t="n"/>
+      <c r="D55" s="35" t="n"/>
+      <c r="E55" s="35" t="n"/>
+      <c r="F55" s="35" t="n"/>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>Who accepts the gap, by name</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="n"/>
+      <c r="C56" s="35" t="n"/>
+      <c r="D56" s="35" t="n"/>
+      <c r="E56" s="35" t="n"/>
+      <c r="F56" s="35" t="n"/>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>The date by which it closes</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="n"/>
+      <c r="C57" s="35" t="n"/>
+      <c r="D57" s="35" t="n"/>
+      <c r="E57" s="35" t="n"/>
+      <c r="F57" s="35" t="n"/>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>How many consecutive sign-offs have accepted this same gap</t>
+        </is>
+      </c>
+      <c r="B58" s="10" t="n"/>
       <c r="C58" s="35" t="n"/>
       <c r="D58" s="35" t="n"/>
       <c r="E58" s="35" t="n"/>
       <c r="F58" s="35" t="n"/>
     </row>
     <row r="59" ht="26" customHeight="1">
-      <c r="A59" s="35" t="n"/>
-      <c r="B59" s="35" t="n"/>
-      <c r="C59" s="35" t="n"/>
-      <c r="D59" s="35" t="n"/>
-      <c r="E59" s="35" t="n"/>
-      <c r="F59" s="35" t="n"/>
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>Answer the last row honestly. A gap accepted once is a legitimate decision made under time pressure. A gap accepted three times in a row is a decision nobody is making, and this count is the only thing on any of these forms that would show it.</t>
+        </is>
+      </c>
+      <c r="B59" s="13" t="n"/>
+      <c r="C59" s="13" t="n"/>
+      <c r="D59" s="13" t="n"/>
+      <c r="E59" s="13" t="n"/>
+      <c r="F59" s="13" t="n"/>
     </row>
     <row r="60" ht="26" customHeight="1">
-      <c r="A60" s="35" t="n"/>
-      <c r="B60" s="35" t="n"/>
-      <c r="C60" s="35" t="n"/>
-      <c r="D60" s="35" t="n"/>
-      <c r="E60" s="35" t="n"/>
-      <c r="F60" s="35" t="n"/>
+      <c r="A60" s="32" t="n"/>
+      <c r="B60" s="32" t="n"/>
+      <c r="C60" s="32" t="n"/>
+      <c r="D60" s="32" t="n"/>
+      <c r="E60" s="32" t="n"/>
+      <c r="F60" s="32" t="n"/>
     </row>
     <row r="61" ht="26" customHeight="1">
-      <c r="A61" s="35" t="n"/>
-      <c r="B61" s="35" t="n"/>
-      <c r="C61" s="35" t="n"/>
-      <c r="D61" s="35" t="n"/>
-      <c r="E61" s="35" t="n"/>
-      <c r="F61" s="35" t="n"/>
+      <c r="A61" s="24" t="inlineStr">
+        <is>
+          <t>The sign-off is against the two versions named above. When live behavior stops matching the description it was granted against, it is void until somebody looks again.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="26" customHeight="1">
-      <c r="A62" s="35" t="n"/>
-      <c r="B62" s="35" t="n"/>
-      <c r="C62" s="35" t="n"/>
-      <c r="D62" s="35" t="n"/>
-      <c r="E62" s="35" t="n"/>
-      <c r="F62" s="35" t="n"/>
-    </row>
-    <row r="63" ht="26" customHeight="1">
-      <c r="A63" s="35" t="n"/>
-      <c r="B63" s="35" t="n"/>
-      <c r="C63" s="35" t="n"/>
-      <c r="D63" s="35" t="n"/>
-      <c r="E63" s="35" t="n"/>
-      <c r="F63" s="35" t="n"/>
-    </row>
-    <row r="64" ht="26" customHeight="1">
-      <c r="A64" s="35" t="n"/>
-      <c r="B64" s="35" t="n"/>
-      <c r="C64" s="35" t="n"/>
-      <c r="D64" s="35" t="n"/>
-      <c r="E64" s="35" t="n"/>
-      <c r="F64" s="35" t="n"/>
+      <c r="A62" s="32" t="n"/>
+      <c r="B62" s="32" t="n"/>
+      <c r="C62" s="32" t="n"/>
+      <c r="D62" s="32" t="n"/>
+      <c r="E62" s="32" t="n"/>
+      <c r="F62" s="32" t="n"/>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>D.  Revision history</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B64" s="14" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>What changed</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+      <c r="E64" s="14" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="F64" s="14" t="inlineStr">
+        <is>
+          <t>Did it need a new sign-off</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="26" customHeight="1">
       <c r="A65" s="35" t="n"/>
@@ -3445,7 +3473,63 @@
       <c r="F67" s="35" t="n"/>
     </row>
     <row r="68" ht="26" customHeight="1">
-      <c r="A68" s="13" t="inlineStr">
+      <c r="A68" s="35" t="n"/>
+      <c r="B68" s="35" t="n"/>
+      <c r="C68" s="35" t="n"/>
+      <c r="D68" s="35" t="n"/>
+      <c r="E68" s="35" t="n"/>
+      <c r="F68" s="35" t="n"/>
+    </row>
+    <row r="69" ht="26" customHeight="1">
+      <c r="A69" s="35" t="n"/>
+      <c r="B69" s="35" t="n"/>
+      <c r="C69" s="35" t="n"/>
+      <c r="D69" s="35" t="n"/>
+      <c r="E69" s="35" t="n"/>
+      <c r="F69" s="35" t="n"/>
+    </row>
+    <row r="70" ht="26" customHeight="1">
+      <c r="A70" s="35" t="n"/>
+      <c r="B70" s="35" t="n"/>
+      <c r="C70" s="35" t="n"/>
+      <c r="D70" s="35" t="n"/>
+      <c r="E70" s="35" t="n"/>
+      <c r="F70" s="35" t="n"/>
+    </row>
+    <row r="71" ht="26" customHeight="1">
+      <c r="A71" s="35" t="n"/>
+      <c r="B71" s="35" t="n"/>
+      <c r="C71" s="35" t="n"/>
+      <c r="D71" s="35" t="n"/>
+      <c r="E71" s="35" t="n"/>
+      <c r="F71" s="35" t="n"/>
+    </row>
+    <row r="72" ht="26" customHeight="1">
+      <c r="A72" s="35" t="n"/>
+      <c r="B72" s="35" t="n"/>
+      <c r="C72" s="35" t="n"/>
+      <c r="D72" s="35" t="n"/>
+      <c r="E72" s="35" t="n"/>
+      <c r="F72" s="35" t="n"/>
+    </row>
+    <row r="73" ht="26" customHeight="1">
+      <c r="A73" s="35" t="n"/>
+      <c r="B73" s="35" t="n"/>
+      <c r="C73" s="35" t="n"/>
+      <c r="D73" s="35" t="n"/>
+      <c r="E73" s="35" t="n"/>
+      <c r="F73" s="35" t="n"/>
+    </row>
+    <row r="74" ht="26" customHeight="1">
+      <c r="A74" s="35" t="n"/>
+      <c r="B74" s="35" t="n"/>
+      <c r="C74" s="35" t="n"/>
+      <c r="D74" s="35" t="n"/>
+      <c r="E74" s="35" t="n"/>
+      <c r="F74" s="35" t="n"/>
+    </row>
+    <row r="75" ht="26" customHeight="1">
+      <c r="A75" s="13" t="inlineStr">
         <is>
           <t>A model version bump, a framework upgrade, a new tool, or a change of host all produce a row. Answer the last column every time, because an auditor will ask which changes went live without a fresh sign-off.</t>
         </is>
@@ -3453,18 +3537,22 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="79">
+  <mergeCells count="91">
     <mergeCell ref="C52:F52"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="C39:F39"/>
+    <mergeCell ref="A75:F75"/>
     <mergeCell ref="C13:F13"/>
+    <mergeCell ref="A54:B54"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A41:B41"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="C15:F15"/>
     <mergeCell ref="C24:F24"/>
     <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C54:F54"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="C41:F41"/>
     <mergeCell ref="C10:F10"/>
@@ -3472,8 +3560,9 @@
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="A51:F51"/>
+    <mergeCell ref="C56:F56"/>
+    <mergeCell ref="C27:F27"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C27:F27"/>
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="A39:B39"/>
     <mergeCell ref="A48:B48"/>
@@ -3484,20 +3573,25 @@
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A30:F30"/>
     <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A59:F59"/>
     <mergeCell ref="A52:B52"/>
     <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A61:F61"/>
     <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A54:F54"/>
     <mergeCell ref="C8:F8"/>
     <mergeCell ref="A49:B49"/>
     <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="C57:F57"/>
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="C34:F34"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="C58:F58"/>
+    <mergeCell ref="A55:B55"/>
     <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A63:F63"/>
     <mergeCell ref="C45:F45"/>
-    <mergeCell ref="A68:F68"/>
     <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A57:B57"/>
     <mergeCell ref="C20:F20"/>
     <mergeCell ref="C29:F29"/>
     <mergeCell ref="A14:B14"/>
@@ -3525,6 +3619,7 @@
     <mergeCell ref="C35:F35"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C55:F55"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A29:B29"/>
@@ -3532,13 +3627,14 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="C11:F11"/>
+    <mergeCell ref="A58:B58"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C16 C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Level 1,Level 2,Level 3"</formula1>
     </dataValidation>
-    <dataValidation sqref="F58:F67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F65:F74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Bound the grant list per classification, and name the adversarial testing.
Give each starter classification a widest-grant-list row, so a classification
constrains what the agent may reach and not only how it is watched. Ask the
sign-off record what adversarial testing was done, pointed at the OWASP
agentic list the incident playbook already works from. Point the autonomy row
at the CSA scale. Say which platform to score when an agent touches several.
Update the workbook to match.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -2757,7 +2757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2990,7 +2990,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Autonomy level, if you keep an autonomy scale</t>
+          <t>Autonomy level, on the four-level scale in the CSA agentic profile, or your own if you keep one</t>
         </is>
       </c>
       <c r="B22" s="15" t="n"/>
@@ -3098,34 +3098,34 @@
       <c r="E33" s="36" t="n"/>
       <c r="F33" s="34" t="n"/>
     </row>
-    <row r="34" ht="30" customHeight="1">
+    <row r="34" ht="56" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
+          <t>Adversarial testing performed, and against which failure modes</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="35" t="n"/>
+      <c r="D34" s="35" t="n"/>
+      <c r="E34" s="35" t="n"/>
+      <c r="F34" s="35" t="n"/>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>For any agent that reads content it did not author, whether it can be talked into something is what the sign-off most needs to know. Name the failure modes from OWASP's Top 10 for Agentic Applications, the same list the Monitoring sheet's playbook works from.</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="n"/>
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="13" t="n"/>
+      <c r="E35" s="13" t="n"/>
+      <c r="F35" s="13" t="n"/>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
           <t>Against which configuration, matching section A</t>
-        </is>
-      </c>
-      <c r="B34" s="15" t="n"/>
-      <c r="C34" s="35" t="n"/>
-      <c r="D34" s="36" t="n"/>
-      <c r="E34" s="36" t="n"/>
-      <c r="F34" s="34" t="n"/>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>Date of the run</t>
-        </is>
-      </c>
-      <c r="B35" s="15" t="n"/>
-      <c r="C35" s="35" t="n"/>
-      <c r="D35" s="36" t="n"/>
-      <c r="E35" s="36" t="n"/>
-      <c r="F35" s="34" t="n"/>
-    </row>
-    <row r="36" ht="56" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>What they found</t>
         </is>
       </c>
       <c r="B36" s="15" t="n"/>
@@ -3134,17 +3134,22 @@
       <c r="E36" s="36" t="n"/>
       <c r="F36" s="34" t="n"/>
     </row>
-    <row r="37" ht="13" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
-        <is>
-          <t>This is what the person signing off is accepting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="30" customHeight="1">
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Date of the run</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n"/>
+      <c r="C37" s="35" t="n"/>
+      <c r="D37" s="36" t="n"/>
+      <c r="E37" s="36" t="n"/>
+      <c r="F37" s="34" t="n"/>
+    </row>
+    <row r="38" ht="56" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>What you changed because of it</t>
+          <t>What they found</t>
         </is>
       </c>
       <c r="B38" s="15" t="n"/>
@@ -3153,29 +3158,29 @@
       <c r="E38" s="36" t="n"/>
       <c r="F38" s="34" t="n"/>
     </row>
-    <row r="39" ht="56" customHeight="1">
-      <c r="A39" s="10" t="inlineStr">
+    <row r="39" ht="13" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>This is what the person signing off is accepting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>What you changed because of it</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="n"/>
+      <c r="C40" s="35" t="n"/>
+      <c r="D40" s="36" t="n"/>
+      <c r="E40" s="36" t="n"/>
+      <c r="F40" s="34" t="n"/>
+    </row>
+    <row r="41" ht="56" customHeight="1">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>What you know you did NOT test</t>
-        </is>
-      </c>
-      <c r="B39" s="15" t="n"/>
-      <c r="C39" s="35" t="n"/>
-      <c r="D39" s="36" t="n"/>
-      <c r="E39" s="36" t="n"/>
-      <c r="F39" s="34" t="n"/>
-    </row>
-    <row r="40" ht="13" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t>This is where stage 4 monitoring has to begin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>Where the results are kept</t>
         </is>
       </c>
       <c r="B41" s="15" t="n"/>
@@ -3184,49 +3189,44 @@
       <c r="E41" s="36" t="n"/>
       <c r="F41" s="34" t="n"/>
     </row>
-    <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="32" t="n"/>
-      <c r="B42" s="32" t="n"/>
-      <c r="C42" s="32" t="n"/>
-      <c r="D42" s="32" t="n"/>
-      <c r="E42" s="32" t="n"/>
-      <c r="F42" s="32" t="n"/>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="9" t="inlineStr">
+    <row r="42" ht="13" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>This is where stage 4 monitoring has to begin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Where the results are kept</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="n"/>
+      <c r="C43" s="35" t="n"/>
+      <c r="D43" s="36" t="n"/>
+      <c r="E43" s="36" t="n"/>
+      <c r="F43" s="34" t="n"/>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="32" t="n"/>
+      <c r="B44" s="32" t="n"/>
+      <c r="C44" s="32" t="n"/>
+      <c r="D44" s="32" t="n"/>
+      <c r="E44" s="32" t="n"/>
+      <c r="F44" s="32" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>C.  Sign-off</t>
         </is>
       </c>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B44" s="15" t="n"/>
-      <c r="C44" s="35" t="n"/>
-      <c r="D44" s="36" t="n"/>
-      <c r="E44" s="36" t="n"/>
-      <c r="F44" s="34" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="10" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="B45" s="15" t="n"/>
-      <c r="C45" s="35" t="n"/>
-      <c r="D45" s="36" t="n"/>
-      <c r="E45" s="36" t="n"/>
-      <c r="F45" s="34" t="n"/>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B46" s="15" t="n"/>
@@ -3238,7 +3238,7 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>Version of the design document signed</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="B47" s="15" t="n"/>
@@ -3250,7 +3250,7 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>Version of this record signed</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B48" s="15" t="n"/>
@@ -3259,10 +3259,10 @@
       <c r="E48" s="36" t="n"/>
       <c r="F48" s="34" t="n"/>
     </row>
-    <row r="49" ht="56" customHeight="1">
+    <row r="49" ht="30" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>The risk that is left, stated in their words</t>
+          <t>Version of the design document signed</t>
         </is>
       </c>
       <c r="B49" s="15" t="n"/>
@@ -3274,7 +3274,7 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="10" t="inlineStr">
         <is>
-          <t>Any classification floor lowered by a compensating control</t>
+          <t>Version of this record signed</t>
         </is>
       </c>
       <c r="B50" s="15" t="n"/>
@@ -3283,17 +3283,22 @@
       <c r="E50" s="36" t="n"/>
       <c r="F50" s="34" t="n"/>
     </row>
-    <row r="51" ht="13" customHeight="1">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>A floor lowered in the design document and not repeated here has not been accepted by anybody.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="56" customHeight="1">
+    <row r="51" ht="56" customHeight="1">
+      <c r="A51" s="10" t="inlineStr">
+        <is>
+          <t>The risk that is left, stated in their words</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="n"/>
+      <c r="C51" s="35" t="n"/>
+      <c r="D51" s="36" t="n"/>
+      <c r="E51" s="36" t="n"/>
+      <c r="F51" s="34" t="n"/>
+    </row>
+    <row r="52" ht="30" customHeight="1">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>Conditions on the sign-off, and when it must be looked at again</t>
+          <t>Any classification floor lowered by a compensating control</t>
         </is>
       </c>
       <c r="B52" s="15" t="n"/>
@@ -3302,102 +3307,96 @@
       <c r="E52" s="36" t="n"/>
       <c r="F52" s="34" t="n"/>
     </row>
-    <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="24" t="inlineStr">
+    <row r="53" ht="13" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>A floor lowered in the design document and not repeated here has not been accepted by anybody.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="56" customHeight="1">
+      <c r="A54" s="10" t="inlineStr">
+        <is>
+          <t>Conditions on the sign-off, and when it must be looked at again</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="n"/>
+      <c r="C54" s="35" t="n"/>
+      <c r="D54" s="36" t="n"/>
+      <c r="E54" s="36" t="n"/>
+      <c r="F54" s="34" t="n"/>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="24" t="inlineStr">
         <is>
           <t>THE LEVEL GAP.  The agent's classification names a platform control level and a monitoring level that an agent in it requires. Where the level applied is lower, the gap is accepted here, by name, or it is not accepted at all.</t>
         </is>
       </c>
-      <c r="B53" s="24" t="n"/>
-      <c r="C53" s="24" t="n"/>
-      <c r="D53" s="24" t="n"/>
-      <c r="E53" s="24" t="n"/>
-      <c r="F53" s="24" t="n"/>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="10" t="inlineStr">
-        <is>
-          <t>Platform control level the classification requires, and the level applied</t>
-        </is>
-      </c>
-      <c r="B54" s="10" t="n"/>
-      <c r="C54" s="35" t="n"/>
-      <c r="D54" s="35" t="n"/>
-      <c r="E54" s="35" t="n"/>
-      <c r="F54" s="35" t="n"/>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="10" t="inlineStr">
-        <is>
-          <t>Monitoring level the classification requires, and the level applied</t>
-        </is>
-      </c>
-      <c r="B55" s="10" t="n"/>
-      <c r="C55" s="35" t="n"/>
-      <c r="D55" s="35" t="n"/>
-      <c r="E55" s="35" t="n"/>
-      <c r="F55" s="35" t="n"/>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>Who accepts the gap, by name</t>
-        </is>
-      </c>
-      <c r="B56" s="10" t="n"/>
+          <t>Platform control level the classification requires, and the level applied</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="n"/>
       <c r="C56" s="35" t="n"/>
-      <c r="D56" s="35" t="n"/>
-      <c r="E56" s="35" t="n"/>
-      <c r="F56" s="35" t="n"/>
+      <c r="D56" s="36" t="n"/>
+      <c r="E56" s="36" t="n"/>
+      <c r="F56" s="34" t="n"/>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>The date by which it closes</t>
-        </is>
-      </c>
-      <c r="B57" s="10" t="n"/>
+          <t>Monitoring level the classification requires, and the level applied</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="n"/>
       <c r="C57" s="35" t="n"/>
-      <c r="D57" s="35" t="n"/>
-      <c r="E57" s="35" t="n"/>
-      <c r="F57" s="35" t="n"/>
+      <c r="D57" s="36" t="n"/>
+      <c r="E57" s="36" t="n"/>
+      <c r="F57" s="34" t="n"/>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
+          <t>Who accepts the gap, by name</t>
+        </is>
+      </c>
+      <c r="B58" s="15" t="n"/>
+      <c r="C58" s="35" t="n"/>
+      <c r="D58" s="36" t="n"/>
+      <c r="E58" s="36" t="n"/>
+      <c r="F58" s="34" t="n"/>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="10" t="inlineStr">
+        <is>
+          <t>The date by which it closes</t>
+        </is>
+      </c>
+      <c r="B59" s="15" t="n"/>
+      <c r="C59" s="35" t="n"/>
+      <c r="D59" s="36" t="n"/>
+      <c r="E59" s="36" t="n"/>
+      <c r="F59" s="34" t="n"/>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
           <t>How many consecutive sign-offs have accepted this same gap</t>
         </is>
       </c>
-      <c r="B58" s="10" t="n"/>
-      <c r="C58" s="35" t="n"/>
-      <c r="D58" s="35" t="n"/>
-      <c r="E58" s="35" t="n"/>
-      <c r="F58" s="35" t="n"/>
-    </row>
-    <row r="59" ht="26" customHeight="1">
-      <c r="A59" s="13" t="inlineStr">
+      <c r="B60" s="15" t="n"/>
+      <c r="C60" s="35" t="n"/>
+      <c r="D60" s="36" t="n"/>
+      <c r="E60" s="36" t="n"/>
+      <c r="F60" s="34" t="n"/>
+    </row>
+    <row r="61" ht="26" customHeight="1">
+      <c r="A61" s="13" t="inlineStr">
         <is>
           <t>Answer the last row honestly. A gap accepted once is a legitimate decision made under time pressure. A gap accepted three times in a row is a decision nobody is making, and this count is the only thing on any of these forms that would show it.</t>
-        </is>
-      </c>
-      <c r="B59" s="13" t="n"/>
-      <c r="C59" s="13" t="n"/>
-      <c r="D59" s="13" t="n"/>
-      <c r="E59" s="13" t="n"/>
-      <c r="F59" s="13" t="n"/>
-    </row>
-    <row r="60" ht="26" customHeight="1">
-      <c r="A60" s="32" t="n"/>
-      <c r="B60" s="32" t="n"/>
-      <c r="C60" s="32" t="n"/>
-      <c r="D60" s="32" t="n"/>
-      <c r="E60" s="32" t="n"/>
-      <c r="F60" s="32" t="n"/>
-    </row>
-    <row r="61" ht="26" customHeight="1">
-      <c r="A61" s="24" t="inlineStr">
-        <is>
-          <t>The sign-off is against the two versions named above. When live behavior stops matching the description it was granted against, it is void until somebody looks again.</t>
         </is>
       </c>
     </row>
@@ -3409,60 +3408,59 @@
       <c r="E62" s="32" t="n"/>
       <c r="F62" s="32" t="n"/>
     </row>
-    <row r="63" ht="22" customHeight="1">
-      <c r="A63" s="9" t="inlineStr">
+    <row r="63" ht="26" customHeight="1">
+      <c r="A63" s="24" t="inlineStr">
+        <is>
+          <t>The sign-off is against the two versions named above. When live behavior stops matching the description it was granted against, it is void until somebody looks again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="26" customHeight="1">
+      <c r="A64" s="32" t="n"/>
+      <c r="B64" s="32" t="n"/>
+      <c r="C64" s="32" t="n"/>
+      <c r="D64" s="32" t="n"/>
+      <c r="E64" s="32" t="n"/>
+      <c r="F64" s="32" t="n"/>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="9" t="inlineStr">
         <is>
           <t>D.  Revision history</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="28" customHeight="1">
-      <c r="A64" s="14" t="inlineStr">
+    <row r="66" ht="28" customHeight="1">
+      <c r="A66" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B64" s="14" t="inlineStr">
+      <c r="B66" s="14" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="C64" s="14" t="inlineStr">
+      <c r="C66" s="14" t="inlineStr">
         <is>
           <t>What changed</t>
         </is>
       </c>
-      <c r="D64" s="14" t="inlineStr">
+      <c r="D66" s="14" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="E64" s="14" t="inlineStr">
+      <c r="E66" s="14" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="F64" s="14" t="inlineStr">
+      <c r="F66" s="14" t="inlineStr">
         <is>
           <t>Did it need a new sign-off</t>
         </is>
       </c>
-    </row>
-    <row r="65" ht="26" customHeight="1">
-      <c r="A65" s="35" t="n"/>
-      <c r="B65" s="35" t="n"/>
-      <c r="C65" s="35" t="n"/>
-      <c r="D65" s="35" t="n"/>
-      <c r="E65" s="35" t="n"/>
-      <c r="F65" s="35" t="n"/>
-    </row>
-    <row r="66" ht="26" customHeight="1">
-      <c r="A66" s="35" t="n"/>
-      <c r="B66" s="35" t="n"/>
-      <c r="C66" s="35" t="n"/>
-      <c r="D66" s="35" t="n"/>
-      <c r="E66" s="35" t="n"/>
-      <c r="F66" s="35" t="n"/>
     </row>
     <row r="67" ht="26" customHeight="1">
       <c r="A67" s="35" t="n"/>
@@ -3529,7 +3527,23 @@
       <c r="F74" s="35" t="n"/>
     </row>
     <row r="75" ht="26" customHeight="1">
-      <c r="A75" s="13" t="inlineStr">
+      <c r="A75" s="35" t="n"/>
+      <c r="B75" s="35" t="n"/>
+      <c r="C75" s="35" t="n"/>
+      <c r="D75" s="35" t="n"/>
+      <c r="E75" s="35" t="n"/>
+      <c r="F75" s="35" t="n"/>
+    </row>
+    <row r="76" ht="26" customHeight="1">
+      <c r="A76" s="35" t="n"/>
+      <c r="B76" s="35" t="n"/>
+      <c r="C76" s="35" t="n"/>
+      <c r="D76" s="35" t="n"/>
+      <c r="E76" s="35" t="n"/>
+      <c r="F76" s="35" t="n"/>
+    </row>
+    <row r="77" ht="26" customHeight="1">
+      <c r="A77" s="13" t="inlineStr">
         <is>
           <t>A model version bump, a framework upgrade, a new tool, or a change of host all produce a row. Answer the last column every time, because an auditor will ask which changes went live without a fresh sign-off.</t>
         </is>
@@ -3537,43 +3551,44 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="91">
+  <mergeCells count="94">
     <mergeCell ref="C52:F52"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="C39:F39"/>
-    <mergeCell ref="A75:F75"/>
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="A55:F55"/>
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="A54:B54"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A41:B41"/>
     <mergeCell ref="A32:F32"/>
     <mergeCell ref="C15:F15"/>
+    <mergeCell ref="A56:B56"/>
     <mergeCell ref="C24:F24"/>
     <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A56:B56"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="C54:F54"/>
-    <mergeCell ref="A40:F40"/>
     <mergeCell ref="C41:F41"/>
     <mergeCell ref="C10:F10"/>
     <mergeCell ref="C50:F50"/>
     <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A51:F51"/>
     <mergeCell ref="C56:F56"/>
+    <mergeCell ref="C43:F43"/>
+    <mergeCell ref="A9:B9"/>
     <mergeCell ref="C27:F27"/>
-    <mergeCell ref="A9:B9"/>
     <mergeCell ref="C36:F36"/>
-    <mergeCell ref="A39:B39"/>
     <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A59:B59"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A37:B37"/>
     <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A35:F35"/>
     <mergeCell ref="C14:F14"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A30:F30"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="C40:F40"/>
     <mergeCell ref="A52:B52"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A61:F61"/>
@@ -3586,27 +3601,31 @@
     <mergeCell ref="C34:F34"/>
     <mergeCell ref="A53:F53"/>
     <mergeCell ref="C58:F58"/>
-    <mergeCell ref="A55:B55"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A63:F63"/>
-    <mergeCell ref="C45:F45"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A57:B57"/>
     <mergeCell ref="C20:F20"/>
     <mergeCell ref="C29:F29"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="C47:F47"/>
-    <mergeCell ref="C44:F44"/>
+    <mergeCell ref="A39:F39"/>
     <mergeCell ref="C22:F22"/>
     <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A43:B43"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C12:F12"/>
+    <mergeCell ref="A45:F45"/>
     <mergeCell ref="C46:F46"/>
+    <mergeCell ref="C51:F51"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C60:F60"/>
+    <mergeCell ref="A65:F65"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="C48:F48"/>
-    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="C38:F38"/>
     <mergeCell ref="C7:F7"/>
-    <mergeCell ref="C38:F38"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="C49:F49"/>
@@ -3615,17 +3634,15 @@
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A50:B50"/>
-    <mergeCell ref="A43:F43"/>
-    <mergeCell ref="C35:F35"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C55:F55"/>
+    <mergeCell ref="A77:F77"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="C59:F59"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A44:B44"/>
     <mergeCell ref="C11:F11"/>
     <mergeCell ref="A58:B58"/>
     <mergeCell ref="A25:F25"/>
@@ -3634,7 +3651,7 @@
     <dataValidation sqref="C16 C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Level 1,Level 2,Level 3"</formula1>
     </dataValidation>
-    <dataValidation sqref="F65:F74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F67:F76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Carry an incident through to notification, resumption, and the sign-off.
Add the outside-notification clock and the resume decision to the alert
stages, since the stage 3 sign-off is void from the moment live behavior
stops matching it. Record the monitoring level the classification requires,
and say the gap is accepted in the sign-off record rather than here. Give
ASI05 its own playbook row and ask for "the agent cannot do this" instead of
a blank. Name who owns extending the eval set, and where the monitor reads
the grant list from. Update the workbook to match.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -3104,11 +3104,11 @@
           <t>Adversarial testing performed, and against which failure modes</t>
         </is>
       </c>
-      <c r="B34" s="10" t="n"/>
+      <c r="B34" s="15" t="n"/>
       <c r="C34" s="35" t="n"/>
-      <c r="D34" s="35" t="n"/>
-      <c r="E34" s="35" t="n"/>
-      <c r="F34" s="35" t="n"/>
+      <c r="D34" s="36" t="n"/>
+      <c r="E34" s="36" t="n"/>
+      <c r="F34" s="34" t="n"/>
     </row>
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
@@ -3116,11 +3116,6 @@
           <t>For any agent that reads content it did not author, whether it can be talked into something is what the sign-off most needs to know. Name the failure modes from OWASP's Top 10 for Agentic Applications, the same list the Monitoring sheet's playbook works from.</t>
         </is>
       </c>
-      <c r="B35" s="13" t="n"/>
-      <c r="C35" s="13" t="n"/>
-      <c r="D35" s="13" t="n"/>
-      <c r="E35" s="13" t="n"/>
-      <c r="F35" s="13" t="n"/>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
@@ -3568,8 +3563,8 @@
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="A33:B33"/>
     <mergeCell ref="C54:F54"/>
+    <mergeCell ref="C10:F10"/>
     <mergeCell ref="C41:F41"/>
-    <mergeCell ref="C10:F10"/>
     <mergeCell ref="C50:F50"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="C56:F56"/>
@@ -3674,7 +3669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3773,7 +3768,7 @@
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Monitoring level of the platform it runs on: 1, 2 or 3</t>
+          <t>Monitoring level the classification requires</t>
         </is>
       </c>
       <c r="B10" s="15" t="n"/>
@@ -3785,7 +3780,7 @@
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Monitoring level actually applied to this agent: can be lower than the platform's, never higher</t>
+          <t>Monitoring level of the platform it runs on: 1, 2 or 3</t>
         </is>
       </c>
       <c r="B11" s="15" t="n"/>
@@ -3797,7 +3792,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Who owns this monitoring</t>
+          <t>Monitoring level actually applied to this agent: can be lower than the platform's, never higher</t>
         </is>
       </c>
       <c r="B12" s="15" t="n"/>
@@ -3806,66 +3801,61 @@
       <c r="E12" s="36" t="n"/>
       <c r="F12" s="34" t="n"/>
     </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="32" t="n"/>
-      <c r="B13" s="32" t="n"/>
-      <c r="C13" s="32" t="n"/>
-      <c r="D13" s="32" t="n"/>
-      <c r="E13" s="32" t="n"/>
-      <c r="F13" s="32" t="n"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Who owns this monitoring</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="35" t="n"/>
+      <c r="D13" s="36" t="n"/>
+      <c r="E13" s="36" t="n"/>
+      <c r="F13" s="34" t="n"/>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Where the level applied is lower than the level the classification requires, the gap is accepted in section C of the Platform &amp; Sign-off sheet, not here. This sheet records what is true; that one records who accepted it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="32" t="n"/>
+      <c r="B15" s="32" t="n"/>
+      <c r="C15" s="32" t="n"/>
+      <c r="D15" s="32" t="n"/>
+      <c r="E15" s="32" t="n"/>
+      <c r="F15" s="32" t="n"/>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>What you record</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Do you record it</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>Where it goes</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>How long you keep it</t>
         </is>
       </c>
-      <c r="E14" s="16" t="n"/>
-      <c r="F14" s="15" t="n"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="25" t="inlineStr">
-        <is>
-          <t>Every tool call, and its arguments</t>
-        </is>
-      </c>
-      <c r="B15" s="35" t="n"/>
-      <c r="C15" s="35" t="n"/>
-      <c r="D15" s="35" t="n"/>
-      <c r="E15" s="36" t="n"/>
-      <c r="F15" s="34" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="25" t="inlineStr">
-        <is>
-          <t>Inputs to the run</t>
-        </is>
-      </c>
-      <c r="B16" s="35" t="n"/>
-      <c r="C16" s="35" t="n"/>
-      <c r="D16" s="35" t="n"/>
-      <c r="E16" s="36" t="n"/>
-      <c r="F16" s="34" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="15" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>Outputs of the run</t>
+          <t>Every tool call, and its arguments</t>
         </is>
       </c>
       <c r="B17" s="35" t="n"/>
@@ -3877,7 +3867,7 @@
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>The prompt and context as sent</t>
+          <t>Inputs to the run</t>
         </is>
       </c>
       <c r="B18" s="35" t="n"/>
@@ -3889,7 +3879,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>Escalations to a person, and the outcome</t>
+          <t>Outputs of the run</t>
         </is>
       </c>
       <c r="B19" s="35" t="n"/>
@@ -3901,7 +3891,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>Enough of the run to replay it</t>
+          <t>The prompt and context as sent</t>
         </is>
       </c>
       <c r="B20" s="35" t="n"/>
@@ -3913,7 +3903,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>Cost and token use per run</t>
+          <t>Escalations to a person, and the outcome</t>
         </is>
       </c>
       <c r="B21" s="35" t="n"/>
@@ -3922,37 +3912,42 @@
       <c r="E21" s="36" t="n"/>
       <c r="F21" s="34" t="n"/>
     </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="32" t="n"/>
-      <c r="B22" s="32" t="n"/>
-      <c r="C22" s="32" t="n"/>
-      <c r="D22" s="32" t="n"/>
-      <c r="E22" s="32" t="n"/>
-      <c r="F22" s="32" t="n"/>
-    </row>
-    <row r="23" ht="56" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>What you deliberately do NOT record, and why</t>
-        </is>
-      </c>
-      <c r="B23" s="15" t="n"/>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="25" t="inlineStr">
+        <is>
+          <t>Enough of the run to replay it</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="n"/>
+      <c r="C22" s="35" t="n"/>
+      <c r="D22" s="35" t="n"/>
+      <c r="E22" s="36" t="n"/>
+      <c r="F22" s="34" t="n"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="25" t="inlineStr">
+        <is>
+          <t>Cost and token use per run</t>
+        </is>
+      </c>
+      <c r="B23" s="35" t="n"/>
       <c r="C23" s="35" t="n"/>
-      <c r="D23" s="36" t="n"/>
+      <c r="D23" s="35" t="n"/>
       <c r="E23" s="36" t="n"/>
       <c r="F23" s="34" t="n"/>
     </row>
-    <row r="24" ht="13" customHeight="1">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>Usually personal data you have no basis to retain. Say what you lose by not recording it.</t>
-        </is>
-      </c>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="32" t="n"/>
+      <c r="B24" s="32" t="n"/>
+      <c r="C24" s="32" t="n"/>
+      <c r="D24" s="32" t="n"/>
+      <c r="E24" s="32" t="n"/>
+      <c r="F24" s="32" t="n"/>
     </row>
     <row r="25" ht="56" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>Who can read these records, and who can change them</t>
+          <t>What you deliberately do NOT record, and why</t>
         </is>
       </c>
       <c r="B25" s="15" t="n"/>
@@ -3964,60 +3959,60 @@
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="13" t="inlineStr">
         <is>
+          <t>Usually personal data you have no basis to retain. Say what you lose by not recording it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="56" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Who can read these records, and who can change them</t>
+        </is>
+      </c>
+      <c r="B27" s="15" t="n"/>
+      <c r="C27" s="35" t="n"/>
+      <c r="D27" s="36" t="n"/>
+      <c r="E27" s="36" t="n"/>
+      <c r="F27" s="34" t="n"/>
+    </row>
+    <row r="28" ht="13" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
           <t>If the team that operates the agent can edit its own logs, say so here. Stage 5 needs records an auditor will accept.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="26" customHeight="1">
-      <c r="A27" s="32" t="n"/>
-      <c r="B27" s="32" t="n"/>
-      <c r="C27" s="32" t="n"/>
-      <c r="D27" s="32" t="n"/>
-      <c r="E27" s="32" t="n"/>
-      <c r="F27" s="32" t="n"/>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="32" t="n"/>
+      <c r="B29" s="32" t="n"/>
+      <c r="C29" s="32" t="n"/>
+      <c r="D29" s="32" t="n"/>
+      <c r="E29" s="32" t="n"/>
+      <c r="F29" s="32" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>B.  The evals, and what runs them</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="56" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
+    <row r="31" ht="56" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>Which evals run against the live agent</t>
         </is>
       </c>
-      <c r="B29" s="15" t="n"/>
-      <c r="C29" s="35" t="n"/>
-      <c r="D29" s="36" t="n"/>
-      <c r="E29" s="36" t="n"/>
-      <c r="F29" s="34" t="n"/>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="B31" s="15" t="n"/>
+      <c r="C31" s="35" t="n"/>
+      <c r="D31" s="36" t="n"/>
+      <c r="E31" s="36" t="n"/>
+      <c r="F31" s="34" t="n"/>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>What starts them</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="n"/>
-      <c r="C30" s="35" t="n"/>
-      <c r="D30" s="36" t="n"/>
-      <c r="E30" s="36" t="n"/>
-      <c r="F30" s="34" t="n"/>
-    </row>
-    <row r="31" ht="13" customHeight="1">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>A schedule, a deployment, live traffic, or a person. An eval a person has to remember to run is not assurance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="56" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>How often, or what share of live traffic if they run continuously</t>
         </is>
       </c>
       <c r="B32" s="15" t="n"/>
@@ -4026,22 +4021,17 @@
       <c r="E32" s="36" t="n"/>
       <c r="F32" s="34" t="n"/>
     </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>Where the results go</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n"/>
-      <c r="C33" s="35" t="n"/>
-      <c r="D33" s="36" t="n"/>
-      <c r="E33" s="36" t="n"/>
-      <c r="F33" s="34" t="n"/>
-    </row>
-    <row r="34" ht="30" customHeight="1">
+    <row r="33" ht="13" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>A schedule, a deployment, live traffic, or a person. An eval a person has to remember to run is not assurance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="56" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Who is told when one fails</t>
+          <t>How often, or what share of live traffic if they run continuously</t>
         </is>
       </c>
       <c r="B34" s="15" t="n"/>
@@ -4050,10 +4040,10 @@
       <c r="E34" s="36" t="n"/>
       <c r="F34" s="34" t="n"/>
     </row>
-    <row r="35" ht="56" customHeight="1">
+    <row r="35" ht="30" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>How you would know they had stopped running</t>
+          <t>Where the results go</t>
         </is>
       </c>
       <c r="B35" s="15" t="n"/>
@@ -4062,17 +4052,22 @@
       <c r="E35" s="36" t="n"/>
       <c r="F35" s="34" t="n"/>
     </row>
-    <row r="36" ht="13" customHeight="1">
-      <c r="A36" s="13" t="inlineStr">
-        <is>
-          <t>A dead scheduler and a continuous job that quietly stopped look the same from outside: everything is green because nothing is running.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="56" customHeight="1">
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Who is told when one fails</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="n"/>
+      <c r="C36" s="35" t="n"/>
+      <c r="D36" s="36" t="n"/>
+      <c r="E36" s="36" t="n"/>
+      <c r="F36" s="34" t="n"/>
+    </row>
+    <row r="37" ht="30" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>Which baseline the results are compared against</t>
+          <t>Who owns extending the eval set as the agent changes</t>
         </is>
       </c>
       <c r="B37" s="15" t="n"/>
@@ -4081,96 +4076,91 @@
       <c r="E37" s="36" t="n"/>
       <c r="F37" s="34" t="n"/>
     </row>
-    <row r="38" ht="13" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
+    <row r="38" ht="56" customHeight="1">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>How you would know they had stopped running</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="n"/>
+      <c r="C38" s="35" t="n"/>
+      <c r="D38" s="36" t="n"/>
+      <c r="E38" s="36" t="n"/>
+      <c r="F38" s="34" t="n"/>
+    </row>
+    <row r="39" ht="13" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>A dead scheduler and a continuous job that quietly stopped look the same from outside: everything is green because nothing is running.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="56" customHeight="1">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Which baseline the results are compared against</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="n"/>
+      <c r="C40" s="35" t="n"/>
+      <c r="D40" s="36" t="n"/>
+      <c r="E40" s="36" t="n"/>
+      <c r="F40" s="34" t="n"/>
+    </row>
+    <row r="41" ht="13" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
         <is>
           <t>Normally the eval results recorded at sign-off. Name the version.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="32" t="n"/>
-      <c r="B39" s="32" t="n"/>
-      <c r="C39" s="32" t="n"/>
-      <c r="D39" s="32" t="n"/>
-      <c r="E39" s="32" t="n"/>
-      <c r="F39" s="32" t="n"/>
-    </row>
-    <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="9" t="inlineStr">
+    <row r="42" ht="26" customHeight="1">
+      <c r="A42" s="32" t="n"/>
+      <c r="B42" s="32" t="n"/>
+      <c r="C42" s="32" t="n"/>
+      <c r="D42" s="32" t="n"/>
+      <c r="E42" s="32" t="n"/>
+      <c r="F42" s="32" t="n"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
         <is>
           <t>C.  What counts as normal, and what starts an alert</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="14" t="inlineStr">
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>What normal looks like</t>
         </is>
       </c>
-      <c r="C41" s="14" t="inlineStr">
+      <c r="C44" s="14" t="inlineStr">
         <is>
           <t>What starts an alert</t>
         </is>
       </c>
-      <c r="D41" s="14" t="inlineStr">
+      <c r="D44" s="14" t="inlineStr">
         <is>
           <t>Who receives it</t>
         </is>
       </c>
-      <c r="E41" s="14" t="inlineStr">
+      <c r="E44" s="14" t="inlineStr">
         <is>
           <t>Implemented today</t>
         </is>
       </c>
-      <c r="F41" s="15" t="n"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="25" t="inlineStr">
-        <is>
-          <t>A call to a tool outside the declared set</t>
-        </is>
-      </c>
-      <c r="B42" s="35" t="n"/>
-      <c r="C42" s="35" t="n"/>
-      <c r="D42" s="35" t="n"/>
-      <c r="E42" s="35" t="n"/>
-      <c r="F42" s="34" t="n"/>
-    </row>
-    <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="25" t="inlineStr">
-        <is>
-          <t>Volume of runs</t>
-        </is>
-      </c>
-      <c r="B43" s="35" t="n"/>
-      <c r="C43" s="35" t="n"/>
-      <c r="D43" s="35" t="n"/>
-      <c r="E43" s="35" t="n"/>
-      <c r="F43" s="34" t="n"/>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="25" t="inlineStr">
-        <is>
-          <t>Escalation rate to a person</t>
-        </is>
-      </c>
-      <c r="B44" s="35" t="n"/>
-      <c r="C44" s="35" t="n"/>
-      <c r="D44" s="35" t="n"/>
-      <c r="E44" s="35" t="n"/>
-      <c r="F44" s="34" t="n"/>
+      <c r="F44" s="15" t="n"/>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="25" t="inlineStr">
         <is>
-          <t>Eval failure</t>
+          <t>A call to a tool outside the declared set</t>
         </is>
       </c>
       <c r="B45" s="35" t="n"/>
@@ -4182,7 +4172,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>Cost per run or per day</t>
+          <t>Volume of runs</t>
         </is>
       </c>
       <c r="B46" s="35" t="n"/>
@@ -4194,7 +4184,7 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>Error or retry rate</t>
+          <t>Escalation rate to a person</t>
         </is>
       </c>
       <c r="B47" s="35" t="n"/>
@@ -4206,7 +4196,7 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>Drift from the design document</t>
+          <t>Eval failure</t>
         </is>
       </c>
       <c r="B48" s="35" t="n"/>
@@ -4216,99 +4206,99 @@
       <c r="F48" s="34" t="n"/>
     </row>
     <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="37" t="n"/>
+      <c r="A49" s="25" t="inlineStr">
+        <is>
+          <t>Cost per run or per day</t>
+        </is>
+      </c>
       <c r="B49" s="35" t="n"/>
       <c r="C49" s="35" t="n"/>
       <c r="D49" s="35" t="n"/>
       <c r="E49" s="35" t="n"/>
       <c r="F49" s="34" t="n"/>
     </row>
-    <row r="50" ht="14" customHeight="1">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>Answer the last column for what is implemented today, not what is planned. A row with nothing behind it is a gap the sign-off has to carry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="26" customHeight="1">
-      <c r="A51" s="32" t="n"/>
-      <c r="B51" s="32" t="n"/>
-      <c r="C51" s="32" t="n"/>
-      <c r="D51" s="32" t="n"/>
-      <c r="E51" s="32" t="n"/>
-      <c r="F51" s="32" t="n"/>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="9" t="inlineStr">
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="25" t="inlineStr">
+        <is>
+          <t>Error or retry rate</t>
+        </is>
+      </c>
+      <c r="B50" s="35" t="n"/>
+      <c r="C50" s="35" t="n"/>
+      <c r="D50" s="35" t="n"/>
+      <c r="E50" s="35" t="n"/>
+      <c r="F50" s="34" t="n"/>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="25" t="inlineStr">
+        <is>
+          <t>Drift from the design document</t>
+        </is>
+      </c>
+      <c r="B51" s="35" t="n"/>
+      <c r="C51" s="35" t="n"/>
+      <c r="D51" s="35" t="n"/>
+      <c r="E51" s="35" t="n"/>
+      <c r="F51" s="34" t="n"/>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="37" t="n"/>
+      <c r="B52" s="35" t="n"/>
+      <c r="C52" s="35" t="n"/>
+      <c r="D52" s="35" t="n"/>
+      <c r="E52" s="35" t="n"/>
+      <c r="F52" s="34" t="n"/>
+    </row>
+    <row r="53" ht="14" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>Answer the last column for what is implemented today, not what is planned. A row with nothing behind it is a gap the sign-off has to carry. The first row needs the section 3 grant list in a form the monitor can read. It is the only machine-checkable claim in the framework, and naming where the monitor gets it is the difference between an alert you can build and one you intend to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="26" customHeight="1">
+      <c r="A54" s="32" t="n"/>
+      <c r="B54" s="32" t="n"/>
+      <c r="C54" s="32" t="n"/>
+      <c r="D54" s="32" t="n"/>
+      <c r="E54" s="32" t="n"/>
+      <c r="F54" s="32" t="n"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="9" t="inlineStr">
         <is>
           <t>D.  What an alert starts</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="14" t="inlineStr">
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="14" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="B53" s="14" t="inlineStr">
+      <c r="B56" s="14" t="inlineStr">
         <is>
           <t>What happens</t>
         </is>
       </c>
-      <c r="C53" s="15" t="n"/>
-      <c r="D53" s="14" t="inlineStr">
+      <c r="C56" s="15" t="n"/>
+      <c r="D56" s="14" t="inlineStr">
         <is>
           <t>Who does it</t>
         </is>
       </c>
-      <c r="E53" s="14" t="inlineStr">
+      <c r="E56" s="14" t="inlineStr">
         <is>
           <t>Within what time</t>
         </is>
       </c>
-      <c r="F53" s="15" t="n"/>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="25" t="inlineStr">
-        <is>
-          <t>Triage: is this real</t>
-        </is>
-      </c>
-      <c r="B54" s="35" t="n"/>
-      <c r="C54" s="34" t="n"/>
-      <c r="D54" s="35" t="n"/>
-      <c r="E54" s="35" t="n"/>
-      <c r="F54" s="34" t="n"/>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="25" t="inlineStr">
-        <is>
-          <t>Contain: stop or narrow the agent</t>
-        </is>
-      </c>
-      <c r="B55" s="35" t="n"/>
-      <c r="C55" s="34" t="n"/>
-      <c r="D55" s="35" t="n"/>
-      <c r="E55" s="35" t="n"/>
-      <c r="F55" s="34" t="n"/>
-    </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="25" t="inlineStr">
-        <is>
-          <t>Review the run records</t>
-        </is>
-      </c>
-      <c r="B56" s="35" t="n"/>
-      <c r="C56" s="34" t="n"/>
-      <c r="D56" s="35" t="n"/>
-      <c r="E56" s="35" t="n"/>
-      <c r="F56" s="34" t="n"/>
+      <c r="F56" s="15" t="n"/>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Triage: is this real</t>
         </is>
       </c>
       <c r="B57" s="35" t="n"/>
@@ -4320,7 +4310,7 @@
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>Tell the people affected</t>
+          <t>Contain: stop or narrow the agent</t>
         </is>
       </c>
       <c r="B58" s="35" t="n"/>
@@ -4332,7 +4322,7 @@
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>Review after the incident</t>
+          <t>Review the run records</t>
         </is>
       </c>
       <c r="B59" s="35" t="n"/>
@@ -4341,212 +4331,174 @@
       <c r="E59" s="35" t="n"/>
       <c r="F59" s="34" t="n"/>
     </row>
-    <row r="60" ht="26" customHeight="1">
-      <c r="A60" s="32" t="n"/>
-      <c r="B60" s="32" t="n"/>
-      <c r="C60" s="32" t="n"/>
-      <c r="D60" s="32" t="n"/>
-      <c r="E60" s="32" t="n"/>
-      <c r="F60" s="32" t="n"/>
-    </row>
-    <row r="61" ht="56" customHeight="1">
-      <c r="A61" s="10" t="inlineStr">
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="25" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="B60" s="35" t="n"/>
+      <c r="C60" s="34" t="n"/>
+      <c r="D60" s="35" t="n"/>
+      <c r="E60" s="35" t="n"/>
+      <c r="F60" s="34" t="n"/>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="25" t="inlineStr">
+        <is>
+          <t>Tell the people affected</t>
+        </is>
+      </c>
+      <c r="B61" s="35" t="n"/>
+      <c r="C61" s="34" t="n"/>
+      <c r="D61" s="35" t="n"/>
+      <c r="E61" s="35" t="n"/>
+      <c r="F61" s="34" t="n"/>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
+          <t>Decide whether anybody outside has to be told, and start that clock</t>
+        </is>
+      </c>
+      <c r="B62" s="35" t="n"/>
+      <c r="C62" s="34" t="n"/>
+      <c r="D62" s="35" t="n"/>
+      <c r="E62" s="35" t="n"/>
+      <c r="F62" s="34" t="n"/>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="25" t="inlineStr">
+        <is>
+          <t>Review after the incident</t>
+        </is>
+      </c>
+      <c r="B63" s="35" t="n"/>
+      <c r="C63" s="34" t="n"/>
+      <c r="D63" s="35" t="n"/>
+      <c r="E63" s="35" t="n"/>
+      <c r="F63" s="34" t="n"/>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="A64" s="25" t="inlineStr">
+        <is>
+          <t>Decide whether the agent resumes, and whether the sign-off still holds</t>
+        </is>
+      </c>
+      <c r="B64" s="35" t="n"/>
+      <c r="C64" s="34" t="n"/>
+      <c r="D64" s="35" t="n"/>
+      <c r="E64" s="35" t="n"/>
+      <c r="F64" s="34" t="n"/>
+    </row>
+    <row r="65" ht="26" customHeight="1">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>For an agent inside a regulated process, notifying a regulator or a data-protection authority runs on a clock that starts well before the fix is finished. Stage 2 classifies agents on whether a mistake is reportable, so somebody has to decide here whether this one is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="26" customHeight="1">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>The stage 3 sign-off is void once live behavior stops matching what it was granted against, and an incident is that moment. Name who re-confirms it, or re-issues it, before the agent runs again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="26" customHeight="1">
+      <c r="A67" s="32" t="n"/>
+      <c r="B67" s="32" t="n"/>
+      <c r="C67" s="32" t="n"/>
+      <c r="D67" s="32" t="n"/>
+      <c r="E67" s="32" t="n"/>
+      <c r="F67" s="32" t="n"/>
+    </row>
+    <row r="68" ht="56" customHeight="1">
+      <c r="A68" s="10" t="inlineStr">
         <is>
           <t>How the agent is stopped, and by whom</t>
         </is>
       </c>
-      <c r="B61" s="15" t="n"/>
-      <c r="C61" s="35" t="n"/>
-      <c r="D61" s="36" t="n"/>
-      <c r="E61" s="36" t="n"/>
-      <c r="F61" s="34" t="n"/>
-    </row>
-    <row r="62" ht="13" customHeight="1">
-      <c r="A62" s="13" t="inlineStr">
+      <c r="B68" s="15" t="n"/>
+      <c r="C68" s="35" t="n"/>
+      <c r="D68" s="36" t="n"/>
+      <c r="E68" s="36" t="n"/>
+      <c r="F68" s="34" t="n"/>
+    </row>
+    <row r="69" ht="13" customHeight="1">
+      <c r="A69" s="13" t="inlineStr">
         <is>
           <t>Point at section 5 of the design document rather than restating it. Say who is on call.</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="56" customHeight="1">
-      <c r="A63" s="10" t="inlineStr">
+    <row r="70" ht="56" customHeight="1">
+      <c r="A70" s="10" t="inlineStr">
         <is>
           <t>What you tell a customer, and who decides</t>
         </is>
       </c>
-      <c r="B63" s="15" t="n"/>
-      <c r="C63" s="35" t="n"/>
-      <c r="D63" s="36" t="n"/>
-      <c r="E63" s="36" t="n"/>
-      <c r="F63" s="34" t="n"/>
-    </row>
-    <row r="64" ht="13" customHeight="1">
-      <c r="A64" s="13" t="inlineStr">
+      <c r="B70" s="15" t="n"/>
+      <c r="C70" s="35" t="n"/>
+      <c r="D70" s="36" t="n"/>
+      <c r="E70" s="36" t="n"/>
+      <c r="F70" s="34" t="n"/>
+    </row>
+    <row r="71" ht="13" customHeight="1">
+      <c r="A71" s="13" t="inlineStr">
         <is>
           <t>For any agent where the person on the other end is not internal staff.</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="26" customHeight="1">
-      <c r="A65" s="32" t="n"/>
-      <c r="B65" s="32" t="n"/>
-      <c r="C65" s="32" t="n"/>
-      <c r="D65" s="32" t="n"/>
-      <c r="E65" s="32" t="n"/>
-      <c r="F65" s="32" t="n"/>
-    </row>
-    <row r="66" ht="22" customHeight="1">
-      <c r="A66" s="9" t="inlineStr">
-        <is>
-          <t>E.  The failure modes this playbook covers</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="38" customHeight="1">
-      <c r="A67" s="13" t="inlineStr">
-        <is>
-          <t>Agents fail in ways ordinary software does not. Write what you would do, or write "not covered" and let the sign-off carry it. Drawn from the OWASP Top 10 for Agentic Applications. The OWASP column names the entry each row comes from. ASI05, unexpected code execution, has no row: add one if your agent can run code it composed itself.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="30" customHeight="1">
-      <c r="A68" s="14" t="inlineStr">
-        <is>
-          <t>Failure mode</t>
-        </is>
-      </c>
-      <c r="B68" s="14" t="inlineStr">
-        <is>
-          <t>OWASP</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>What you do</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="30" customHeight="1">
-      <c r="A69" s="25" t="inlineStr">
-        <is>
-          <t>The agent calls a tool outside its declared set</t>
-        </is>
-      </c>
-      <c r="B69" s="25" t="inlineStr">
-        <is>
-          <t>ASI02, ASI03</t>
-        </is>
-      </c>
-      <c r="C69" s="32" t="n"/>
-      <c r="D69" s="32" t="n"/>
-      <c r="E69" s="32" t="n"/>
-      <c r="F69" s="32" t="n"/>
-    </row>
-    <row r="70" ht="30" customHeight="1">
-      <c r="A70" s="25" t="inlineStr">
-        <is>
-          <t>A chain of tool calls each succeeds but the outcome is wrong</t>
-        </is>
-      </c>
-      <c r="B70" s="25" t="inlineStr">
-        <is>
-          <t>ASI08</t>
-        </is>
-      </c>
-      <c r="C70" s="32" t="n"/>
-      <c r="D70" s="32" t="n"/>
-      <c r="E70" s="32" t="n"/>
-      <c r="F70" s="32" t="n"/>
-    </row>
-    <row r="71" ht="30" customHeight="1">
-      <c r="A71" s="25" t="inlineStr">
-        <is>
-          <t>Prompt injection through content the agent reads</t>
-        </is>
-      </c>
-      <c r="B71" s="25" t="inlineStr">
-        <is>
-          <t>ASI01</t>
-        </is>
-      </c>
-      <c r="C71" s="32" t="n"/>
-      <c r="D71" s="32" t="n"/>
-      <c r="E71" s="32" t="n"/>
-      <c r="F71" s="32" t="n"/>
-    </row>
-    <row r="72" ht="30" customHeight="1">
-      <c r="A72" s="25" t="inlineStr">
-        <is>
-          <t>Scope creep: used for work it was not designed for</t>
-        </is>
-      </c>
-      <c r="B72" s="25" t="inlineStr">
-        <is>
-          <t>ASI09</t>
-        </is>
-      </c>
+    <row r="72" ht="26" customHeight="1">
+      <c r="A72" s="32" t="n"/>
+      <c r="B72" s="32" t="n"/>
       <c r="C72" s="32" t="n"/>
       <c r="D72" s="32" t="n"/>
       <c r="E72" s="32" t="n"/>
       <c r="F72" s="32" t="n"/>
     </row>
-    <row r="73" ht="30" customHeight="1">
-      <c r="A73" s="25" t="inlineStr">
-        <is>
-          <t>The agent loops, or runs away on cost</t>
-        </is>
-      </c>
-      <c r="B73" s="25" t="inlineStr">
-        <is>
-          <t>ASI08</t>
-        </is>
-      </c>
-      <c r="C73" s="32" t="n"/>
-      <c r="D73" s="32" t="n"/>
-      <c r="E73" s="32" t="n"/>
-      <c r="F73" s="32" t="n"/>
-    </row>
-    <row r="74" ht="30" customHeight="1">
-      <c r="A74" s="25" t="inlineStr">
-        <is>
-          <t>A model or framework update changes behavior with no code change</t>
-        </is>
-      </c>
-      <c r="B74" s="25" t="inlineStr">
-        <is>
-          <t>ASI04</t>
-        </is>
-      </c>
-      <c r="C74" s="32" t="n"/>
-      <c r="D74" s="32" t="n"/>
-      <c r="E74" s="32" t="n"/>
-      <c r="F74" s="32" t="n"/>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="9" t="inlineStr">
+        <is>
+          <t>E.  The failure modes this playbook covers</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="38" customHeight="1">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>Agents fail in ways ordinary software does not. Write what you would do, or write "not covered" and let the sign-off carry it. Where a row does not apply, write "the agent cannot do this" rather than leaving it blank. Drawn from the OWASP Top 10 for Agentic Applications; the OWASP column names the entry each row comes from.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="30" customHeight="1">
-      <c r="A75" s="25" t="inlineStr">
-        <is>
-          <t>Memory or retrieved context has been poisoned</t>
-        </is>
-      </c>
-      <c r="B75" s="25" t="inlineStr">
-        <is>
-          <t>ASI06</t>
-        </is>
-      </c>
-      <c r="C75" s="32" t="n"/>
-      <c r="D75" s="32" t="n"/>
-      <c r="E75" s="32" t="n"/>
-      <c r="F75" s="32" t="n"/>
+      <c r="A75" s="14" t="inlineStr">
+        <is>
+          <t>Failure mode</t>
+        </is>
+      </c>
+      <c r="B75" s="14" t="inlineStr">
+        <is>
+          <t>OWASP</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>What you do</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="25" t="inlineStr">
         <is>
-          <t>The agent is confidently wrong and a person acts on it</t>
+          <t>The agent calls a tool outside its declared set</t>
         </is>
       </c>
       <c r="B76" s="25" t="inlineStr">
         <is>
-          <t>ASI09</t>
+          <t>ASI02, ASI03</t>
         </is>
       </c>
       <c r="C76" s="32" t="n"/>
@@ -4557,12 +4509,12 @@
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="25" t="inlineStr">
         <is>
-          <t>The agent stops escalating when it should</t>
+          <t>A chain of tool calls each succeeds but the outcome is wrong</t>
         </is>
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>ASI09</t>
+          <t>ASI08</t>
         </is>
       </c>
       <c r="C77" s="32" t="n"/>
@@ -4573,12 +4525,12 @@
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="25" t="inlineStr">
         <is>
-          <t>A supervising agent fails, or supervises wrongly</t>
+          <t>Prompt injection through content the agent reads</t>
         </is>
       </c>
       <c r="B78" s="25" t="inlineStr">
         <is>
-          <t>ASI07, ASI10</t>
+          <t>ASI01</t>
         </is>
       </c>
       <c r="C78" s="32" t="n"/>
@@ -4586,224 +4538,364 @@
       <c r="E78" s="32" t="n"/>
       <c r="F78" s="32" t="n"/>
     </row>
-    <row r="79" ht="26" customHeight="1">
-      <c r="A79" s="32" t="n"/>
-      <c r="B79" s="32" t="n"/>
+    <row r="79" ht="30" customHeight="1">
+      <c r="A79" s="25" t="inlineStr">
+        <is>
+          <t>Scope creep: used for work it was not designed for</t>
+        </is>
+      </c>
+      <c r="B79" s="25" t="inlineStr">
+        <is>
+          <t>ASI09</t>
+        </is>
+      </c>
       <c r="C79" s="32" t="n"/>
       <c r="D79" s="32" t="n"/>
       <c r="E79" s="32" t="n"/>
       <c r="F79" s="32" t="n"/>
     </row>
-    <row r="80" ht="22" customHeight="1">
-      <c r="A80" s="9" t="inlineStr">
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="25" t="inlineStr">
+        <is>
+          <t>The agent loops, or runs away on cost</t>
+        </is>
+      </c>
+      <c r="B80" s="25" t="inlineStr">
+        <is>
+          <t>ASI08</t>
+        </is>
+      </c>
+      <c r="C80" s="32" t="n"/>
+      <c r="D80" s="32" t="n"/>
+      <c r="E80" s="32" t="n"/>
+      <c r="F80" s="32" t="n"/>
+    </row>
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="25" t="inlineStr">
+        <is>
+          <t>A model or framework update changes behavior with no code change</t>
+        </is>
+      </c>
+      <c r="B81" s="25" t="inlineStr">
+        <is>
+          <t>ASI04</t>
+        </is>
+      </c>
+      <c r="C81" s="32" t="n"/>
+      <c r="D81" s="32" t="n"/>
+      <c r="E81" s="32" t="n"/>
+      <c r="F81" s="32" t="n"/>
+    </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="25" t="inlineStr">
+        <is>
+          <t>Memory or retrieved context has been poisoned</t>
+        </is>
+      </c>
+      <c r="B82" s="25" t="inlineStr">
+        <is>
+          <t>ASI06</t>
+        </is>
+      </c>
+      <c r="C82" s="32" t="n"/>
+      <c r="D82" s="32" t="n"/>
+      <c r="E82" s="32" t="n"/>
+      <c r="F82" s="32" t="n"/>
+    </row>
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="25" t="inlineStr">
+        <is>
+          <t>The agent is confidently wrong and a person acts on it</t>
+        </is>
+      </c>
+      <c r="B83" s="25" t="inlineStr">
+        <is>
+          <t>ASI09</t>
+        </is>
+      </c>
+      <c r="C83" s="32" t="n"/>
+      <c r="D83" s="32" t="n"/>
+      <c r="E83" s="32" t="n"/>
+      <c r="F83" s="32" t="n"/>
+    </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="25" t="inlineStr">
+        <is>
+          <t>The agent stops escalating when it should</t>
+        </is>
+      </c>
+      <c r="B84" s="25" t="inlineStr">
+        <is>
+          <t>ASI09</t>
+        </is>
+      </c>
+      <c r="C84" s="32" t="n"/>
+      <c r="D84" s="32" t="n"/>
+      <c r="E84" s="32" t="n"/>
+      <c r="F84" s="32" t="n"/>
+    </row>
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="25" t="inlineStr">
+        <is>
+          <t>The agent runs code or shell commands it composed itself</t>
+        </is>
+      </c>
+      <c r="B85" s="25" t="inlineStr">
+        <is>
+          <t>ASI05</t>
+        </is>
+      </c>
+      <c r="C85" s="32" t="n"/>
+      <c r="D85" s="32" t="n"/>
+      <c r="E85" s="32" t="n"/>
+      <c r="F85" s="32" t="n"/>
+    </row>
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="25" t="inlineStr">
+        <is>
+          <t>A supervising agent fails, or supervises wrongly</t>
+        </is>
+      </c>
+      <c r="B86" s="25" t="inlineStr">
+        <is>
+          <t>ASI07, ASI10</t>
+        </is>
+      </c>
+      <c r="C86" s="32" t="n"/>
+      <c r="D86" s="32" t="n"/>
+      <c r="E86" s="32" t="n"/>
+      <c r="F86" s="32" t="n"/>
+    </row>
+    <row r="87" ht="26" customHeight="1">
+      <c r="A87" s="32" t="n"/>
+      <c r="B87" s="32" t="n"/>
+      <c r="C87" s="32" t="n"/>
+      <c r="D87" s="32" t="n"/>
+      <c r="E87" s="32" t="n"/>
+      <c r="F87" s="32" t="n"/>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="9" t="inlineStr">
         <is>
           <t>F.  Revision history</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="30" customHeight="1">
-      <c r="A81" s="14" t="inlineStr">
+    <row r="89" ht="30" customHeight="1">
+      <c r="A89" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B81" s="14" t="inlineStr">
+      <c r="B89" s="14" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="C81" s="14" t="inlineStr">
+      <c r="C89" s="14" t="inlineStr">
         <is>
           <t>What changed</t>
         </is>
       </c>
-      <c r="D81" s="14" t="inlineStr">
+      <c r="D89" s="14" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="E81" s="14" t="inlineStr">
+      <c r="E89" s="14" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="F81" s="15" t="n"/>
-    </row>
-    <row r="82" ht="30" customHeight="1">
-      <c r="A82" s="35" t="n"/>
-      <c r="B82" s="35" t="n"/>
-      <c r="C82" s="35" t="n"/>
-      <c r="D82" s="35" t="n"/>
-      <c r="E82" s="35" t="n"/>
-      <c r="F82" s="34" t="n"/>
-    </row>
-    <row r="83" ht="30" customHeight="1">
-      <c r="A83" s="35" t="n"/>
-      <c r="B83" s="35" t="n"/>
-      <c r="C83" s="35" t="n"/>
-      <c r="D83" s="35" t="n"/>
-      <c r="E83" s="35" t="n"/>
-      <c r="F83" s="34" t="n"/>
-    </row>
-    <row r="84" ht="30" customHeight="1">
-      <c r="A84" s="35" t="n"/>
-      <c r="B84" s="35" t="n"/>
-      <c r="C84" s="35" t="n"/>
-      <c r="D84" s="35" t="n"/>
-      <c r="E84" s="35" t="n"/>
-      <c r="F84" s="34" t="n"/>
-    </row>
-    <row r="85" ht="30" customHeight="1">
-      <c r="A85" s="35" t="n"/>
-      <c r="B85" s="35" t="n"/>
-      <c r="C85" s="35" t="n"/>
-      <c r="D85" s="35" t="n"/>
-      <c r="E85" s="35" t="n"/>
-      <c r="F85" s="34" t="n"/>
-    </row>
-    <row r="86" ht="30" customHeight="1">
-      <c r="A86" s="35" t="n"/>
-      <c r="B86" s="35" t="n"/>
-      <c r="C86" s="35" t="n"/>
-      <c r="D86" s="35" t="n"/>
-      <c r="E86" s="35" t="n"/>
-      <c r="F86" s="34" t="n"/>
-    </row>
-    <row r="87" ht="30" customHeight="1">
-      <c r="A87" s="35" t="n"/>
-      <c r="B87" s="35" t="n"/>
-      <c r="C87" s="35" t="n"/>
-      <c r="D87" s="35" t="n"/>
-      <c r="E87" s="35" t="n"/>
-      <c r="F87" s="34" t="n"/>
-    </row>
-    <row r="88" ht="30" customHeight="1">
-      <c r="A88" s="35" t="n"/>
-      <c r="B88" s="35" t="n"/>
-      <c r="C88" s="35" t="n"/>
-      <c r="D88" s="35" t="n"/>
-      <c r="E88" s="35" t="n"/>
-      <c r="F88" s="34" t="n"/>
-    </row>
-    <row r="89" ht="30" customHeight="1">
-      <c r="A89" s="35" t="n"/>
-      <c r="B89" s="35" t="n"/>
-      <c r="C89" s="35" t="n"/>
-      <c r="D89" s="35" t="n"/>
-      <c r="E89" s="35" t="n"/>
-      <c r="F89" s="34" t="n"/>
+      <c r="F89" s="15" t="n"/>
+    </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="35" t="n"/>
+      <c r="B90" s="35" t="n"/>
+      <c r="C90" s="35" t="n"/>
+      <c r="D90" s="35" t="n"/>
+      <c r="E90" s="35" t="n"/>
+      <c r="F90" s="34" t="n"/>
+    </row>
+    <row r="91" ht="30" customHeight="1">
+      <c r="A91" s="35" t="n"/>
+      <c r="B91" s="35" t="n"/>
+      <c r="C91" s="35" t="n"/>
+      <c r="D91" s="35" t="n"/>
+      <c r="E91" s="35" t="n"/>
+      <c r="F91" s="34" t="n"/>
+    </row>
+    <row r="92" ht="30" customHeight="1">
+      <c r="A92" s="35" t="n"/>
+      <c r="B92" s="35" t="n"/>
+      <c r="C92" s="35" t="n"/>
+      <c r="D92" s="35" t="n"/>
+      <c r="E92" s="35" t="n"/>
+      <c r="F92" s="34" t="n"/>
+    </row>
+    <row r="93" ht="30" customHeight="1">
+      <c r="A93" s="35" t="n"/>
+      <c r="B93" s="35" t="n"/>
+      <c r="C93" s="35" t="n"/>
+      <c r="D93" s="35" t="n"/>
+      <c r="E93" s="35" t="n"/>
+      <c r="F93" s="34" t="n"/>
+    </row>
+    <row r="94" ht="30" customHeight="1">
+      <c r="A94" s="35" t="n"/>
+      <c r="B94" s="35" t="n"/>
+      <c r="C94" s="35" t="n"/>
+      <c r="D94" s="35" t="n"/>
+      <c r="E94" s="35" t="n"/>
+      <c r="F94" s="34" t="n"/>
+    </row>
+    <row r="95" ht="30" customHeight="1">
+      <c r="A95" s="35" t="n"/>
+      <c r="B95" s="35" t="n"/>
+      <c r="C95" s="35" t="n"/>
+      <c r="D95" s="35" t="n"/>
+      <c r="E95" s="35" t="n"/>
+      <c r="F95" s="34" t="n"/>
+    </row>
+    <row r="96" ht="30" customHeight="1">
+      <c r="A96" s="35" t="n"/>
+      <c r="B96" s="35" t="n"/>
+      <c r="C96" s="35" t="n"/>
+      <c r="D96" s="35" t="n"/>
+      <c r="E96" s="35" t="n"/>
+      <c r="F96" s="34" t="n"/>
+    </row>
+    <row r="97" ht="30" customHeight="1">
+      <c r="A97" s="35" t="n"/>
+      <c r="B97" s="35" t="n"/>
+      <c r="C97" s="35" t="n"/>
+      <c r="D97" s="35" t="n"/>
+      <c r="E97" s="35" t="n"/>
+      <c r="F97" s="34" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="102">
-    <mergeCell ref="C61:F61"/>
+  <mergeCells count="114">
+    <mergeCell ref="E62:F62"/>
     <mergeCell ref="A66:F66"/>
-    <mergeCell ref="C72:F72"/>
-    <mergeCell ref="A50:F50"/>
     <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C81:F81"/>
+    <mergeCell ref="A70:B70"/>
     <mergeCell ref="C37:F37"/>
-    <mergeCell ref="E87:F87"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="E64:F64"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="E51:F51"/>
     <mergeCell ref="C78:F78"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A38:F38"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="C73:F73"/>
-    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="E63:F63"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C79:F79"/>
+    <mergeCell ref="D23:F23"/>
     <mergeCell ref="E49:F49"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A40:F40"/>
-    <mergeCell ref="C63:F63"/>
     <mergeCell ref="C10:F10"/>
-    <mergeCell ref="A64:F64"/>
     <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="E85:F85"/>
-    <mergeCell ref="E53:F53"/>
+    <mergeCell ref="A73:F73"/>
+    <mergeCell ref="E91:F91"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="E93:F93"/>
+    <mergeCell ref="B63:C63"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="E55:F55"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="E48:F48"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="C69:F69"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="C83:F83"/>
     <mergeCell ref="A37:B37"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="A62:F62"/>
-    <mergeCell ref="B53:C53"/>
     <mergeCell ref="A28:F28"/>
+    <mergeCell ref="E90:F90"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="C40:F40"/>
     <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A88:F88"/>
     <mergeCell ref="D21:F21"/>
-    <mergeCell ref="C71:F71"/>
     <mergeCell ref="E58:F58"/>
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="C76:F76"/>
-    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="E50:F50"/>
     <mergeCell ref="C8:F8"/>
-    <mergeCell ref="E83:F83"/>
+    <mergeCell ref="C82:F82"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A74:F74"/>
+    <mergeCell ref="E52:F52"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="B56:C56"/>
+    <mergeCell ref="E92:F92"/>
     <mergeCell ref="D16:F16"/>
     <mergeCell ref="E44:F44"/>
     <mergeCell ref="B58:C58"/>
+    <mergeCell ref="A71:F71"/>
     <mergeCell ref="C77:F77"/>
     <mergeCell ref="C34:F34"/>
+    <mergeCell ref="E94:F94"/>
+    <mergeCell ref="C86:F86"/>
     <mergeCell ref="D18:F18"/>
     <mergeCell ref="C68:F68"/>
-    <mergeCell ref="E84:F84"/>
+    <mergeCell ref="B60:C60"/>
     <mergeCell ref="B57:C57"/>
+    <mergeCell ref="A53:F53"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="E59:F59"/>
     <mergeCell ref="E46:F46"/>
-    <mergeCell ref="E86:F86"/>
-    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="E95:F95"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="E89:F89"/>
-    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="E61:F61"/>
     <mergeCell ref="D20:F20"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="C84:F84"/>
     <mergeCell ref="E57:F57"/>
-    <mergeCell ref="E54:F54"/>
-    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C80:F80"/>
+    <mergeCell ref="C31:F31"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C12:F12"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E81:F81"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="A40:B40"/>
     <mergeCell ref="E56:F56"/>
-    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E96:F96"/>
+    <mergeCell ref="A65:F65"/>
     <mergeCell ref="C70:F70"/>
-    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="B62:C62"/>
     <mergeCell ref="B59:C59"/>
-    <mergeCell ref="A80:F80"/>
     <mergeCell ref="C7:F7"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="E88:F88"/>
-    <mergeCell ref="E82:F82"/>
+    <mergeCell ref="C38:F38"/>
     <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="C74:F74"/>
-    <mergeCell ref="A52:F52"/>
+    <mergeCell ref="E60:F60"/>
+    <mergeCell ref="A43:F43"/>
     <mergeCell ref="C35:F35"/>
-    <mergeCell ref="A67:F67"/>
     <mergeCell ref="E45:F45"/>
     <mergeCell ref="C25:F25"/>
+    <mergeCell ref="C85:F85"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="D19:F19"/>
     <mergeCell ref="C75:F75"/>
-    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A6:F6"/>
+    <mergeCell ref="E97:F97"/>
     <mergeCell ref="C11:F11"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A69:F69"/>
     <mergeCell ref="E47:F47"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="C10 C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C10 C11 C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Level 1,Level 2,Level 3"</formula1>
     </dataValidation>
-    <dataValidation sqref="B15:B21 E42:E49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B17:B23 E45:E52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Partly"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Ask whether one person's data can be removed, and log what the agent remembers.
Add the memory row to both the log rules and the retention table, so what an
agent carries between runs is governed like everything else it holds. Ask each
agent whether one person's data can be found and removed from those records,
and name the privacy regime as a standard the rules already sit under. Name
who is accountable for reading the eval results. Add stage 5 to the corrective
loop, since a standard short a case is a finding too. Update the workbook.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -4918,7 +4918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4932,7 +4932,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Audit and Assurance Record  —  sections A to E</t>
+          <t>Audit and Assurance Record  —  sections A to F</t>
         </is>
       </c>
     </row>
@@ -5108,19 +5108,19 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>Model, tool and prompt versions in play on a run</t>
+          <t>What the agent remembers between runs</t>
         </is>
       </c>
       <c r="B17" s="35" t="n"/>
       <c r="C17" s="35" t="n"/>
       <c r="D17" s="35" t="n"/>
       <c r="E17" s="35" t="n"/>
-      <c r="F17" s="34" t="n"/>
+      <c r="F17" s="35" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>Escalations and their outcomes</t>
+          <t>Model, tool and prompt versions in play on a run</t>
         </is>
       </c>
       <c r="B18" s="35" t="n"/>
@@ -5132,7 +5132,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>Decisions the agent took alone</t>
+          <t>Escalations and their outcomes</t>
         </is>
       </c>
       <c r="B19" s="35" t="n"/>
@@ -5144,7 +5144,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>Sign-off records</t>
+          <t>Decisions the agent took alone</t>
         </is>
       </c>
       <c r="B20" s="35" t="n"/>
@@ -5156,7 +5156,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>Design document versions</t>
+          <t>Sign-off records</t>
         </is>
       </c>
       <c r="B21" s="35" t="n"/>
@@ -5168,7 +5168,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>Eval results</t>
+          <t>Design document versions</t>
         </is>
       </c>
       <c r="B22" s="35" t="n"/>
@@ -5180,7 +5180,7 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>Incident records</t>
+          <t>Eval results</t>
         </is>
       </c>
       <c r="B23" s="35" t="n"/>
@@ -5189,114 +5189,114 @@
       <c r="E23" s="35" t="n"/>
       <c r="F23" s="34" t="n"/>
     </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="32" t="n"/>
-      <c r="B24" s="32" t="n"/>
-      <c r="C24" s="32" t="n"/>
-      <c r="D24" s="32" t="n"/>
-      <c r="E24" s="32" t="n"/>
-      <c r="F24" s="32" t="n"/>
-    </row>
-    <row r="25" ht="56" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>Incident records</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="n"/>
+      <c r="C24" s="35" t="n"/>
+      <c r="D24" s="35" t="n"/>
+      <c r="E24" s="35" t="n"/>
+      <c r="F24" s="34" t="n"/>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="32" t="n"/>
+      <c r="B25" s="32" t="n"/>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="32" t="n"/>
+      <c r="E25" s="32" t="n"/>
+      <c r="F25" s="32" t="n"/>
+    </row>
+    <row r="26" ht="56" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Where personal data sits in the rows above, and under what basis it is kept</t>
         </is>
       </c>
-      <c r="B25" s="15" t="n"/>
-      <c r="C25" s="35" t="n"/>
-      <c r="D25" s="36" t="n"/>
-      <c r="E25" s="36" t="n"/>
-      <c r="F25" s="34" t="n"/>
-    </row>
-    <row r="26" ht="13" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="35" t="n"/>
+      <c r="D26" s="36" t="n"/>
+      <c r="E26" s="36" t="n"/>
+      <c r="F26" s="34" t="n"/>
+    </row>
+    <row r="27" ht="13" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Name the fields. Free-text inputs and outputs are where it turns up unplanned.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="56" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
+    <row r="28" ht="56" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Whether one person's data can be found and removed from the rows above, and how long that takes</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="35" t="n"/>
+      <c r="E28" s="35" t="n"/>
+      <c r="F28" s="35" t="n"/>
+    </row>
+    <row r="29" ht="13" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>For records in an append-only store or a trace backend the answer is often no. That is a finding the sign-off carries, not a box to leave blank.</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="13" t="n"/>
+      <c r="F29" s="13" t="n"/>
+    </row>
+    <row r="30" ht="56" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>Which of these rows nothing currently records, and who owns closing that</t>
         </is>
       </c>
-      <c r="B27" s="15" t="n"/>
-      <c r="C27" s="35" t="n"/>
-      <c r="D27" s="36" t="n"/>
-      <c r="E27" s="36" t="n"/>
-      <c r="F27" s="34" t="n"/>
-    </row>
-    <row r="28" ht="13" customHeight="1">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="B30" s="15" t="n"/>
+      <c r="C30" s="35" t="n"/>
+      <c r="D30" s="36" t="n"/>
+      <c r="E30" s="36" t="n"/>
+      <c r="F30" s="34" t="n"/>
+    </row>
+    <row r="31" ht="13" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>A blank read as "yes, we have that" is worse than a stated gap with a name against it.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="32" t="n"/>
-      <c r="B29" s="32" t="n"/>
-      <c r="C29" s="32" t="n"/>
-      <c r="D29" s="32" t="n"/>
-      <c r="E29" s="32" t="n"/>
-      <c r="F29" s="32" t="n"/>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
+    <row r="32" ht="26" customHeight="1">
+      <c r="A32" s="32" t="n"/>
+      <c r="B32" s="32" t="n"/>
+      <c r="C32" s="32" t="n"/>
+      <c r="D32" s="32" t="n"/>
+      <c r="E32" s="32" t="n"/>
+      <c r="F32" s="32" t="n"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>B.  Where this agent departs from the standard</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="26" customHeight="1">
-      <c r="A31" s="13" t="inlineStr">
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>What happens to each kind of record is settled once, for every agent, in the Audit Log Rules standard in the framework repository. Record only the differences here.</t>
         </is>
       </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>Retention that differs from the rule the standard points at, and who agreed it</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="n"/>
-      <c r="C32" s="35" t="n"/>
-      <c r="D32" s="36" t="n"/>
-      <c r="E32" s="36" t="n"/>
-      <c r="F32" s="34" t="n"/>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>Records the standard expects that this agent does not keep, and who accepted that</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n"/>
-      <c r="C33" s="35" t="n"/>
-      <c r="D33" s="36" t="n"/>
-      <c r="E33" s="36" t="n"/>
-      <c r="F33" s="34" t="n"/>
-    </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>Records this agent keeps longer than the applicable rule allows, and on what basis</t>
-        </is>
-      </c>
-      <c r="B34" s="15" t="n"/>
-      <c r="C34" s="35" t="n"/>
-      <c r="D34" s="36" t="n"/>
-      <c r="E34" s="36" t="n"/>
-      <c r="F34" s="34" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
         <is>
-          <t>Anything about this agent the standard did not anticipate</t>
+          <t>Retention that differs from the rule the standard points at, and who agreed it</t>
         </is>
       </c>
       <c r="B35" s="15" t="n"/>
@@ -5305,87 +5305,87 @@
       <c r="E35" s="36" t="n"/>
       <c r="F35" s="34" t="n"/>
     </row>
-    <row r="36" ht="13" customHeight="1">
-      <c r="A36" s="13" t="inlineStr">
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>Records the standard expects that this agent does not keep, and who accepted that</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="n"/>
+      <c r="C36" s="35" t="n"/>
+      <c r="D36" s="36" t="n"/>
+      <c r="E36" s="36" t="n"/>
+      <c r="F36" s="34" t="n"/>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Records this agent keeps longer than the applicable rule allows, and on what basis</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n"/>
+      <c r="C37" s="35" t="n"/>
+      <c r="D37" s="36" t="n"/>
+      <c r="E37" s="36" t="n"/>
+      <c r="F37" s="34" t="n"/>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Anything about this agent the standard did not anticipate</t>
+        </is>
+      </c>
+      <c r="B38" s="15" t="n"/>
+      <c r="C38" s="35" t="n"/>
+      <c r="D38" s="36" t="n"/>
+      <c r="E38" s="36" t="n"/>
+      <c r="F38" s="34" t="n"/>
+    </row>
+    <row r="39" ht="13" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>The last row is the useful one. An agent that does not fit the standard means the standard is short a case, and that belongs in its revision history.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="26" customHeight="1">
-      <c r="A37" s="32" t="n"/>
-      <c r="B37" s="32" t="n"/>
-      <c r="C37" s="32" t="n"/>
-      <c r="D37" s="32" t="n"/>
-      <c r="E37" s="32" t="n"/>
-      <c r="F37" s="32" t="n"/>
-    </row>
-    <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="9" t="inlineStr">
+    <row r="40" ht="26" customHeight="1">
+      <c r="A40" s="32" t="n"/>
+      <c r="B40" s="32" t="n"/>
+      <c r="C40" s="32" t="n"/>
+      <c r="D40" s="32" t="n"/>
+      <c r="E40" s="32" t="n"/>
+      <c r="F40" s="32" t="n"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>C.  Assurance: the evals, and who reads them</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="38" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
+    <row r="42" ht="38" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>Sheet 4 says what starts the evals. This is not a second copy of their output: if they run on every deploy, or continuously against live traffic, the runs live in your eval system and there are thousands of them. What is needed here is where the signal comes from, whether it is still arriving, and what a person concluded from it.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="56" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="10" t="inlineStr">
+        <is>
+          <t>Who is accountable for reading these results, by name</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="n"/>
+      <c r="C43" s="35" t="n"/>
+      <c r="D43" s="35" t="n"/>
+      <c r="E43" s="35" t="n"/>
+      <c r="F43" s="35" t="n"/>
+    </row>
+    <row r="44" ht="56" customHeight="1">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>Which evals run continuously, and against what traffic</t>
-        </is>
-      </c>
-      <c r="B40" s="15" t="n"/>
-      <c r="C40" s="35" t="n"/>
-      <c r="D40" s="36" t="n"/>
-      <c r="E40" s="36" t="n"/>
-      <c r="F40" s="34" t="n"/>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>Which run on a deploy, and which on a fixed schedule</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="n"/>
-      <c r="C41" s="35" t="n"/>
-      <c r="D41" s="36" t="n"/>
-      <c r="E41" s="36" t="n"/>
-      <c r="F41" s="34" t="n"/>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>Where the results are held</t>
-        </is>
-      </c>
-      <c r="B42" s="15" t="n"/>
-      <c r="C42" s="35" t="n"/>
-      <c r="D42" s="36" t="n"/>
-      <c r="E42" s="36" t="n"/>
-      <c r="F42" s="34" t="n"/>
-    </row>
-    <row r="43" ht="56" customHeight="1">
-      <c r="A43" s="10" t="inlineStr">
-        <is>
-          <t>Current results against the baseline recorded at sign-off</t>
-        </is>
-      </c>
-      <c r="B43" s="15" t="n"/>
-      <c r="C43" s="35" t="n"/>
-      <c r="D43" s="36" t="n"/>
-      <c r="E43" s="36" t="n"/>
-      <c r="F43" s="34" t="n"/>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>What alerts on a regression, and who receives it</t>
         </is>
       </c>
       <c r="B44" s="15" t="n"/>
@@ -5397,7 +5397,7 @@
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="10" t="inlineStr">
         <is>
-          <t>How you would know the evals had stopped running</t>
+          <t>Which run on a deploy, and which on a fixed schedule</t>
         </is>
       </c>
       <c r="B45" s="15" t="n"/>
@@ -5406,10 +5406,10 @@
       <c r="E45" s="36" t="n"/>
       <c r="F45" s="34" t="n"/>
     </row>
-    <row r="46" ht="56" customHeight="1">
+    <row r="46" ht="30" customHeight="1">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>When the eval set was last extended, and what prompted it</t>
+          <t>Where the results are held</t>
         </is>
       </c>
       <c r="B46" s="15" t="n"/>
@@ -5418,87 +5418,103 @@
       <c r="E46" s="36" t="n"/>
       <c r="F46" s="34" t="n"/>
     </row>
-    <row r="47" ht="26" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
+    <row r="47" ht="56" customHeight="1">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>Current results against the baseline recorded at sign-off</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="n"/>
+      <c r="C47" s="35" t="n"/>
+      <c r="D47" s="36" t="n"/>
+      <c r="E47" s="36" t="n"/>
+      <c r="F47" s="34" t="n"/>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>What alerts on a regression, and who receives it</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="n"/>
+      <c r="C48" s="35" t="n"/>
+      <c r="D48" s="36" t="n"/>
+      <c r="E48" s="36" t="n"/>
+      <c r="F48" s="34" t="n"/>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>How you would know the evals had stopped running</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="n"/>
+      <c r="C49" s="35" t="n"/>
+      <c r="D49" s="36" t="n"/>
+      <c r="E49" s="36" t="n"/>
+      <c r="F49" s="34" t="n"/>
+    </row>
+    <row r="50" ht="56" customHeight="1">
+      <c r="A50" s="10" t="inlineStr">
+        <is>
+          <t>When the eval set was last extended, and what prompted it</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="n"/>
+      <c r="C50" s="35" t="n"/>
+      <c r="D50" s="36" t="n"/>
+      <c r="E50" s="36" t="n"/>
+      <c r="F50" s="34" t="n"/>
+    </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="13" t="inlineStr">
         <is>
           <t>Running continuously shows the suite still works. It does not show the suite still covers the agent: new tools, new failure modes and new scope need new evals, and an unchanged eval set against a changed agent goes green for the wrong reason.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="26" customHeight="1">
-      <c r="A48" s="32" t="n"/>
-      <c r="B48" s="32" t="n"/>
-      <c r="C48" s="32" t="n"/>
-      <c r="D48" s="32" t="n"/>
-      <c r="E48" s="32" t="n"/>
-      <c r="F48" s="32" t="n"/>
-    </row>
-    <row r="49" ht="26" customHeight="1">
-      <c r="A49" s="13" t="inlineStr">
+    <row r="52" ht="26" customHeight="1">
+      <c r="A52" s="32" t="n"/>
+      <c r="B52" s="32" t="n"/>
+      <c r="C52" s="32" t="n"/>
+      <c r="D52" s="32" t="n"/>
+      <c r="E52" s="32" t="n"/>
+      <c r="F52" s="32" t="n"/>
+    </row>
+    <row r="53" ht="26" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
         <is>
           <t>The review. One row per occasion somebody read the results and reached a conclusion. This is the record that shows somebody is still checking, on a date after the sign-off.</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="14" t="inlineStr">
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B50" s="14" t="inlineStr">
+      <c r="B54" s="14" t="inlineStr">
         <is>
           <t>What period or runs were reviewed</t>
         </is>
       </c>
-      <c r="C50" s="14" t="inlineStr">
+      <c r="C54" s="14" t="inlineStr">
         <is>
           <t>What the evals covered</t>
         </is>
       </c>
-      <c r="D50" s="14" t="inlineStr">
+      <c r="D54" s="14" t="inlineStr">
         <is>
           <t>What the results showed, and what changed</t>
         </is>
       </c>
-      <c r="E50" s="14" t="inlineStr">
+      <c r="E54" s="14" t="inlineStr">
         <is>
           <t>Who reviewed, and where the evidence is</t>
         </is>
       </c>
-      <c r="F50" s="15" t="n"/>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="37" t="n"/>
-      <c r="B51" s="35" t="n"/>
-      <c r="C51" s="35" t="n"/>
-      <c r="D51" s="35" t="n"/>
-      <c r="E51" s="35" t="n"/>
-      <c r="F51" s="34" t="n"/>
-    </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="37" t="n"/>
-      <c r="B52" s="35" t="n"/>
-      <c r="C52" s="35" t="n"/>
-      <c r="D52" s="35" t="n"/>
-      <c r="E52" s="35" t="n"/>
-      <c r="F52" s="34" t="n"/>
-    </row>
-    <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="37" t="n"/>
-      <c r="B53" s="35" t="n"/>
-      <c r="C53" s="35" t="n"/>
-      <c r="D53" s="35" t="n"/>
-      <c r="E53" s="35" t="n"/>
-      <c r="F53" s="34" t="n"/>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="37" t="n"/>
-      <c r="B54" s="35" t="n"/>
-      <c r="C54" s="35" t="n"/>
-      <c r="D54" s="35" t="n"/>
-      <c r="E54" s="35" t="n"/>
-      <c r="F54" s="34" t="n"/>
+      <c r="F54" s="15" t="n"/>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="37" t="n"/>
@@ -5532,118 +5548,118 @@
       <c r="E58" s="35" t="n"/>
       <c r="F58" s="34" t="n"/>
     </row>
-    <row r="59" ht="32" customHeight="1">
-      <c r="A59" s="10" t="inlineStr">
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="37" t="n"/>
+      <c r="B59" s="35" t="n"/>
+      <c r="C59" s="35" t="n"/>
+      <c r="D59" s="35" t="n"/>
+      <c r="E59" s="35" t="n"/>
+      <c r="F59" s="34" t="n"/>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="37" t="n"/>
+      <c r="B60" s="35" t="n"/>
+      <c r="C60" s="35" t="n"/>
+      <c r="D60" s="35" t="n"/>
+      <c r="E60" s="35" t="n"/>
+      <c r="F60" s="34" t="n"/>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="37" t="n"/>
+      <c r="B61" s="35" t="n"/>
+      <c r="C61" s="35" t="n"/>
+      <c r="D61" s="35" t="n"/>
+      <c r="E61" s="35" t="n"/>
+      <c r="F61" s="34" t="n"/>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="37" t="n"/>
+      <c r="B62" s="35" t="n"/>
+      <c r="C62" s="35" t="n"/>
+      <c r="D62" s="35" t="n"/>
+      <c r="E62" s="35" t="n"/>
+      <c r="F62" s="34" t="n"/>
+    </row>
+    <row r="63" ht="32" customHeight="1">
+      <c r="A63" s="10" t="inlineStr">
         <is>
           <t>The date of the most recent review, and the interval it is meant to run at</t>
         </is>
       </c>
-      <c r="B59" s="15" t="n"/>
-      <c r="C59" s="35" t="n"/>
-      <c r="D59" s="36" t="n"/>
-      <c r="E59" s="36" t="n"/>
-      <c r="F59" s="34" t="n"/>
-    </row>
-    <row r="60" ht="32" customHeight="1">
-      <c r="A60" s="10" t="inlineStr">
+      <c r="B63" s="15" t="n"/>
+      <c r="C63" s="35" t="n"/>
+      <c r="D63" s="36" t="n"/>
+      <c r="E63" s="36" t="n"/>
+      <c r="F63" s="34" t="n"/>
+    </row>
+    <row r="64" ht="32" customHeight="1">
+      <c r="A64" s="10" t="inlineStr">
         <is>
           <t>Whether the signal is still arriving, and whether that interval is being met</t>
         </is>
       </c>
-      <c r="B60" s="15" t="n"/>
-      <c r="C60" s="35" t="n"/>
-      <c r="D60" s="36" t="n"/>
-      <c r="E60" s="36" t="n"/>
-      <c r="F60" s="34" t="n"/>
-    </row>
-    <row r="61" ht="13" customHeight="1">
-      <c r="A61" s="13" t="inlineStr">
+      <c r="B64" s="15" t="n"/>
+      <c r="C64" s="35" t="n"/>
+      <c r="D64" s="36" t="n"/>
+      <c r="E64" s="36" t="n"/>
+      <c r="F64" s="34" t="n"/>
+    </row>
+    <row r="65" ht="13" customHeight="1">
+      <c r="A65" s="13" t="inlineStr">
         <is>
           <t>A stream nobody reads looks identical to a healthy one, and both look identical to a stream that stopped. Say which you have. An assurance record that has gone quiet is itself a finding.</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="26" customHeight="1">
-      <c r="A62" s="32" t="n"/>
-      <c r="B62" s="32" t="n"/>
-      <c r="C62" s="32" t="n"/>
-      <c r="D62" s="32" t="n"/>
-      <c r="E62" s="32" t="n"/>
-      <c r="F62" s="32" t="n"/>
-    </row>
-    <row r="63" ht="22" customHeight="1">
-      <c r="A63" s="9" t="inlineStr">
+    <row r="66" ht="26" customHeight="1">
+      <c r="A66" s="32" t="n"/>
+      <c r="B66" s="32" t="n"/>
+      <c r="C66" s="32" t="n"/>
+      <c r="D66" s="32" t="n"/>
+      <c r="E66" s="32" t="n"/>
+      <c r="F66" s="32" t="n"/>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="9" t="inlineStr">
         <is>
           <t>D.  Findings, and what they changed upstream</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="14" customHeight="1">
-      <c r="A64" s="13" t="inlineStr">
-        <is>
-          <t>Every arrow that runs back up the five stages is evidenced here, or it did not happen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="14" t="inlineStr">
+    <row r="68" ht="14" customHeight="1">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>Every arrow that runs back up the five stages is evidenced here, or it did not happen. Stage 5 is in the list because section B's last row feeds findings back into the Audit Log Rules. A standard short a case is a finding like any other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="A69" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B65" s="14" t="inlineStr">
+      <c r="B69" s="14" t="inlineStr">
         <is>
           <t>What was found</t>
         </is>
       </c>
-      <c r="C65" s="14" t="inlineStr">
+      <c r="C69" s="14" t="inlineStr">
         <is>
           <t>Which stage it corrects</t>
         </is>
       </c>
-      <c r="D65" s="14" t="inlineStr">
+      <c r="D69" s="14" t="inlineStr">
         <is>
           <t>What changed, and who approved it</t>
         </is>
       </c>
-      <c r="E65" s="14" t="inlineStr">
+      <c r="E69" s="14" t="inlineStr">
         <is>
           <t>Change confirmed live</t>
         </is>
       </c>
-      <c r="F65" s="15" t="n"/>
-    </row>
-    <row r="66" ht="30" customHeight="1">
-      <c r="A66" s="37" t="n"/>
-      <c r="B66" s="35" t="n"/>
-      <c r="C66" s="35" t="n"/>
-      <c r="D66" s="35" t="n"/>
-      <c r="E66" s="35" t="n"/>
-      <c r="F66" s="34" t="n"/>
-    </row>
-    <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="37" t="n"/>
-      <c r="B67" s="35" t="n"/>
-      <c r="C67" s="35" t="n"/>
-      <c r="D67" s="35" t="n"/>
-      <c r="E67" s="35" t="n"/>
-      <c r="F67" s="34" t="n"/>
-    </row>
-    <row r="68" ht="30" customHeight="1">
-      <c r="A68" s="37" t="n"/>
-      <c r="B68" s="35" t="n"/>
-      <c r="C68" s="35" t="n"/>
-      <c r="D68" s="35" t="n"/>
-      <c r="E68" s="35" t="n"/>
-      <c r="F68" s="34" t="n"/>
-    </row>
-    <row r="69" ht="30" customHeight="1">
-      <c r="A69" s="37" t="n"/>
-      <c r="B69" s="35" t="n"/>
-      <c r="C69" s="35" t="n"/>
-      <c r="D69" s="35" t="n"/>
-      <c r="E69" s="35" t="n"/>
-      <c r="F69" s="34" t="n"/>
+      <c r="F69" s="15" t="n"/>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="37" t="n"/>
@@ -5669,7 +5685,7 @@
       <c r="E72" s="35" t="n"/>
       <c r="F72" s="34" t="n"/>
     </row>
-    <row r="73" ht="56" customHeight="1">
+    <row r="73" ht="30" customHeight="1">
       <c r="A73" s="37" t="n"/>
       <c r="B73" s="35" t="n"/>
       <c r="C73" s="35" t="n"/>
@@ -5677,107 +5693,91 @@
       <c r="E73" s="35" t="n"/>
       <c r="F73" s="34" t="n"/>
     </row>
-    <row r="74" ht="56" customHeight="1">
-      <c r="A74" s="32" t="n"/>
-      <c r="B74" s="32" t="n"/>
-      <c r="C74" s="32" t="n"/>
-      <c r="D74" s="32" t="n"/>
-      <c r="E74" s="32" t="n"/>
-      <c r="F74" s="32" t="n"/>
-    </row>
-    <row r="75" ht="38" customHeight="1">
-      <c r="A75" s="10" t="inlineStr">
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="37" t="n"/>
+      <c r="B74" s="35" t="n"/>
+      <c r="C74" s="35" t="n"/>
+      <c r="D74" s="35" t="n"/>
+      <c r="E74" s="35" t="n"/>
+      <c r="F74" s="34" t="n"/>
+    </row>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="37" t="n"/>
+      <c r="B75" s="35" t="n"/>
+      <c r="C75" s="35" t="n"/>
+      <c r="D75" s="35" t="n"/>
+      <c r="E75" s="35" t="n"/>
+      <c r="F75" s="34" t="n"/>
+    </row>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="37" t="n"/>
+      <c r="B76" s="35" t="n"/>
+      <c r="C76" s="35" t="n"/>
+      <c r="D76" s="35" t="n"/>
+      <c r="E76" s="35" t="n"/>
+      <c r="F76" s="34" t="n"/>
+    </row>
+    <row r="77" ht="56" customHeight="1">
+      <c r="A77" s="37" t="n"/>
+      <c r="B77" s="35" t="n"/>
+      <c r="C77" s="35" t="n"/>
+      <c r="D77" s="35" t="n"/>
+      <c r="E77" s="35" t="n"/>
+      <c r="F77" s="34" t="n"/>
+    </row>
+    <row r="78" ht="56" customHeight="1">
+      <c r="A78" s="32" t="n"/>
+      <c r="B78" s="32" t="n"/>
+      <c r="C78" s="32" t="n"/>
+      <c r="D78" s="32" t="n"/>
+      <c r="E78" s="32" t="n"/>
+      <c r="F78" s="32" t="n"/>
+    </row>
+    <row r="79" ht="38" customHeight="1">
+      <c r="A79" s="10" t="inlineStr">
         <is>
           <t>Findings raised and not acted on, and why</t>
         </is>
       </c>
-      <c r="B75" s="15" t="n"/>
-      <c r="C75" s="35" t="n"/>
-      <c r="D75" s="36" t="n"/>
-      <c r="E75" s="36" t="n"/>
-      <c r="F75" s="34" t="n"/>
-    </row>
-    <row r="76" ht="13" customHeight="1">
-      <c r="A76" s="13" t="inlineStr">
+      <c r="B79" s="15" t="n"/>
+      <c r="C79" s="35" t="n"/>
+      <c r="D79" s="36" t="n"/>
+      <c r="E79" s="36" t="n"/>
+      <c r="F79" s="34" t="n"/>
+    </row>
+    <row r="80" ht="13" customHeight="1">
+      <c r="A80" s="13" t="inlineStr">
         <is>
           <t>A finding consciously accepted is a legitimate outcome. A finding quietly dropped is not, and from the outside they look identical unless somebody wrote down which happened.</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="26" customHeight="1">
-      <c r="A77" s="32" t="n"/>
-      <c r="B77" s="32" t="n"/>
-      <c r="C77" s="32" t="n"/>
-      <c r="D77" s="32" t="n"/>
-      <c r="E77" s="32" t="n"/>
-      <c r="F77" s="32" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="9" t="inlineStr">
+    <row r="81" ht="26" customHeight="1">
+      <c r="A81" s="32" t="n"/>
+      <c r="B81" s="32" t="n"/>
+      <c r="C81" s="32" t="n"/>
+      <c r="D81" s="32" t="n"/>
+      <c r="E81" s="32" t="n"/>
+      <c r="F81" s="32" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="9" t="inlineStr">
         <is>
           <t>E.  When this agent is retired</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="46" customHeight="1">
-      <c r="A79" s="13" t="inlineStr">
+    <row r="83" ht="46" customHeight="1">
+      <c r="A83" s="13" t="inlineStr">
         <is>
           <t>An agent gets switched off long before the questions about it stop arriving. Four kinds of record in section A outlive it: sign-offs, design document versions, eval results and incident records. All four usually sit on infrastructure that is torn down with the agent. Fill this section in when the agent is retired, and not before.</t>
         </is>
       </c>
-    </row>
-    <row r="80" ht="30" customHeight="1">
-      <c r="A80" s="10" t="inlineStr">
-        <is>
-          <t>Date it was switched off, and who decided</t>
-        </is>
-      </c>
-      <c r="B80" s="15" t="n"/>
-      <c r="C80" s="35" t="n"/>
-      <c r="D80" s="36" t="n"/>
-      <c r="E80" s="36" t="n"/>
-      <c r="F80" s="34" t="n"/>
-    </row>
-    <row r="81" ht="30" customHeight="1">
-      <c r="A81" s="10" t="inlineStr">
-        <is>
-          <t>Where its agent login and credentials were revoked, and who confirmed that</t>
-        </is>
-      </c>
-      <c r="B81" s="15" t="n"/>
-      <c r="C81" s="35" t="n"/>
-      <c r="D81" s="36" t="n"/>
-      <c r="E81" s="36" t="n"/>
-      <c r="F81" s="34" t="n"/>
-    </row>
-    <row r="82" ht="30" customHeight="1">
-      <c r="A82" s="10" t="inlineStr">
-        <is>
-          <t>Which records in section A were moved, and where they sit now</t>
-        </is>
-      </c>
-      <c r="B82" s="15" t="n"/>
-      <c r="C82" s="35" t="n"/>
-      <c r="D82" s="36" t="n"/>
-      <c r="E82" s="36" t="n"/>
-      <c r="F82" s="34" t="n"/>
-    </row>
-    <row r="83" ht="30" customHeight="1">
-      <c r="A83" s="10" t="inlineStr">
-        <is>
-          <t>Who holds them now</t>
-        </is>
-      </c>
-      <c r="B83" s="15" t="n"/>
-      <c r="C83" s="35" t="n"/>
-      <c r="D83" s="36" t="n"/>
-      <c r="E83" s="36" t="n"/>
-      <c r="F83" s="34" t="n"/>
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>Until when, and under which rule</t>
+          <t>Date it was switched off, and who decided</t>
         </is>
       </c>
       <c r="B84" s="15" t="n"/>
@@ -5789,7 +5789,7 @@
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>Which records were deleted on purpose, and on what basis</t>
+          <t>Where its agent login and credentials were revoked, and who confirmed that</t>
         </is>
       </c>
       <c r="B85" s="15" t="n"/>
@@ -5798,10 +5798,22 @@
       <c r="E85" s="36" t="n"/>
       <c r="F85" s="34" t="n"/>
     </row>
-    <row r="87" ht="56" customHeight="1">
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>Which records in section A were moved, and where they sit now</t>
+        </is>
+      </c>
+      <c r="B86" s="15" t="n"/>
+      <c r="C86" s="35" t="n"/>
+      <c r="D86" s="36" t="n"/>
+      <c r="E86" s="36" t="n"/>
+      <c r="F86" s="34" t="n"/>
+    </row>
+    <row r="87" ht="30" customHeight="1">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>What still points at this agent</t>
+          <t>Who holds them now</t>
         </is>
       </c>
       <c r="B87" s="15" t="n"/>
@@ -5810,17 +5822,22 @@
       <c r="E87" s="36" t="n"/>
       <c r="F87" s="34" t="n"/>
     </row>
-    <row r="88" ht="13" customHeight="1">
-      <c r="A88" s="13" t="inlineStr">
-        <is>
-          <t>Other agents that called it, processes that assumed it, and reports that read its output. Say what happens to each.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="56" customHeight="1">
+    <row r="88" ht="30" customHeight="1">
+      <c r="A88" s="10" t="inlineStr">
+        <is>
+          <t>Until when, and under which rule</t>
+        </is>
+      </c>
+      <c r="B88" s="15" t="n"/>
+      <c r="C88" s="35" t="n"/>
+      <c r="D88" s="36" t="n"/>
+      <c r="E88" s="36" t="n"/>
+      <c r="F88" s="34" t="n"/>
+    </row>
+    <row r="89" ht="30" customHeight="1">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>Who to ask about this agent now</t>
+          <t>Which records were deleted on purpose, and on what basis</t>
         </is>
       </c>
       <c r="B89" s="15" t="n"/>
@@ -5829,79 +5846,80 @@
       <c r="E89" s="36" t="n"/>
       <c r="F89" s="34" t="n"/>
     </row>
-    <row r="90" ht="13" customHeight="1">
-      <c r="A90" s="13" t="inlineStr">
+    <row r="90"/>
+    <row r="91" ht="56" customHeight="1">
+      <c r="A91" s="10" t="inlineStr">
+        <is>
+          <t>What still points at this agent</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="n"/>
+      <c r="C91" s="35" t="n"/>
+      <c r="D91" s="36" t="n"/>
+      <c r="E91" s="36" t="n"/>
+      <c r="F91" s="34" t="n"/>
+    </row>
+    <row r="92" ht="13" customHeight="1">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>Other agents that called it, processes that assumed it, and reports that read its output. Say what happens to each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="56" customHeight="1">
+      <c r="A93" s="10" t="inlineStr">
+        <is>
+          <t>Who to ask about this agent now</t>
+        </is>
+      </c>
+      <c r="B93" s="15" t="n"/>
+      <c r="C93" s="35" t="n"/>
+      <c r="D93" s="36" t="n"/>
+      <c r="E93" s="36" t="n"/>
+      <c r="F93" s="34" t="n"/>
+    </row>
+    <row r="94" ht="13" customHeight="1">
+      <c r="A94" s="13" t="inlineStr">
         <is>
           <t>The owner in section 0 of the design document has probably moved on. Name whoever answers a question about it in three years.</t>
         </is>
       </c>
     </row>
-    <row r="92" ht="22" customHeight="1">
-      <c r="A92" s="9" t="inlineStr">
+    <row r="95"/>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="9" t="inlineStr">
         <is>
           <t>F.  Revision history</t>
         </is>
       </c>
     </row>
-    <row r="93" ht="30" customHeight="1">
-      <c r="A93" s="14" t="inlineStr">
+    <row r="97" ht="30" customHeight="1">
+      <c r="A97" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B93" s="14" t="inlineStr">
+      <c r="B97" s="14" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="C93" s="14" t="inlineStr">
+      <c r="C97" s="14" t="inlineStr">
         <is>
           <t>What changed</t>
         </is>
       </c>
-      <c r="D93" s="14" t="inlineStr">
+      <c r="D97" s="14" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="E93" s="14" t="inlineStr">
+      <c r="E97" s="14" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="F93" s="15" t="n"/>
-    </row>
-    <row r="94" ht="30" customHeight="1">
-      <c r="A94" s="37" t="n"/>
-      <c r="B94" s="35" t="n"/>
-      <c r="C94" s="35" t="n"/>
-      <c r="D94" s="35" t="n"/>
-      <c r="E94" s="35" t="n"/>
-      <c r="F94" s="34" t="n"/>
-    </row>
-    <row r="95" ht="30" customHeight="1">
-      <c r="A95" s="37" t="n"/>
-      <c r="B95" s="35" t="n"/>
-      <c r="C95" s="35" t="n"/>
-      <c r="D95" s="35" t="n"/>
-      <c r="E95" s="35" t="n"/>
-      <c r="F95" s="34" t="n"/>
-    </row>
-    <row r="96" ht="30" customHeight="1">
-      <c r="A96" s="37" t="n"/>
-      <c r="B96" s="35" t="n"/>
-      <c r="C96" s="35" t="n"/>
-      <c r="D96" s="35" t="n"/>
-      <c r="E96" s="35" t="n"/>
-      <c r="F96" s="34" t="n"/>
-    </row>
-    <row r="97" ht="30" customHeight="1">
-      <c r="A97" s="37" t="n"/>
-      <c r="B97" s="35" t="n"/>
-      <c r="C97" s="35" t="n"/>
-      <c r="D97" s="35" t="n"/>
-      <c r="E97" s="35" t="n"/>
-      <c r="F97" s="34" t="n"/>
+      <c r="F97" s="15" t="n"/>
     </row>
     <row r="98" ht="30" customHeight="1">
       <c r="A98" s="37" t="n"/>
@@ -5919,135 +5937,173 @@
       <c r="E99" s="35" t="n"/>
       <c r="F99" s="34" t="n"/>
     </row>
+    <row r="100" ht="30" customHeight="1">
+      <c r="A100" s="37" t="n"/>
+      <c r="B100" s="35" t="n"/>
+      <c r="C100" s="35" t="n"/>
+      <c r="D100" s="35" t="n"/>
+      <c r="E100" s="35" t="n"/>
+      <c r="F100" s="34" t="n"/>
+    </row>
+    <row r="101" ht="30" customHeight="1">
+      <c r="A101" s="37" t="n"/>
+      <c r="B101" s="35" t="n"/>
+      <c r="C101" s="35" t="n"/>
+      <c r="D101" s="35" t="n"/>
+      <c r="E101" s="35" t="n"/>
+      <c r="F101" s="34" t="n"/>
+    </row>
+    <row r="102" ht="30" customHeight="1">
+      <c r="A102" s="37" t="n"/>
+      <c r="B102" s="35" t="n"/>
+      <c r="C102" s="35" t="n"/>
+      <c r="D102" s="35" t="n"/>
+      <c r="E102" s="35" t="n"/>
+      <c r="F102" s="34" t="n"/>
+    </row>
+    <row r="103" ht="30" customHeight="1">
+      <c r="A103" s="37" t="n"/>
+      <c r="B103" s="35" t="n"/>
+      <c r="C103" s="35" t="n"/>
+      <c r="D103" s="35" t="n"/>
+      <c r="E103" s="35" t="n"/>
+      <c r="F103" s="34" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="114">
+  <mergeCells count="120">
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="E62:F62"/>
     <mergeCell ref="E71:F71"/>
     <mergeCell ref="E23:F23"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C81:F81"/>
+    <mergeCell ref="A88:B88"/>
+    <mergeCell ref="C37:F37"/>
     <mergeCell ref="E73:F73"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="A47:F47"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C87:F87"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A29:F29"/>
     <mergeCell ref="C89:F89"/>
-    <mergeCell ref="E65:F65"/>
-    <mergeCell ref="A38:F38"/>
     <mergeCell ref="E99:F99"/>
-    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="C64:F64"/>
+    <mergeCell ref="C79:F79"/>
+    <mergeCell ref="C88:F88"/>
+    <mergeCell ref="C26:F26"/>
     <mergeCell ref="A85:B85"/>
-    <mergeCell ref="A42:B42"/>
     <mergeCell ref="A31:F31"/>
-    <mergeCell ref="C41:F41"/>
+    <mergeCell ref="C63:F63"/>
     <mergeCell ref="C10:F10"/>
-    <mergeCell ref="A64:F64"/>
+    <mergeCell ref="E101:F101"/>
+    <mergeCell ref="C93:F93"/>
+    <mergeCell ref="C50:F50"/>
     <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A82:F82"/>
+    <mergeCell ref="E100:F100"/>
     <mergeCell ref="C43:F43"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="E75:F75"/>
     <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E53:F53"/>
-    <mergeCell ref="E93:F93"/>
-    <mergeCell ref="C27:F27"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="E102:F102"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A30:B30"/>
     <mergeCell ref="E55:F55"/>
     <mergeCell ref="A45:B45"/>
-    <mergeCell ref="E67:F67"/>
+    <mergeCell ref="A27:F27"/>
     <mergeCell ref="E14:F14"/>
+    <mergeCell ref="A79:B79"/>
+    <mergeCell ref="C28:F28"/>
     <mergeCell ref="A87:B87"/>
-    <mergeCell ref="C83:F83"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A42:F42"/>
     <mergeCell ref="A46:B46"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="A37:B37"/>
     <mergeCell ref="A89:B89"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A26:B26"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C40:F40"/>
+    <mergeCell ref="A91:B91"/>
     <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E76:F76"/>
+    <mergeCell ref="A63:B63"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A79:F79"/>
-    <mergeCell ref="A61:F61"/>
-    <mergeCell ref="A88:F88"/>
-    <mergeCell ref="E66:F66"/>
+    <mergeCell ref="A93:B93"/>
     <mergeCell ref="E58:F58"/>
     <mergeCell ref="E18:F18"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A83:B83"/>
-    <mergeCell ref="E50:F50"/>
-    <mergeCell ref="A90:F90"/>
     <mergeCell ref="C8:F8"/>
-    <mergeCell ref="E68:F68"/>
-    <mergeCell ref="C82:F82"/>
-    <mergeCell ref="E52:F52"/>
-    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="C91:F91"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A36:B36"/>
     <mergeCell ref="E20:F20"/>
-    <mergeCell ref="A76:F76"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="E94:F94"/>
-    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="E103:F103"/>
+    <mergeCell ref="C86:F86"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="E69:F69"/>
-    <mergeCell ref="A80:B80"/>
-    <mergeCell ref="A63:F63"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="E59:F59"/>
     <mergeCell ref="C45:F45"/>
+    <mergeCell ref="E77:F77"/>
+    <mergeCell ref="A68:F68"/>
     <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E95:F95"/>
-    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A83:F83"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="C47:F47"/>
     <mergeCell ref="A92:F92"/>
+    <mergeCell ref="E70:F70"/>
     <mergeCell ref="A39:F39"/>
-    <mergeCell ref="E70:F70"/>
     <mergeCell ref="C44:F44"/>
     <mergeCell ref="C84:F84"/>
     <mergeCell ref="E57:F57"/>
-    <mergeCell ref="A49:F49"/>
-    <mergeCell ref="C80:F80"/>
+    <mergeCell ref="A38:B38"/>
     <mergeCell ref="E54:F54"/>
-    <mergeCell ref="A36:F36"/>
     <mergeCell ref="A43:B43"/>
     <mergeCell ref="E72:F72"/>
+    <mergeCell ref="A94:F94"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C46:F46"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A78:F78"/>
     <mergeCell ref="E56:F56"/>
-    <mergeCell ref="C60:F60"/>
-    <mergeCell ref="E96:F96"/>
-    <mergeCell ref="A82:B82"/>
-    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="A65:F65"/>
+    <mergeCell ref="C48:F48"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="A80:F80"/>
     <mergeCell ref="E98:F98"/>
     <mergeCell ref="C7:F7"/>
+    <mergeCell ref="C38:F38"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="E17:F17"/>
-    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C49:F49"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="A84:B84"/>
-    <mergeCell ref="C33:F33"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="C42:F42"/>
+    <mergeCell ref="E60:F60"/>
+    <mergeCell ref="A96:F96"/>
+    <mergeCell ref="E74:F74"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A86:B86"/>
     <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A67:F67"/>
     <mergeCell ref="C85:F85"/>
     <mergeCell ref="C9:F9"/>
-    <mergeCell ref="C75:F75"/>
-    <mergeCell ref="A81:B81"/>
-    <mergeCell ref="C59:F59"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="E97:F97"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="E21:F21"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation sqref="B14:B23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B14:B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Partly,Not known"</formula1>
     </dataValidation>
-    <dataValidation sqref="C66:C73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1,2,3,4"</formula1>
+    <dataValidation sqref="C70:C77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation sqref="E66:E73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E70:E77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Not yet verified"</formula1>
     </dataValidation>
-    <dataValidation sqref="C32:C35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C35:C38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"None,See below"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Move the sign-off after the monitoring rows, so the gate can be answered.
Section C of the sign-off record compares the monitoring level applied with
the one the classification requires, which nobody can answer before the
monitoring record exists. The gate is now row 7. Update the workbook to match.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -230,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -330,6 +330,10 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
@@ -886,7 +890,11 @@
     </row>
     <row r="24" ht="14" customHeight="1">
       <c r="A24" s="32" t="n"/>
-      <c r="B24" s="33" t="inlineStr"/>
+      <c r="B24" s="38" t="inlineStr">
+        <is>
+          <t>Nothing goes live until section C of sheet 3 is signed. Everything on sheets 1, 2 and 4 is what the person signing it reads.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="14" customHeight="1">
       <c r="A25" s="32" t="n"/>
@@ -5115,7 +5123,7 @@
       <c r="C17" s="35" t="n"/>
       <c r="D17" s="35" t="n"/>
       <c r="E17" s="35" t="n"/>
-      <c r="F17" s="35" t="n"/>
+      <c r="F17" s="34" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="25" t="inlineStr">
@@ -5234,11 +5242,11 @@
           <t>Whether one person's data can be found and removed from the rows above, and how long that takes</t>
         </is>
       </c>
-      <c r="B28" s="10" t="n"/>
+      <c r="B28" s="15" t="n"/>
       <c r="C28" s="35" t="n"/>
-      <c r="D28" s="35" t="n"/>
-      <c r="E28" s="35" t="n"/>
-      <c r="F28" s="35" t="n"/>
+      <c r="D28" s="36" t="n"/>
+      <c r="E28" s="36" t="n"/>
+      <c r="F28" s="34" t="n"/>
     </row>
     <row r="29" ht="13" customHeight="1">
       <c r="A29" s="13" t="inlineStr">
@@ -5246,11 +5254,6 @@
           <t>For records in an append-only store or a trace backend the answer is often no. That is a finding the sign-off carries, not a box to leave blank.</t>
         </is>
       </c>
-      <c r="B29" s="13" t="n"/>
-      <c r="C29" s="13" t="n"/>
-      <c r="D29" s="13" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="13" t="n"/>
     </row>
     <row r="30" ht="56" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
@@ -5376,11 +5379,11 @@
           <t>Who is accountable for reading these results, by name</t>
         </is>
       </c>
-      <c r="B43" s="10" t="n"/>
+      <c r="B43" s="15" t="n"/>
       <c r="C43" s="35" t="n"/>
-      <c r="D43" s="35" t="n"/>
-      <c r="E43" s="35" t="n"/>
-      <c r="F43" s="35" t="n"/>
+      <c r="D43" s="36" t="n"/>
+      <c r="E43" s="36" t="n"/>
+      <c r="F43" s="34" t="n"/>
     </row>
     <row r="44" ht="56" customHeight="1">
       <c r="A44" s="10" t="inlineStr">
@@ -5846,7 +5849,6 @@
       <c r="E89" s="36" t="n"/>
       <c r="F89" s="34" t="n"/>
     </row>
-    <row r="90"/>
     <row r="91" ht="56" customHeight="1">
       <c r="A91" s="10" t="inlineStr">
         <is>
@@ -5885,7 +5887,6 @@
         </is>
       </c>
     </row>
-    <row r="95"/>
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix row heights in the workbook so long cells are not clipped.
Six rows across four sheets were sized for shorter text than they now hold.
No content changes.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -1435,7 +1435,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="64" customHeight="1">
+    <row r="44" ht="70" customHeight="1">
       <c r="A44" s="10" t="inlineStr">
         <is>
           <t>What the agent remembers between runs. Conversation history, retrieved documents, learned preferences, or a store it writes to itself. Say who that memory is scoped to — one user, one account, or everybody — and how long it is kept. Write "nothing" if every run starts clean.</t>
@@ -1617,7 +1617,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="64" customHeight="1">
+    <row r="62" ht="83" customHeight="1">
       <c r="A62" s="10" t="inlineStr">
         <is>
           <t>If any row above says "In the prompt", say how the prompt is controlled. Where it lives, who can change it, and whether a change is reviewed before it reaches production. A control written into a prompt that anybody can edit is not a weak control, it is a removable one, and nothing in section 7 will show you that it went.</t>
@@ -1850,7 +1850,7 @@
       <c r="F84" s="34" t="n"/>
       <c r="G84" s="35" t="n"/>
     </row>
-    <row r="85">
+    <row r="85" ht="39" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
           <t>One more tool, a widened scope, or a new audience all produce a row. So do stage 4 and stage 5 findings: an eval that catches drift, an audit finding against your classification criteria, or a monitor reporting a tool call outside section 3. A new model version does not; that changes the Platform and Sign-off Record instead. Retiring the agent produces the last row: set Status above to retired, date it, and fill in section E of the Audit &amp; Assurance sheet.</t>
@@ -3072,7 +3072,7 @@
       <c r="E29" s="36" t="n"/>
       <c r="F29" s="34" t="n"/>
     </row>
-    <row r="30" ht="13" customHeight="1">
+    <row r="30" ht="27" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
           <t>Anything the agent can reach that section 3 does not name. This should be empty. Where it is not, carry it into section C as remaining risk. Do not fix it quietly and leave this blank.</t>
@@ -4257,7 +4257,7 @@
       <c r="E52" s="35" t="n"/>
       <c r="F52" s="34" t="n"/>
     </row>
-    <row r="53" ht="14" customHeight="1">
+    <row r="53" ht="39" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
           <t>Answer the last column for what is implemented today, not what is planned. A row with nothing behind it is a gap the sign-off has to carry. The first row needs the section 3 grant list in a form the monitor can read. It is the only machine-checkable claim in the framework, and naming where the monitor gets it is the difference between an alert you can build and one you intend to.</t>
@@ -5629,7 +5629,7 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="14" customHeight="1">
+    <row r="68" ht="27" customHeight="1">
       <c r="A68" s="13" t="inlineStr">
         <is>
           <t>Every arrow that runs back up the five stages is evidenced here, or it did not happen. Stage 5 is in the list because section B's last row feeds findings back into the Audit Log Rules. A standard short a case is a finding like any other.</t>

</xml_diff>

<commit_message>
Answer the review: rename the stage 4 record, drop the failure-mode label, and require the run's trace.
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -3109,7 +3109,7 @@
     <row r="34" ht="56" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>Adversarial testing performed, and against which failure modes</t>
+          <t>Adversarial testing performed, and what it was tested against</t>
         </is>
       </c>
       <c r="B34" s="15" t="n"/>
@@ -3121,7 +3121,7 @@
     <row r="35" ht="26" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>For any agent that reads content it did not author, whether it can be talked into something is what the sign-off most needs to know. Name the failure modes from OWASP's Top 10 for Agentic Applications, the same list the Monitoring sheet's playbook works from.</t>
+          <t>For any agent that reads content it did not author, whether it can be talked into something is what the sign-off most needs to know. Name what you tested against from OWASP's Top 10 for Agentic Applications, the same list the Monitoring sheet's playbook works from.</t>
         </is>
       </c>
     </row>
@@ -3677,7 +3677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3691,7 +3691,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Monitoring and Incident Record  —  sections A to F</t>
+          <t>Monitoring and Incident Preparedness Record  —  sections A to F</t>
         </is>
       </c>
     </row>
@@ -3911,7 +3911,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>Escalations to a person, and the outcome</t>
+          <t>The agent's steps between the request and the answer</t>
         </is>
       </c>
       <c r="B21" s="35" t="n"/>
@@ -3923,7 +3923,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>Enough of the run to replay it</t>
+          <t>Escalations to a person, and the outcome</t>
         </is>
       </c>
       <c r="B22" s="35" t="n"/>
@@ -3935,7 +3935,7 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>Cost and token use per run</t>
+          <t>Enough of the run to replay it</t>
         </is>
       </c>
       <c r="B23" s="35" t="n"/>
@@ -3944,83 +3944,83 @@
       <c r="E23" s="36" t="n"/>
       <c r="F23" s="34" t="n"/>
     </row>
-    <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="32" t="n"/>
-      <c r="B24" s="32" t="n"/>
-      <c r="C24" s="32" t="n"/>
-      <c r="D24" s="32" t="n"/>
-      <c r="E24" s="32" t="n"/>
-      <c r="F24" s="32" t="n"/>
-    </row>
-    <row r="25" ht="56" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
+    <row r="24" ht="30" customHeight="1">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>Cost and token use per run</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="n"/>
+      <c r="C24" s="35" t="n"/>
+      <c r="D24" s="35" t="n"/>
+      <c r="E24" s="36" t="n"/>
+      <c r="F24" s="34" t="n"/>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="32" t="n"/>
+      <c r="B25" s="32" t="n"/>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="32" t="n"/>
+      <c r="E25" s="32" t="n"/>
+      <c r="F25" s="32" t="n"/>
+    </row>
+    <row r="26" ht="56" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>What you deliberately do NOT record, and why</t>
         </is>
       </c>
-      <c r="B25" s="15" t="n"/>
-      <c r="C25" s="35" t="n"/>
-      <c r="D25" s="36" t="n"/>
-      <c r="E25" s="36" t="n"/>
-      <c r="F25" s="34" t="n"/>
-    </row>
-    <row r="26" ht="13" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="35" t="n"/>
+      <c r="D26" s="36" t="n"/>
+      <c r="E26" s="36" t="n"/>
+      <c r="F26" s="34" t="n"/>
+    </row>
+    <row r="27" ht="13" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Usually personal data you have no basis to retain. Say what you lose by not recording it.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="56" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
+    <row r="28" ht="56" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Who can read these records, and who can change them</t>
         </is>
       </c>
-      <c r="B27" s="15" t="n"/>
-      <c r="C27" s="35" t="n"/>
-      <c r="D27" s="36" t="n"/>
-      <c r="E27" s="36" t="n"/>
-      <c r="F27" s="34" t="n"/>
-    </row>
-    <row r="28" ht="13" customHeight="1">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="B28" s="15" t="n"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="36" t="n"/>
+      <c r="E28" s="36" t="n"/>
+      <c r="F28" s="34" t="n"/>
+    </row>
+    <row r="29" ht="13" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>If the team that operates the agent can edit its own logs, say so here. Stage 5 needs records an auditor will accept.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="32" t="n"/>
-      <c r="B29" s="32" t="n"/>
-      <c r="C29" s="32" t="n"/>
-      <c r="D29" s="32" t="n"/>
-      <c r="E29" s="32" t="n"/>
-      <c r="F29" s="32" t="n"/>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="9" t="inlineStr">
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="32" t="n"/>
+      <c r="B30" s="32" t="n"/>
+      <c r="C30" s="32" t="n"/>
+      <c r="D30" s="32" t="n"/>
+      <c r="E30" s="32" t="n"/>
+      <c r="F30" s="32" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>B.  The evals, and what runs them</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="56" customHeight="1">
-      <c r="A31" s="10" t="inlineStr">
+    <row r="32" ht="56" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>Which evals run against the live agent</t>
-        </is>
-      </c>
-      <c r="B31" s="15" t="n"/>
-      <c r="C31" s="35" t="n"/>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="36" t="n"/>
-      <c r="F31" s="34" t="n"/>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>What starts them</t>
         </is>
       </c>
       <c r="B32" s="15" t="n"/>
@@ -4029,29 +4029,29 @@
       <c r="E32" s="36" t="n"/>
       <c r="F32" s="34" t="n"/>
     </row>
-    <row r="33" ht="13" customHeight="1">
-      <c r="A33" s="13" t="inlineStr">
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>What starts them</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="n"/>
+      <c r="C33" s="35" t="n"/>
+      <c r="D33" s="36" t="n"/>
+      <c r="E33" s="36" t="n"/>
+      <c r="F33" s="34" t="n"/>
+    </row>
+    <row r="34" ht="13" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>A schedule, a deployment, live traffic, or a person. An eval a person has to remember to run is not assurance.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="56" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
+    <row r="35" ht="56" customHeight="1">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>How often, or what share of live traffic if they run continuously</t>
-        </is>
-      </c>
-      <c r="B34" s="15" t="n"/>
-      <c r="C34" s="35" t="n"/>
-      <c r="D34" s="36" t="n"/>
-      <c r="E34" s="36" t="n"/>
-      <c r="F34" s="34" t="n"/>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>Where the results go</t>
         </is>
       </c>
       <c r="B35" s="15" t="n"/>
@@ -4063,7 +4063,7 @@
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>Who is told when one fails</t>
+          <t>Where the results go</t>
         </is>
       </c>
       <c r="B36" s="15" t="n"/>
@@ -4075,7 +4075,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>Who owns extending the eval set as the agent changes</t>
+          <t>Who is told when one fails</t>
         </is>
       </c>
       <c r="B37" s="15" t="n"/>
@@ -4084,10 +4084,10 @@
       <c r="E37" s="36" t="n"/>
       <c r="F37" s="34" t="n"/>
     </row>
-    <row r="38" ht="56" customHeight="1">
+    <row r="38" ht="30" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>How you would know they had stopped running</t>
+          <t>Who owns extending the eval set as the agent changes</t>
         </is>
       </c>
       <c r="B38" s="15" t="n"/>
@@ -4096,91 +4096,91 @@
       <c r="E38" s="36" t="n"/>
       <c r="F38" s="34" t="n"/>
     </row>
-    <row r="39" ht="13" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
+    <row r="39" ht="56" customHeight="1">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>How you would know they had stopped running</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="n"/>
+      <c r="C39" s="35" t="n"/>
+      <c r="D39" s="36" t="n"/>
+      <c r="E39" s="36" t="n"/>
+      <c r="F39" s="34" t="n"/>
+    </row>
+    <row r="40" ht="13" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>A dead scheduler and a continuous job that quietly stopped look the same from outside: everything is green because nothing is running.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="56" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
+    <row r="41" ht="56" customHeight="1">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>Which baseline the results are compared against</t>
         </is>
       </c>
-      <c r="B40" s="15" t="n"/>
-      <c r="C40" s="35" t="n"/>
-      <c r="D40" s="36" t="n"/>
-      <c r="E40" s="36" t="n"/>
-      <c r="F40" s="34" t="n"/>
-    </row>
-    <row r="41" ht="13" customHeight="1">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="B41" s="15" t="n"/>
+      <c r="C41" s="35" t="n"/>
+      <c r="D41" s="36" t="n"/>
+      <c r="E41" s="36" t="n"/>
+      <c r="F41" s="34" t="n"/>
+    </row>
+    <row r="42" ht="13" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>Normally the eval results recorded at sign-off. Name the version.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="32" t="n"/>
-      <c r="B42" s="32" t="n"/>
-      <c r="C42" s="32" t="n"/>
-      <c r="D42" s="32" t="n"/>
-      <c r="E42" s="32" t="n"/>
-      <c r="F42" s="32" t="n"/>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="9" t="inlineStr">
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="32" t="n"/>
+      <c r="B43" s="32" t="n"/>
+      <c r="C43" s="32" t="n"/>
+      <c r="D43" s="32" t="n"/>
+      <c r="E43" s="32" t="n"/>
+      <c r="F43" s="32" t="n"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="9" t="inlineStr">
         <is>
           <t>C.  What counts as normal, and what starts an alert</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="14" t="inlineStr">
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="B44" s="14" t="inlineStr">
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>What normal looks like</t>
         </is>
       </c>
-      <c r="C44" s="14" t="inlineStr">
+      <c r="C45" s="14" t="inlineStr">
         <is>
           <t>What starts an alert</t>
         </is>
       </c>
-      <c r="D44" s="14" t="inlineStr">
+      <c r="D45" s="14" t="inlineStr">
         <is>
           <t>Who receives it</t>
         </is>
       </c>
-      <c r="E44" s="14" t="inlineStr">
+      <c r="E45" s="14" t="inlineStr">
         <is>
           <t>Implemented today</t>
         </is>
       </c>
-      <c r="F44" s="15" t="n"/>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="25" t="inlineStr">
-        <is>
-          <t>A call to a tool outside the declared set</t>
-        </is>
-      </c>
-      <c r="B45" s="35" t="n"/>
-      <c r="C45" s="35" t="n"/>
-      <c r="D45" s="35" t="n"/>
-      <c r="E45" s="35" t="n"/>
-      <c r="F45" s="34" t="n"/>
+      <c r="F45" s="15" t="n"/>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
-          <t>Volume of runs</t>
+          <t>A call to a tool outside the declared set</t>
         </is>
       </c>
       <c r="B46" s="35" t="n"/>
@@ -4192,7 +4192,7 @@
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>Escalation rate to a person</t>
+          <t>Volume of runs</t>
         </is>
       </c>
       <c r="B47" s="35" t="n"/>
@@ -4204,7 +4204,7 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>Eval failure</t>
+          <t>Escalation rate to a person</t>
         </is>
       </c>
       <c r="B48" s="35" t="n"/>
@@ -4216,7 +4216,7 @@
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>Cost per run or per day</t>
+          <t>Eval failure</t>
         </is>
       </c>
       <c r="B49" s="35" t="n"/>
@@ -4228,7 +4228,7 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>Error or retry rate</t>
+          <t>Cost per run or per day</t>
         </is>
       </c>
       <c r="B50" s="35" t="n"/>
@@ -4240,7 +4240,7 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>Drift from the design document</t>
+          <t>Error or retry rate</t>
         </is>
       </c>
       <c r="B51" s="35" t="n"/>
@@ -4250,75 +4250,75 @@
       <c r="F51" s="34" t="n"/>
     </row>
     <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="37" t="n"/>
+      <c r="A52" s="25" t="inlineStr">
+        <is>
+          <t>Drift from the design document</t>
+        </is>
+      </c>
       <c r="B52" s="35" t="n"/>
       <c r="C52" s="35" t="n"/>
       <c r="D52" s="35" t="n"/>
       <c r="E52" s="35" t="n"/>
       <c r="F52" s="34" t="n"/>
     </row>
-    <row r="53" ht="39" customHeight="1">
-      <c r="A53" s="13" t="inlineStr">
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="37" t="n"/>
+      <c r="B53" s="35" t="n"/>
+      <c r="C53" s="35" t="n"/>
+      <c r="D53" s="35" t="n"/>
+      <c r="E53" s="35" t="n"/>
+      <c r="F53" s="34" t="n"/>
+    </row>
+    <row r="54" ht="39" customHeight="1">
+      <c r="A54" s="13" t="inlineStr">
         <is>
           <t>Answer the last column for what is implemented today, not what is planned. A row with nothing behind it is a gap the sign-off has to carry. The first row needs the section 3 grant list in a form the monitor can read. It is the only machine-checkable claim in the framework, and naming where the monitor gets it is the difference between an alert you can build and one you intend to.</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="26" customHeight="1">
-      <c r="A54" s="32" t="n"/>
-      <c r="B54" s="32" t="n"/>
-      <c r="C54" s="32" t="n"/>
-      <c r="D54" s="32" t="n"/>
-      <c r="E54" s="32" t="n"/>
-      <c r="F54" s="32" t="n"/>
-    </row>
-    <row r="55" ht="22" customHeight="1">
-      <c r="A55" s="9" t="inlineStr">
+    <row r="55" ht="26" customHeight="1">
+      <c r="A55" s="32" t="n"/>
+      <c r="B55" s="32" t="n"/>
+      <c r="C55" s="32" t="n"/>
+      <c r="D55" s="32" t="n"/>
+      <c r="E55" s="32" t="n"/>
+      <c r="F55" s="32" t="n"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="9" t="inlineStr">
         <is>
           <t>D.  What an alert starts</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="14" t="inlineStr">
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="14" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="B56" s="14" t="inlineStr">
+      <c r="B57" s="14" t="inlineStr">
         <is>
           <t>What happens</t>
         </is>
       </c>
-      <c r="C56" s="15" t="n"/>
-      <c r="D56" s="14" t="inlineStr">
+      <c r="C57" s="15" t="n"/>
+      <c r="D57" s="14" t="inlineStr">
         <is>
           <t>Who does it</t>
         </is>
       </c>
-      <c r="E56" s="14" t="inlineStr">
+      <c r="E57" s="14" t="inlineStr">
         <is>
           <t>Within what time</t>
         </is>
       </c>
-      <c r="F56" s="15" t="n"/>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="25" t="inlineStr">
-        <is>
-          <t>Triage: is this real</t>
-        </is>
-      </c>
-      <c r="B57" s="35" t="n"/>
-      <c r="C57" s="34" t="n"/>
-      <c r="D57" s="35" t="n"/>
-      <c r="E57" s="35" t="n"/>
-      <c r="F57" s="34" t="n"/>
+      <c r="F57" s="15" t="n"/>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>Contain: stop or narrow the agent</t>
+          <t>Triage: is this real</t>
         </is>
       </c>
       <c r="B58" s="35" t="n"/>
@@ -4330,7 +4330,7 @@
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>Review the run records</t>
+          <t>Contain: stop or narrow the agent</t>
         </is>
       </c>
       <c r="B59" s="35" t="n"/>
@@ -4342,7 +4342,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Review the run records</t>
         </is>
       </c>
       <c r="B60" s="35" t="n"/>
@@ -4354,7 +4354,7 @@
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>Tell the people affected</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="B61" s="35" t="n"/>
@@ -4366,7 +4366,7 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>Decide whether anybody outside has to be told, and start that clock</t>
+          <t>Tell the people affected</t>
         </is>
       </c>
       <c r="B62" s="35" t="n"/>
@@ -4378,7 +4378,7 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>Review after the incident</t>
+          <t>Decide whether anybody outside has to be told, and start that clock</t>
         </is>
       </c>
       <c r="B63" s="35" t="n"/>
@@ -4390,7 +4390,7 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="25" t="inlineStr">
         <is>
-          <t>Decide whether the agent resumes, and whether the sign-off still holds</t>
+          <t>Review after the incident</t>
         </is>
       </c>
       <c r="B64" s="35" t="n"/>
@@ -4399,130 +4399,126 @@
       <c r="E64" s="35" t="n"/>
       <c r="F64" s="34" t="n"/>
     </row>
-    <row r="65" ht="26" customHeight="1">
-      <c r="A65" s="13" t="inlineStr">
-        <is>
-          <t>For an agent inside a regulated process, notifying a regulator or a data-protection authority runs on a clock that starts well before the fix is finished. Stage 2 classifies agents on whether a mistake is reportable, so somebody has to decide here whether this one is.</t>
-        </is>
-      </c>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="25" t="inlineStr">
+        <is>
+          <t>Decide whether the agent resumes, and whether the sign-off still holds</t>
+        </is>
+      </c>
+      <c r="B65" s="35" t="n"/>
+      <c r="C65" s="34" t="n"/>
+      <c r="D65" s="35" t="n"/>
+      <c r="E65" s="35" t="n"/>
+      <c r="F65" s="34" t="n"/>
     </row>
     <row r="66" ht="26" customHeight="1">
       <c r="A66" s="13" t="inlineStr">
         <is>
+          <t>For an agent inside a regulated process, notifying a regulator or a data-protection authority runs on a clock that starts well before the fix is finished. Stage 2 classifies agents on whether a mistake is reportable, so somebody has to decide here whether this one is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="26" customHeight="1">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
           <t>The stage 3 sign-off is void once live behavior stops matching what it was granted against, and an incident is that moment. Name who re-confirms it, or re-issues it, before the agent runs again.</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="26" customHeight="1">
-      <c r="A67" s="32" t="n"/>
-      <c r="B67" s="32" t="n"/>
-      <c r="C67" s="32" t="n"/>
-      <c r="D67" s="32" t="n"/>
-      <c r="E67" s="32" t="n"/>
-      <c r="F67" s="32" t="n"/>
-    </row>
-    <row r="68" ht="56" customHeight="1">
-      <c r="A68" s="10" t="inlineStr">
+    <row r="68" ht="26" customHeight="1">
+      <c r="A68" s="32" t="n"/>
+      <c r="B68" s="32" t="n"/>
+      <c r="C68" s="32" t="n"/>
+      <c r="D68" s="32" t="n"/>
+      <c r="E68" s="32" t="n"/>
+      <c r="F68" s="32" t="n"/>
+    </row>
+    <row r="69" ht="56" customHeight="1">
+      <c r="A69" s="10" t="inlineStr">
         <is>
           <t>How the agent is stopped, and by whom</t>
         </is>
       </c>
-      <c r="B68" s="15" t="n"/>
-      <c r="C68" s="35" t="n"/>
-      <c r="D68" s="36" t="n"/>
-      <c r="E68" s="36" t="n"/>
-      <c r="F68" s="34" t="n"/>
-    </row>
-    <row r="69" ht="13" customHeight="1">
-      <c r="A69" s="13" t="inlineStr">
+      <c r="B69" s="15" t="n"/>
+      <c r="C69" s="35" t="n"/>
+      <c r="D69" s="36" t="n"/>
+      <c r="E69" s="36" t="n"/>
+      <c r="F69" s="34" t="n"/>
+    </row>
+    <row r="70" ht="13" customHeight="1">
+      <c r="A70" s="13" t="inlineStr">
         <is>
           <t>Point at section 5 of the design document rather than restating it. Say who is on call.</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="56" customHeight="1">
-      <c r="A70" s="10" t="inlineStr">
+    <row r="71" ht="56" customHeight="1">
+      <c r="A71" s="10" t="inlineStr">
         <is>
           <t>What you tell a customer, and who decides</t>
         </is>
       </c>
-      <c r="B70" s="15" t="n"/>
-      <c r="C70" s="35" t="n"/>
-      <c r="D70" s="36" t="n"/>
-      <c r="E70" s="36" t="n"/>
-      <c r="F70" s="34" t="n"/>
-    </row>
-    <row r="71" ht="13" customHeight="1">
-      <c r="A71" s="13" t="inlineStr">
+      <c r="B71" s="15" t="n"/>
+      <c r="C71" s="35" t="n"/>
+      <c r="D71" s="36" t="n"/>
+      <c r="E71" s="36" t="n"/>
+      <c r="F71" s="34" t="n"/>
+    </row>
+    <row r="72" ht="13" customHeight="1">
+      <c r="A72" s="13" t="inlineStr">
         <is>
           <t>For any agent where the person on the other end is not internal staff.</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="26" customHeight="1">
-      <c r="A72" s="32" t="n"/>
-      <c r="B72" s="32" t="n"/>
-      <c r="C72" s="32" t="n"/>
-      <c r="D72" s="32" t="n"/>
-      <c r="E72" s="32" t="n"/>
-      <c r="F72" s="32" t="n"/>
-    </row>
-    <row r="73" ht="22" customHeight="1">
-      <c r="A73" s="9" t="inlineStr">
-        <is>
-          <t>E.  The failure modes this playbook covers</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="38" customHeight="1">
-      <c r="A74" s="13" t="inlineStr">
+    <row r="73" ht="26" customHeight="1">
+      <c r="A73" s="32" t="n"/>
+      <c r="B73" s="32" t="n"/>
+      <c r="C73" s="32" t="n"/>
+      <c r="D73" s="32" t="n"/>
+      <c r="E73" s="32" t="n"/>
+      <c r="F73" s="32" t="n"/>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="9" t="inlineStr">
+        <is>
+          <t>E.  What goes wrong, and what you do about it</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="38" customHeight="1">
+      <c r="A75" s="13" t="inlineStr">
         <is>
           <t>Agents fail in ways ordinary software does not. Write what you would do, or write "not covered" and let the sign-off carry it. Where a row does not apply, write "the agent cannot do this" rather than leaving it blank. Drawn from the OWASP Top 10 for Agentic Applications; the OWASP column names the entry each row comes from.</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="30" customHeight="1">
-      <c r="A75" s="14" t="inlineStr">
-        <is>
-          <t>Failure mode</t>
-        </is>
-      </c>
-      <c r="B75" s="14" t="inlineStr">
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="14" t="inlineStr">
+        <is>
+          <t>What goes wrong</t>
+        </is>
+      </c>
+      <c r="B76" s="14" t="inlineStr">
         <is>
           <t>OWASP</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>What you do</t>
         </is>
       </c>
-    </row>
-    <row r="76" ht="30" customHeight="1">
-      <c r="A76" s="25" t="inlineStr">
-        <is>
-          <t>The agent calls a tool outside its declared set</t>
-        </is>
-      </c>
-      <c r="B76" s="25" t="inlineStr">
-        <is>
-          <t>ASI02, ASI03</t>
-        </is>
-      </c>
-      <c r="C76" s="32" t="n"/>
-      <c r="D76" s="32" t="n"/>
-      <c r="E76" s="32" t="n"/>
-      <c r="F76" s="32" t="n"/>
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="25" t="inlineStr">
         <is>
-          <t>A chain of tool calls each succeeds but the outcome is wrong</t>
+          <t>The agent calls a tool outside its declared set</t>
         </is>
       </c>
       <c r="B77" s="25" t="inlineStr">
         <is>
-          <t>ASI08</t>
+          <t>ASI02, ASI03</t>
         </is>
       </c>
       <c r="C77" s="32" t="n"/>
@@ -4533,12 +4529,12 @@
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="25" t="inlineStr">
         <is>
-          <t>Prompt injection through content the agent reads</t>
+          <t>A chain of tool calls each succeeds but the outcome is wrong</t>
         </is>
       </c>
       <c r="B78" s="25" t="inlineStr">
         <is>
-          <t>ASI01</t>
+          <t>ASI08</t>
         </is>
       </c>
       <c r="C78" s="32" t="n"/>
@@ -4549,12 +4545,12 @@
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="25" t="inlineStr">
         <is>
-          <t>Scope creep: used for work it was not designed for</t>
+          <t>Prompt injection through content the agent reads</t>
         </is>
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>ASI09</t>
+          <t>ASI01</t>
         </is>
       </c>
       <c r="C79" s="32" t="n"/>
@@ -4565,12 +4561,12 @@
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="25" t="inlineStr">
         <is>
-          <t>The agent loops, or runs away on cost</t>
+          <t>Scope creep: used for work it was not designed for</t>
         </is>
       </c>
       <c r="B80" s="25" t="inlineStr">
         <is>
-          <t>ASI08</t>
+          <t>ASI09</t>
         </is>
       </c>
       <c r="C80" s="32" t="n"/>
@@ -4581,12 +4577,12 @@
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="25" t="inlineStr">
         <is>
-          <t>A model or framework update changes behavior with no code change</t>
+          <t>The agent loops, or runs away on cost</t>
         </is>
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>ASI04</t>
+          <t>ASI08</t>
         </is>
       </c>
       <c r="C81" s="32" t="n"/>
@@ -4597,12 +4593,12 @@
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="25" t="inlineStr">
         <is>
-          <t>Memory or retrieved context has been poisoned</t>
+          <t>A model or framework update changes behavior with no code change</t>
         </is>
       </c>
       <c r="B82" s="25" t="inlineStr">
         <is>
-          <t>ASI06</t>
+          <t>ASI04</t>
         </is>
       </c>
       <c r="C82" s="32" t="n"/>
@@ -4613,12 +4609,12 @@
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="25" t="inlineStr">
         <is>
-          <t>The agent is confidently wrong and a person acts on it</t>
+          <t>Memory or retrieved context has been poisoned</t>
         </is>
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>ASI09</t>
+          <t>ASI06</t>
         </is>
       </c>
       <c r="C83" s="32" t="n"/>
@@ -4629,7 +4625,7 @@
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="25" t="inlineStr">
         <is>
-          <t>The agent stops escalating when it should</t>
+          <t>The agent is confidently wrong and a person acts on it</t>
         </is>
       </c>
       <c r="B84" s="25" t="inlineStr">
@@ -4645,12 +4641,12 @@
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="25" t="inlineStr">
         <is>
-          <t>The agent runs code or shell commands it composed itself</t>
+          <t>The agent stops escalating when it should</t>
         </is>
       </c>
       <c r="B85" s="25" t="inlineStr">
         <is>
-          <t>ASI05</t>
+          <t>ASI09</t>
         </is>
       </c>
       <c r="C85" s="32" t="n"/>
@@ -4661,12 +4657,12 @@
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="25" t="inlineStr">
         <is>
-          <t>A supervising agent fails, or supervises wrongly</t>
+          <t>The agent runs code or shell commands it composed itself</t>
         </is>
       </c>
       <c r="B86" s="25" t="inlineStr">
         <is>
-          <t>ASI07, ASI10</t>
+          <t>ASI05</t>
         </is>
       </c>
       <c r="C86" s="32" t="n"/>
@@ -4674,56 +4670,64 @@
       <c r="E86" s="32" t="n"/>
       <c r="F86" s="32" t="n"/>
     </row>
-    <row r="87" ht="26" customHeight="1">
-      <c r="A87" s="32" t="n"/>
-      <c r="B87" s="32" t="n"/>
+    <row r="87" ht="30" customHeight="1">
+      <c r="A87" s="25" t="inlineStr">
+        <is>
+          <t>A supervising agent fails, or supervises wrongly</t>
+        </is>
+      </c>
+      <c r="B87" s="25" t="inlineStr">
+        <is>
+          <t>ASI07, ASI10</t>
+        </is>
+      </c>
       <c r="C87" s="32" t="n"/>
       <c r="D87" s="32" t="n"/>
       <c r="E87" s="32" t="n"/>
       <c r="F87" s="32" t="n"/>
     </row>
-    <row r="88" ht="22" customHeight="1">
-      <c r="A88" s="9" t="inlineStr">
+    <row r="88" ht="26" customHeight="1">
+      <c r="A88" s="32" t="n"/>
+      <c r="B88" s="32" t="n"/>
+      <c r="C88" s="32" t="n"/>
+      <c r="D88" s="32" t="n"/>
+      <c r="E88" s="32" t="n"/>
+      <c r="F88" s="32" t="n"/>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="9" t="inlineStr">
         <is>
           <t>F.  Revision history</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="30" customHeight="1">
-      <c r="A89" s="14" t="inlineStr">
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B89" s="14" t="inlineStr">
+      <c r="B90" s="14" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="C89" s="14" t="inlineStr">
+      <c r="C90" s="14" t="inlineStr">
         <is>
           <t>What changed</t>
         </is>
       </c>
-      <c r="D89" s="14" t="inlineStr">
+      <c r="D90" s="14" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="E89" s="14" t="inlineStr">
+      <c r="E90" s="14" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="F89" s="15" t="n"/>
-    </row>
-    <row r="90" ht="30" customHeight="1">
-      <c r="A90" s="35" t="n"/>
-      <c r="B90" s="35" t="n"/>
-      <c r="C90" s="35" t="n"/>
-      <c r="D90" s="35" t="n"/>
-      <c r="E90" s="35" t="n"/>
-      <c r="F90" s="34" t="n"/>
+      <c r="F90" s="15" t="n"/>
     </row>
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="35" t="n"/>
@@ -4781,129 +4785,137 @@
       <c r="E97" s="35" t="n"/>
       <c r="F97" s="34" t="n"/>
     </row>
+    <row r="98" ht="30" customHeight="1">
+      <c r="A98" s="35" t="n"/>
+      <c r="B98" s="35" t="n"/>
+      <c r="C98" s="35" t="n"/>
+      <c r="D98" s="35" t="n"/>
+      <c r="E98" s="35" t="n"/>
+      <c r="F98" s="34" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="114">
-    <mergeCell ref="E62:F62"/>
-    <mergeCell ref="A66:F66"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C81:F81"/>
-    <mergeCell ref="A70:B70"/>
+    <mergeCell ref="E63:F63"/>
+    <mergeCell ref="A67:F67"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C82:F82"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="C38:F38"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="E65:F65"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="C79:F79"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="E64:F64"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C80:F80"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A74:F74"/>
+    <mergeCell ref="E92:F92"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="E94:F94"/>
+    <mergeCell ref="B64:C64"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="C28:F28"/>
     <mergeCell ref="C37:F37"/>
-    <mergeCell ref="A55:F55"/>
-    <mergeCell ref="E64:F64"/>
-    <mergeCell ref="C13:F13"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="C78:F78"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="E63:F63"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C79:F79"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="E49:F49"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A73:F73"/>
-    <mergeCell ref="E91:F91"/>
-    <mergeCell ref="B64:C64"/>
-    <mergeCell ref="A68:B68"/>
-    <mergeCell ref="E93:F93"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A42:F42"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="D17:F17"/>
-    <mergeCell ref="E48:F48"/>
-    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="C84:F84"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="E91:F91"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C41:F41"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A89:F89"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C77:F77"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="C8:F8"/>
     <mergeCell ref="C83:F83"/>
     <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A75:F75"/>
+    <mergeCell ref="E53:F53"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="E93:F93"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="A72:F72"/>
+    <mergeCell ref="C78:F78"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="E95:F95"/>
+    <mergeCell ref="C87:F87"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="C69:F69"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="E60:F60"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="E96:F96"/>
+    <mergeCell ref="A33:B33"/>
     <mergeCell ref="E90:F90"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C40:F40"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A88:F88"/>
-    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="E62:F62"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="C85:F85"/>
     <mergeCell ref="E58:F58"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="C76:F76"/>
-    <mergeCell ref="E50:F50"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C82:F82"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A74:F74"/>
-    <mergeCell ref="E52:F52"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="E92:F92"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="A71:F71"/>
-    <mergeCell ref="C77:F77"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="E94:F94"/>
-    <mergeCell ref="C86:F86"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="C68:F68"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="A53:F53"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="E95:F95"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="E89:F89"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A39:F39"/>
-    <mergeCell ref="C84:F84"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="C80:F80"/>
-    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C81:F81"/>
+    <mergeCell ref="C32:F32"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C12:F12"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="E56:F56"/>
-    <mergeCell ref="E96:F96"/>
-    <mergeCell ref="A65:F65"/>
-    <mergeCell ref="C70:F70"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="A41:B41"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="E97:F97"/>
+    <mergeCell ref="A66:F66"/>
+    <mergeCell ref="C71:F71"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B60:C60"/>
     <mergeCell ref="C7:F7"/>
-    <mergeCell ref="C38:F38"/>
-    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C39:F39"/>
+    <mergeCell ref="A26:B26"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E60:F60"/>
-    <mergeCell ref="A43:F43"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="C85:F85"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="C86:F86"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="D19:F19"/>
-    <mergeCell ref="C75:F75"/>
+    <mergeCell ref="C76:F76"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="E97:F97"/>
+    <mergeCell ref="E98:F98"/>
     <mergeCell ref="C11:F11"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A69:F69"/>
-    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A70:F70"/>
+    <mergeCell ref="E48:F48"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C10 C11 C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Level 1,Level 2,Level 3"</formula1>
     </dataValidation>
-    <dataValidation sqref="B17:B23 E45:E52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B17:B24 E46:E53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Partly"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5472,7 +5484,7 @@
     <row r="51" ht="26" customHeight="1">
       <c r="A51" s="13" t="inlineStr">
         <is>
-          <t>Running continuously shows the suite still works. It does not show the suite still covers the agent: new tools, new failure modes and new scope need new evals, and an unchanged eval set against a changed agent goes green for the wrong reason.</t>
+          <t>Running continuously shows the suite still works. It does not show the suite still covers the agent: new tools, new scope and new ways of going wrong need new evals, and an unchanged eval set against a changed agent goes green for the wrong reason.</t>
         </is>
       </c>
     </row>
@@ -6436,7 +6448,7 @@
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>Every tool call and its arguments logged. Inputs and outputs kept for a fixed period. Alerts on a few coarse signals.</t>
+          <t>Every tool call and its arguments logged. Inputs and outputs kept for a fixed period. Alerts on a few coarse signals. Enough for an agent whose classification asks for Level 1, and not for one that asks for more.</t>
         </is>
       </c>
     </row>
@@ -6449,7 +6461,7 @@
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>Run records stored: prompts, context, outputs. Alerts on drift from the design document, not only on errors.</t>
+          <t>Run records stored: prompts, context, outputs, and the steps in between. Alerts on drift from the design document, not only on errors.</t>
         </is>
       </c>
     </row>
@@ -6462,7 +6474,7 @@
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>A run can be replayed and tested against known failure modes.</t>
+          <t>A run can be replayed and tested against the ways the agent has gone wrong before.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record which version of each standard a record was judged against
The classification standard told people that when they revise the test,
agents classified under the old version can be found. Nothing made that
possible, because no record said which version it was judged against.
The same was true of both level ladders.

Adds a version field to section 6 of the design document, section A of
the Platform and Sign-off Record, and section A of the Monitoring
Record, in the markdown and the workbook. Updates the sentence in the
classification standard to point at the new field, and the note on the
classification sheet whose row reference moved.
</commit_message>
<xml_diff>
--- a/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
+++ b/deliverables/agent-governance-assurance-framework/artifacts/agent-governance-forms.xlsx
@@ -982,7 +982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1431,7 +1431,7 @@
     <row r="43" ht="26" customHeight="1">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>Write rows at a granularity your platform can enforce. "The CRM" is not a row. "Read contact records in region X, write only to the notes field" is a row. Tool-level scoping is portable; data-level scoping is not.</t>
+          <t>Write each row in your own words, at the finest level you would want enforced. "Read contact records, write only to the notes field" is a row. "The CRM" is not. Your platform’s names for these permissions get recorded later, when somebody creates them.</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
     <row r="71" ht="56" customHeight="1">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>Who is told when it fails</t>
+          <t>How the person on the other end challenges what it did</t>
         </is>
       </c>
       <c r="B71" s="15" t="n"/>
@@ -1722,79 +1722,81 @@
     <row r="72" ht="13" customHeight="1">
       <c r="A72" s="13" t="inlineStr">
         <is>
+          <t>For any agent whose audience is not internal staff. Who they raise it with, how a person looks at the decision again, and where that gets recorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="56" customHeight="1">
+      <c r="A73" s="10" t="inlineStr">
+        <is>
+          <t>Who is told when it fails</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="n"/>
+      <c r="C73" s="35" t="n"/>
+      <c r="D73" s="36" t="n"/>
+      <c r="E73" s="36" t="n"/>
+      <c r="F73" s="36" t="n"/>
+      <c r="G73" s="34" t="n"/>
+    </row>
+    <row r="74" ht="13" customHeight="1">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
           <t>The person, the channel, and the time within which they are told.</t>
         </is>
       </c>
     </row>
-    <row r="73" ht="26" customHeight="1">
-      <c r="A73" s="32" t="n"/>
-      <c r="B73" s="32" t="n"/>
-      <c r="C73" s="32" t="n"/>
-      <c r="D73" s="32" t="n"/>
-      <c r="E73" s="32" t="n"/>
-      <c r="F73" s="32" t="n"/>
-      <c r="G73" s="32" t="n"/>
-    </row>
-    <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="9" t="inlineStr">
+    <row r="75" ht="26" customHeight="1">
+      <c r="A75" s="32" t="n"/>
+      <c r="B75" s="32" t="n"/>
+      <c r="C75" s="32" t="n"/>
+      <c r="D75" s="32" t="n"/>
+      <c r="E75" s="32" t="n"/>
+      <c r="F75" s="32" t="n"/>
+      <c r="G75" s="32" t="n"/>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="9" t="inlineStr">
         <is>
           <t>6.  Classification and the Classification Test  →  see the Classification sheet</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="22" customHeight="1">
-      <c r="A75" s="9" t="inlineStr">
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="9" t="inlineStr">
         <is>
           <t>7.  Revision history</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="14" t="inlineStr">
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B76" s="14" t="inlineStr">
+      <c r="B78" s="14" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="C76" s="14" t="inlineStr">
+      <c r="C78" s="14" t="inlineStr">
         <is>
           <t>What changed</t>
         </is>
       </c>
-      <c r="D76" s="14" t="inlineStr">
+      <c r="D78" s="14" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="E76" s="14" t="inlineStr">
+      <c r="E78" s="14" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="F76" s="15" t="n"/>
-      <c r="G76" s="14" t="n"/>
-    </row>
-    <row r="77" ht="26" customHeight="1">
-      <c r="A77" s="35" t="n"/>
-      <c r="B77" s="35" t="n"/>
-      <c r="C77" s="35" t="n"/>
-      <c r="D77" s="35" t="n"/>
-      <c r="E77" s="35" t="n"/>
-      <c r="F77" s="34" t="n"/>
-      <c r="G77" s="35" t="n"/>
-    </row>
-    <row r="78" ht="26" customHeight="1">
-      <c r="A78" s="35" t="n"/>
-      <c r="B78" s="35" t="n"/>
-      <c r="C78" s="35" t="n"/>
-      <c r="D78" s="35" t="n"/>
-      <c r="E78" s="35" t="n"/>
-      <c r="F78" s="34" t="n"/>
-      <c r="G78" s="35" t="n"/>
+      <c r="F78" s="15" t="n"/>
+      <c r="G78" s="14" t="n"/>
     </row>
     <row r="79" ht="26" customHeight="1">
       <c r="A79" s="35" t="n"/>
@@ -1850,8 +1852,26 @@
       <c r="F84" s="34" t="n"/>
       <c r="G84" s="35" t="n"/>
     </row>
-    <row r="85" ht="39" customHeight="1">
-      <c r="A85" s="13" t="inlineStr">
+    <row r="85" ht="26" customHeight="1">
+      <c r="A85" s="35" t="n"/>
+      <c r="B85" s="35" t="n"/>
+      <c r="C85" s="35" t="n"/>
+      <c r="D85" s="35" t="n"/>
+      <c r="E85" s="35" t="n"/>
+      <c r="F85" s="34" t="n"/>
+      <c r="G85" s="35" t="n"/>
+    </row>
+    <row r="86" ht="26" customHeight="1">
+      <c r="A86" s="35" t="n"/>
+      <c r="B86" s="35" t="n"/>
+      <c r="C86" s="35" t="n"/>
+      <c r="D86" s="35" t="n"/>
+      <c r="E86" s="35" t="n"/>
+      <c r="F86" s="34" t="n"/>
+      <c r="G86" s="35" t="n"/>
+    </row>
+    <row r="87" ht="39" customHeight="1">
+      <c r="A87" s="13" t="inlineStr">
         <is>
           <t>One more tool, a widened scope, or a new audience all produce a row. So do stage 4 and stage 5 findings: an eval that catches drift, an audit finding against your classification criteria, or a monitor reporting a tool call outside section 3. A new model version does not; that changes the Platform and Sign-off Record instead. Retiring the agent produces the last row: set Status above to retired, date it, and fill in section E of the Audit &amp; Assurance sheet.</t>
         </is>
@@ -1859,22 +1879,25 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="100">
+  <mergeCells count="103">
     <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A73:B73"/>
     <mergeCell ref="C58:G58"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="C45:G45"/>
+    <mergeCell ref="A68:G68"/>
     <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A68:G68"/>
     <mergeCell ref="E79:F79"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="C65:G65"/>
     <mergeCell ref="C44:G44"/>
     <mergeCell ref="C60:G60"/>
+    <mergeCell ref="A87:G87"/>
     <mergeCell ref="C71:G71"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A62:B62"/>
     <mergeCell ref="C7:G7"/>
+    <mergeCell ref="E85:F85"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="C57:G57"/>
@@ -1888,6 +1911,7 @@
     <mergeCell ref="A45:B45"/>
     <mergeCell ref="A10:G10"/>
     <mergeCell ref="C20:G20"/>
+    <mergeCell ref="A77:G77"/>
     <mergeCell ref="A46:B46"/>
     <mergeCell ref="F42:G42"/>
     <mergeCell ref="C22:G22"/>
@@ -1900,26 +1924,24 @@
     <mergeCell ref="A71:B71"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C48:G48"/>
-    <mergeCell ref="A75:G75"/>
     <mergeCell ref="F39:G39"/>
-    <mergeCell ref="E76:F76"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="E83:F83"/>
     <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A69:B69"/>
     <mergeCell ref="C26:G26"/>
-    <mergeCell ref="A69:B69"/>
     <mergeCell ref="A65:B65"/>
     <mergeCell ref="C16:G16"/>
+    <mergeCell ref="C55:G55"/>
     <mergeCell ref="F36:G36"/>
-    <mergeCell ref="C55:G55"/>
     <mergeCell ref="E84:F84"/>
     <mergeCell ref="E78:F78"/>
     <mergeCell ref="C9:G9"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="E77:F77"/>
+    <mergeCell ref="E86:F86"/>
     <mergeCell ref="E80:F80"/>
+    <mergeCell ref="C11:G11"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C11:G11"/>
     <mergeCell ref="A25:G25"/>
     <mergeCell ref="C52:G52"/>
     <mergeCell ref="A66:G66"/>
@@ -1938,11 +1960,12 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="E82:F82"/>
     <mergeCell ref="A13:G13"/>
+    <mergeCell ref="C73:G73"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="C54:G54"/>
+    <mergeCell ref="A15:G15"/>
     <mergeCell ref="A64:G64"/>
-    <mergeCell ref="A15:G15"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="F41:G41"/>
     <mergeCell ref="A51:G51"/>
@@ -1952,14 +1975,14 @@
     <mergeCell ref="A70:G70"/>
     <mergeCell ref="F38:G38"/>
     <mergeCell ref="C8:G8"/>
+    <mergeCell ref="F37:G37"/>
     <mergeCell ref="A20:B20"/>
-    <mergeCell ref="F37:G37"/>
     <mergeCell ref="A74:G74"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A44:B44"/>
     <mergeCell ref="C53:G53"/>
+    <mergeCell ref="A76:G76"/>
     <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A85:G85"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation sqref="C35:C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1994,7 +2017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2051,78 +2074,76 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="32" t="n"/>
-      <c r="B6" s="32" t="n"/>
-      <c r="C6" s="32" t="n"/>
-      <c r="D6" s="32" t="n"/>
-      <c r="E6" s="32" t="n"/>
-      <c r="F6" s="32" t="n"/>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Version of the Risk Classifications this agent was classified against</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n"/>
+      <c r="C6" s="35" t="n"/>
+      <c r="D6" s="36" t="n"/>
+      <c r="E6" s="36" t="n"/>
+      <c r="F6" s="34" t="n"/>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="32" t="n"/>
+      <c r="B7" s="32" t="n"/>
+      <c r="C7" s="32" t="n"/>
+      <c r="D7" s="32" t="n"/>
+      <c r="E7" s="32" t="n"/>
+      <c r="F7" s="32" t="n"/>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Every question sets a floor: the lowest classification this agent can be in given that answer alone. The anchors that say what an answer has to reach to set each floor are on the Floor Anchors sheet — read them before you fill in the Floor column. The classifications themselves are on the Reference sheet. If you keep your own classifications, use those names instead and rewrite the Floor Anchors sheet with them. Do not use an autonomy scale.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="32" t="n"/>
-      <c r="B8" s="32" t="n"/>
-      <c r="C8" s="32" t="n"/>
-      <c r="D8" s="32" t="n"/>
-      <c r="E8" s="32" t="n"/>
-      <c r="F8" s="32" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="32" t="n"/>
+      <c r="B9" s="32" t="n"/>
+      <c r="C9" s="32" t="n"/>
+      <c r="D9" s="32" t="n"/>
+      <c r="E9" s="32" t="n"/>
+      <c r="F9" s="32" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Question</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Your answer</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Where the evidence is</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>Floor this answer sets</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n"/>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="18" t="inlineStr">
-        <is>
-          <t>How critical is the process it automates? If the agent stopped for a day, what stops with it?</t>
-        </is>
-      </c>
-      <c r="C10" s="35" t="n"/>
-      <c r="D10" s="35" t="n"/>
-      <c r="E10" s="35" t="n"/>
-      <c r="F10" s="34" t="n"/>
+      <c r="F10" s="15" t="n"/>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>How sensitive is the data it can read? Name the most sensitive item, not the average.</t>
+          <t>How critical is the process it automates? If the agent stopped for a day, what stops with it?</t>
         </is>
       </c>
       <c r="C11" s="35" t="n"/>
@@ -2132,11 +2153,11 @@
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>Which regulations reach this process? Name them, or write "none that we have identified" and say who looked.</t>
+          <t>How sensitive is the data it can read? Name the most sensitive item, not the average.</t>
         </is>
       </c>
       <c r="C12" s="35" t="n"/>
@@ -2146,11 +2167,11 @@
     </row>
     <row r="13" ht="36" customHeight="1">
       <c r="A13" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>How much money or value can it move, in one action and in one day?</t>
+          <t>Which regulations reach this process? Name them, or write "none that we have identified" and say who looked.</t>
         </is>
       </c>
       <c r="C13" s="35" t="n"/>
@@ -2160,11 +2181,11 @@
     </row>
     <row r="14" ht="36" customHeight="1">
       <c r="A14" s="17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Can you undo what it does? Name the action that is hardest to undo, and how long you have.</t>
+          <t>How much money or value can it move, in one action and in one day?</t>
         </is>
       </c>
       <c r="C14" s="35" t="n"/>
@@ -2174,11 +2195,11 @@
     </row>
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>How far does the damage spread beyond the system it acted on?</t>
+          <t>Can you undo what it does? Name the action that is hardest to undo, and how long you have.</t>
         </is>
       </c>
       <c r="C15" s="35" t="n"/>
@@ -2188,11 +2209,11 @@
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>What can it do with no person in the loop at all?</t>
+          <t>How far does the damage spread beyond the system it acted on?</t>
         </is>
       </c>
       <c r="C16" s="35" t="n"/>
@@ -2202,11 +2223,11 @@
     </row>
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>Who is on the other end: internal staff, your customers, or the public?</t>
+          <t>What can it do with no person in the loop at all?</t>
         </is>
       </c>
       <c r="C17" s="35" t="n"/>
@@ -2214,135 +2235,149 @@
       <c r="E17" s="35" t="n"/>
       <c r="F17" s="34" t="n"/>
     </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="32" t="n"/>
-      <c r="B18" s="32" t="n"/>
-      <c r="C18" s="32" t="n"/>
-      <c r="D18" s="32" t="n"/>
-      <c r="E18" s="32" t="n"/>
-      <c r="F18" s="32" t="n"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>Who is on the other end: internal staff, your customers, or the public?</t>
+        </is>
+      </c>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="35" t="n"/>
+      <c r="E18" s="35" t="n"/>
+      <c r="F18" s="34" t="n"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
       <c r="A19" s="32" t="n"/>
-      <c r="B19" s="19" t="inlineStr">
+      <c r="B19" s="32" t="n"/>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="32" t="n"/>
+      <c r="E19" s="32" t="n"/>
+      <c r="F19" s="32" t="n"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="32" t="n"/>
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Highest floor set by any single question above:</t>
         </is>
       </c>
-      <c r="E19" s="20">
-        <f>IF(COUNTA(E10:E17)&lt;8,"Answer all eight questions",IF(COUNTIF(E10:E17,"Critical")&gt;0,"Critical",IF(COUNTIF(E10:E17,"Sensitive")&gt;0,"Sensitive",IF(COUNTIF(E10:E17,"Significant")&gt;0,"Significant","Routine"))))</f>
+      <c r="E20" s="20">
+        <f>IF(COUNTA(E11:E18)&lt;8,"Answer all eight questions",IF(COUNTIF(E11:E18,"Critical")&gt;0,"Critical",IF(COUNTIF(E11:E18,"Sensitive")&gt;0,"Sensitive",IF(COUNTIF(E11:E18,"Significant")&gt;0,"Significant","Routine"))))</f>
         <v/>
       </c>
-      <c r="F19" s="15" t="n"/>
-    </row>
-    <row r="20" ht="54" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="F20" s="15" t="n"/>
+    </row>
+    <row r="21" ht="54" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>THE RULE</t>
         </is>
       </c>
-      <c r="B20" s="15" t="n"/>
-      <c r="C20" s="21" t="inlineStr">
-        <is>
-          <t>The classification is the highest floor that any single question sets. One critical answer makes the agent critical, however routine the other seven are. The cell in row 19 calculates it from the eight floors. It reads the four starter names, so if you keep your own classifications, replace the formula with your own order of severity.</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="n"/>
-      <c r="E20" s="16" t="n"/>
-      <c r="F20" s="15" t="n"/>
-    </row>
-    <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="32" t="n"/>
-      <c r="B21" s="32" t="n"/>
-      <c r="C21" s="32" t="n"/>
-      <c r="D21" s="32" t="n"/>
-      <c r="E21" s="32" t="n"/>
-      <c r="F21" s="32" t="n"/>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="21" t="inlineStr">
+        <is>
+          <t>The classification is the highest floor that any single question sets. One critical answer makes the agent critical, however routine the other seven are. The cell in row 20 calculates it from the eight floors. It reads the four starter names, so if you keep your own classifications, replace the formula with your own order of severity.</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="n"/>
+      <c r="E21" s="16" t="n"/>
+      <c r="F21" s="15" t="n"/>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="32" t="n"/>
+      <c r="B22" s="32" t="n"/>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="32" t="n"/>
+      <c r="E22" s="32" t="n"/>
+      <c r="F22" s="32" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>If you are placing this agent lower than its highest floor</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="56" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
+    <row r="24" ht="56" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Name the control that lowers it</t>
         </is>
       </c>
-      <c r="B23" s="15" t="n"/>
-      <c r="C23" s="35" t="n"/>
-      <c r="D23" s="36" t="n"/>
-      <c r="E23" s="36" t="n"/>
-      <c r="F23" s="34" t="n"/>
-    </row>
-    <row r="24" ht="13" customHeight="1">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="B24" s="15" t="n"/>
+      <c r="C24" s="35" t="n"/>
+      <c r="D24" s="36" t="n"/>
+      <c r="E24" s="36" t="n"/>
+      <c r="F24" s="34" t="n"/>
+    </row>
+    <row r="25" ht="13" customHeight="1">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>Where it is enforced, and who confirmed it holds. A control that exists in a plan does not lower a floor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="22" t="inlineStr">
-        <is>
-          <t>1.  Questions 5 and 6 cannot be lowered. A control can stop the agent reaching them, but it cannot make the consequence smaller.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="22" t="inlineStr">
         <is>
-          <t>2.  A control enforced only in the prompt cannot lower a floor. If section 4 says "in the prompt", the floor stands.</t>
+          <t>1.  Questions 5 and 6 cannot be lowered. A control can stop the agent reaching them, but it cannot make the consequence smaller.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="22" t="inlineStr">
         <is>
+          <t>2.  A control enforced only in the prompt cannot lower a floor. If section 4 says "in the prompt", the floor stands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
           <t>3.  A lowered floor must also be named in the sign-off, on the Platform &amp; Sign-off sheet, by the person accepting it.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="32" t="n"/>
-      <c r="B28" s="32" t="n"/>
-      <c r="C28" s="32" t="n"/>
-      <c r="D28" s="32" t="n"/>
-      <c r="E28" s="32" t="n"/>
-      <c r="F28" s="32" t="n"/>
-    </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="23" t="inlineStr">
+    <row r="29" ht="26" customHeight="1">
+      <c r="A29" s="32" t="n"/>
+      <c r="B29" s="32" t="n"/>
+      <c r="C29" s="32" t="n"/>
+      <c r="D29" s="32" t="n"/>
+      <c r="E29" s="32" t="n"/>
+      <c r="F29" s="32" t="n"/>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="23" t="inlineStr">
         <is>
           <t>A blank row is not a low answer. An unanswered question means the classification is not established, and the agent is not ready for sign-off.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="32" t="n"/>
-      <c r="B30" s="32" t="n"/>
-      <c r="C30" s="32" t="n"/>
-      <c r="D30" s="32" t="n"/>
-      <c r="E30" s="32" t="n"/>
-      <c r="F30" s="32" t="n"/>
-    </row>
-    <row r="31" ht="56" customHeight="1">
-      <c r="A31" s="10" t="inlineStr">
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="32" t="n"/>
+      <c r="B31" s="32" t="n"/>
+      <c r="C31" s="32" t="n"/>
+      <c r="D31" s="32" t="n"/>
+      <c r="E31" s="32" t="n"/>
+      <c r="F31" s="32" t="n"/>
+    </row>
+    <row r="32" ht="56" customHeight="1">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>What would change this classification?</t>
         </is>
       </c>
-      <c r="B31" s="15" t="n"/>
-      <c r="C31" s="35" t="n"/>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="36" t="n"/>
-      <c r="F31" s="34" t="n"/>
-    </row>
-    <row r="32" ht="13" customHeight="1">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="35" t="n"/>
+      <c r="D32" s="36" t="n"/>
+      <c r="E32" s="36" t="n"/>
+      <c r="F32" s="34" t="n"/>
+    </row>
+    <row r="33" ht="13" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>The change to the agent, its tools, its data, or its model that would make you run this test again.</t>
         </is>
@@ -2350,39 +2385,41 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="29">
+  <mergeCells count="31">
     <mergeCell ref="E12:F12"/>
-    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="E14:F14"/>
+    <mergeCell ref="C32:F32"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="E17:F17"/>
-    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="E20:F20"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="A5:F5"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="C6:F6"/>
     <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A28:F28"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="C4:F4"/>
-    <mergeCell ref="C20:F20"/>
     <mergeCell ref="E11:F11"/>
-    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A30:F30"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="C31:F31"/>
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="E18:F18"/>
     <mergeCell ref="A25:F25"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C4 E10:E17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4 E11:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Routine,Significant,Sensitive,Critical"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2765,7 +2802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2979,7 +3016,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>When this agent's access is reviewed again, and by whom</t>
+          <t>Version of the Platform Control Levels this score was made against</t>
         </is>
       </c>
       <c r="B20" s="15" t="n"/>
@@ -2988,171 +3025,173 @@
       <c r="E20" s="36" t="n"/>
       <c r="F20" s="34" t="n"/>
     </row>
-    <row r="21" ht="13" customHeight="1">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>When this agent's access is reviewed again, and by whom</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="n"/>
+      <c r="C21" s="35" t="n"/>
+      <c r="D21" s="36" t="n"/>
+      <c r="E21" s="36" t="n"/>
+      <c r="F21" s="34" t="n"/>
+    </row>
+    <row r="22" ht="13" customHeight="1">
+      <c r="A22" s="13" t="inlineStr">
         <is>
           <t>Permissions are granted once and then survive every later change to what the agent does.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Autonomy level, on the four-level scale in the CSA agentic profile, or your own if you keep one</t>
         </is>
       </c>
-      <c r="B22" s="15" t="n"/>
-      <c r="C22" s="35" t="n"/>
-      <c r="D22" s="36" t="n"/>
-      <c r="E22" s="36" t="n"/>
-      <c r="F22" s="34" t="n"/>
-    </row>
-    <row r="23" ht="13" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="35" t="n"/>
+      <c r="D23" s="36" t="n"/>
+      <c r="E23" s="36" t="n"/>
+      <c r="F23" s="34" t="n"/>
+    </row>
+    <row r="24" ht="13" customHeight="1">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>Recorded here, never as the classification.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Tool servers and connectors it reaches, and who publishes each one</t>
         </is>
       </c>
-      <c r="B24" s="15" t="n"/>
-      <c r="C24" s="35" t="n"/>
-      <c r="D24" s="36" t="n"/>
-      <c r="E24" s="36" t="n"/>
-      <c r="F24" s="34" t="n"/>
-    </row>
-    <row r="25" ht="13" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="B25" s="15" t="n"/>
+      <c r="C25" s="35" t="n"/>
+      <c r="D25" s="36" t="n"/>
+      <c r="E25" s="36" t="n"/>
+      <c r="F25" s="34" t="n"/>
+    </row>
+    <row r="26" ht="13" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>An MCP server or a shared connector is a dependency the agent inherits, published by somebody who can change it without telling you.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="26" customHeight="1">
-      <c r="A26" s="32" t="n"/>
-      <c r="B26" s="32" t="n"/>
-      <c r="C26" s="32" t="n"/>
-      <c r="D26" s="32" t="n"/>
-      <c r="E26" s="32" t="n"/>
-      <c r="F26" s="32" t="n"/>
-    </row>
-    <row r="27" ht="56" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
+    <row r="27" ht="26" customHeight="1">
+      <c r="A27" s="32" t="n"/>
+      <c r="B27" s="32" t="n"/>
+      <c r="C27" s="32" t="n"/>
+      <c r="D27" s="32" t="n"/>
+      <c r="E27" s="32" t="n"/>
+      <c r="F27" s="32" t="n"/>
+    </row>
+    <row r="28" ht="56" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Where the grant list is enforced</t>
         </is>
       </c>
-      <c r="B27" s="15" t="n"/>
-      <c r="C27" s="35" t="n"/>
-      <c r="D27" s="36" t="n"/>
-      <c r="E27" s="36" t="n"/>
-      <c r="F27" s="34" t="n"/>
-    </row>
-    <row r="28" ht="13" customHeight="1">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="B28" s="15" t="n"/>
+      <c r="C28" s="35" t="n"/>
+      <c r="D28" s="36" t="n"/>
+      <c r="E28" s="36" t="n"/>
+      <c r="F28" s="34" t="n"/>
+    </row>
+    <row r="29" ht="13" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>Section 3 of the design document lists the tools and the data. Name the component that enforces it: a gateway, a policy engine, scoped credentials, or a tool wrapper.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="56" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>What is granted that the design document does not list</t>
-        </is>
-      </c>
-      <c r="B29" s="15" t="n"/>
-      <c r="C29" s="35" t="n"/>
-      <c r="D29" s="36" t="n"/>
-      <c r="E29" s="36" t="n"/>
-      <c r="F29" s="34" t="n"/>
-    </row>
-    <row r="30" ht="27" customHeight="1">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>Anything the agent can reach that section 3 does not name. This should be empty. Where it is not, carry it into section C as remaining risk. Do not fix it quietly and leave this blank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="26" customHeight="1">
-      <c r="A31" s="32" t="n"/>
-      <c r="B31" s="32" t="n"/>
-      <c r="C31" s="32" t="n"/>
-      <c r="D31" s="32" t="n"/>
-      <c r="E31" s="32" t="n"/>
-      <c r="F31" s="32" t="n"/>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>B.  What the evals found   (against the setup in section A, not a development configuration)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>Which evals you ran</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n"/>
-      <c r="C33" s="35" t="n"/>
-      <c r="D33" s="36" t="n"/>
-      <c r="E33" s="36" t="n"/>
-      <c r="F33" s="34" t="n"/>
-    </row>
-    <row r="34" ht="56" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>Adversarial testing performed, and what it was tested against</t>
-        </is>
-      </c>
-      <c r="B34" s="15" t="n"/>
-      <c r="C34" s="35" t="n"/>
-      <c r="D34" s="36" t="n"/>
+    <row r="30" ht="26" customHeight="1">
+      <c r="A30" s="32" t="n"/>
+      <c r="B30" s="32" t="n"/>
+      <c r="C30" s="32" t="n"/>
+      <c r="D30" s="32" t="n"/>
+      <c r="E30" s="32" t="n"/>
+      <c r="F30" s="32" t="n"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>What was actually granted, row by row</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="n"/>
+      <c r="C31" s="16" t="n"/>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="16" t="n"/>
+      <c r="F31" s="15" t="n"/>
+    </row>
+    <row r="32" ht="13" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Take each row of section 3 and write the permission that was really created for it, using the exact name your platform uses. This is the list your monitor compares live tool calls against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>Row in section 3</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>The permission actually granted, as the platform names it</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>Wider, narrower, or the same</t>
+        </is>
+      </c>
+      <c r="E33" s="16" t="n"/>
+      <c r="F33" s="15" t="n"/>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="35" t="n"/>
+      <c r="B34" s="35" t="n"/>
+      <c r="C34" s="34" t="n"/>
+      <c r="D34" s="35" t="n"/>
       <c r="E34" s="36" t="n"/>
       <c r="F34" s="34" t="n"/>
     </row>
     <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="13" t="inlineStr">
-        <is>
-          <t>For any agent that reads content it did not author, whether it can be talked into something is what the sign-off most needs to know. Name what you tested against from OWASP's Top 10 for Agentic Applications, the same list the Monitoring sheet's playbook works from.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>Against which configuration, matching section A</t>
-        </is>
-      </c>
-      <c r="B36" s="15" t="n"/>
-      <c r="C36" s="35" t="n"/>
-      <c r="D36" s="36" t="n"/>
+      <c r="A35" s="35" t="n"/>
+      <c r="B35" s="35" t="n"/>
+      <c r="C35" s="34" t="n"/>
+      <c r="D35" s="35" t="n"/>
+      <c r="E35" s="36" t="n"/>
+      <c r="F35" s="34" t="n"/>
+    </row>
+    <row r="36" ht="26" customHeight="1">
+      <c r="A36" s="35" t="n"/>
+      <c r="B36" s="35" t="n"/>
+      <c r="C36" s="34" t="n"/>
+      <c r="D36" s="35" t="n"/>
       <c r="E36" s="36" t="n"/>
       <c r="F36" s="34" t="n"/>
     </row>
-    <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>Date of the run</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="n"/>
-      <c r="C37" s="35" t="n"/>
-      <c r="D37" s="36" t="n"/>
-      <c r="E37" s="36" t="n"/>
-      <c r="F37" s="34" t="n"/>
+    <row r="37" ht="26" customHeight="1">
+      <c r="A37" s="32" t="n"/>
+      <c r="B37" s="32" t="n"/>
+      <c r="C37" s="32" t="n"/>
+      <c r="D37" s="32" t="n"/>
+      <c r="E37" s="32" t="n"/>
+      <c r="F37" s="32" t="n"/>
     </row>
     <row r="38" ht="56" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>What they found</t>
+          <t>Anything narrower than the design document asks for</t>
         </is>
       </c>
       <c r="B38" s="15" t="n"/>
@@ -3164,14 +3203,14 @@
     <row r="39" ht="13" customHeight="1">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>This is what the person signing off is accepting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
+          <t>Say what the agent cannot do as a result, and whether anybody has worked around it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="56" customHeight="1">
       <c r="A40" s="10" t="inlineStr">
         <is>
-          <t>What you changed because of it</t>
+          <t>What is granted that the design document does not list</t>
         </is>
       </c>
       <c r="B40" s="15" t="n"/>
@@ -3180,68 +3219,63 @@
       <c r="E40" s="36" t="n"/>
       <c r="F40" s="34" t="n"/>
     </row>
-    <row r="41" ht="56" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>What you know you did NOT test</t>
-        </is>
-      </c>
-      <c r="B41" s="15" t="n"/>
-      <c r="C41" s="35" t="n"/>
-      <c r="D41" s="36" t="n"/>
-      <c r="E41" s="36" t="n"/>
-      <c r="F41" s="34" t="n"/>
-    </row>
-    <row r="42" ht="13" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t>This is where stage 4 monitoring has to begin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="10" t="inlineStr">
-        <is>
-          <t>Where the results are kept</t>
-        </is>
-      </c>
-      <c r="B43" s="15" t="n"/>
-      <c r="C43" s="35" t="n"/>
-      <c r="D43" s="36" t="n"/>
-      <c r="E43" s="36" t="n"/>
-      <c r="F43" s="34" t="n"/>
-    </row>
-    <row r="44" ht="26" customHeight="1">
-      <c r="A44" s="32" t="n"/>
-      <c r="B44" s="32" t="n"/>
-      <c r="C44" s="32" t="n"/>
-      <c r="D44" s="32" t="n"/>
-      <c r="E44" s="32" t="n"/>
-      <c r="F44" s="32" t="n"/>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="9" t="inlineStr">
-        <is>
-          <t>C.  Sign-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="10" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B46" s="15" t="n"/>
-      <c r="C46" s="35" t="n"/>
-      <c r="D46" s="36" t="n"/>
-      <c r="E46" s="36" t="n"/>
-      <c r="F46" s="34" t="n"/>
+    <row r="41" ht="27" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>Anything the agent can reach that section 3 does not name. This should be empty. Where it is not, carry it into section C as remaining risk. Do not fix it quietly and leave this blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="26" customHeight="1">
+      <c r="A42" s="32" t="n"/>
+      <c r="B42" s="32" t="n"/>
+      <c r="C42" s="32" t="n"/>
+      <c r="D42" s="32" t="n"/>
+      <c r="E42" s="32" t="n"/>
+      <c r="F42" s="32" t="n"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>B.  What the evals found   (against the setup in section A, not a development configuration)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>Which evals you ran</t>
+        </is>
+      </c>
+      <c r="B44" s="15" t="n"/>
+      <c r="C44" s="35" t="n"/>
+      <c r="D44" s="36" t="n"/>
+      <c r="E44" s="36" t="n"/>
+      <c r="F44" s="34" t="n"/>
+    </row>
+    <row r="45" ht="56" customHeight="1">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>Adversarial testing performed, and what it was tested against</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="n"/>
+      <c r="C45" s="35" t="n"/>
+      <c r="D45" s="36" t="n"/>
+      <c r="E45" s="36" t="n"/>
+      <c r="F45" s="34" t="n"/>
+    </row>
+    <row r="46" ht="26" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>For any agent that reads content it did not author, whether it can be talked into something is what the sign-off most needs to know. Name what you tested against from OWASP's Top 10 for Agentic Applications, the same list the Monitoring sheet's playbook works from.</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="10" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Against which configuration, matching section A</t>
         </is>
       </c>
       <c r="B47" s="15" t="n"/>
@@ -3253,7 +3287,7 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Date of the run</t>
         </is>
       </c>
       <c r="B48" s="15" t="n"/>
@@ -3262,10 +3296,10 @@
       <c r="E48" s="36" t="n"/>
       <c r="F48" s="34" t="n"/>
     </row>
-    <row r="49" ht="30" customHeight="1">
+    <row r="49" ht="56" customHeight="1">
       <c r="A49" s="10" t="inlineStr">
         <is>
-          <t>Version of the design document signed</t>
+          <t>What they found</t>
         </is>
       </c>
       <c r="B49" s="15" t="n"/>
@@ -3274,22 +3308,17 @@
       <c r="E49" s="36" t="n"/>
       <c r="F49" s="34" t="n"/>
     </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="10" t="inlineStr">
-        <is>
-          <t>Version of this record signed</t>
-        </is>
-      </c>
-      <c r="B50" s="15" t="n"/>
-      <c r="C50" s="35" t="n"/>
-      <c r="D50" s="36" t="n"/>
-      <c r="E50" s="36" t="n"/>
-      <c r="F50" s="34" t="n"/>
-    </row>
-    <row r="51" ht="56" customHeight="1">
+    <row r="50" ht="13" customHeight="1">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>This is what the person signing off is accepting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
-          <t>The risk that is left, stated in their words</t>
+          <t>What you changed because of it</t>
         </is>
       </c>
       <c r="B51" s="15" t="n"/>
@@ -3298,10 +3327,10 @@
       <c r="E51" s="36" t="n"/>
       <c r="F51" s="34" t="n"/>
     </row>
-    <row r="52" ht="30" customHeight="1">
+    <row r="52" ht="56" customHeight="1">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>Any classification floor lowered by a compensating control</t>
+          <t>What you know you did NOT test</t>
         </is>
       </c>
       <c r="B52" s="15" t="n"/>
@@ -3313,14 +3342,14 @@
     <row r="53" ht="13" customHeight="1">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>A floor lowered in the design document and not repeated here has not been accepted by anybody.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="56" customHeight="1">
+          <t>This is where stage 4 monitoring has to begin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>Conditions on the sign-off, and when it must be looked at again</t>
+          <t>Where the results are kept</t>
         </is>
       </c>
       <c r="B54" s="15" t="n"/>
@@ -3329,29 +3358,25 @@
       <c r="E54" s="36" t="n"/>
       <c r="F54" s="34" t="n"/>
     </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="24" t="inlineStr">
-        <is>
-          <t>THE LEVEL GAP.  The agent's classification names a platform control level and a monitoring level that an agent in it requires. Where the level applied is lower, the gap is accepted here, by name, or it is not accepted at all.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="10" t="inlineStr">
-        <is>
-          <t>Platform control level the classification requires, and the level applied</t>
-        </is>
-      </c>
-      <c r="B56" s="15" t="n"/>
-      <c r="C56" s="35" t="n"/>
-      <c r="D56" s="36" t="n"/>
-      <c r="E56" s="36" t="n"/>
-      <c r="F56" s="34" t="n"/>
+    <row r="55" ht="26" customHeight="1">
+      <c r="A55" s="32" t="n"/>
+      <c r="B55" s="32" t="n"/>
+      <c r="C55" s="32" t="n"/>
+      <c r="D55" s="32" t="n"/>
+      <c r="E55" s="32" t="n"/>
+      <c r="F55" s="32" t="n"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="9" t="inlineStr">
+        <is>
+          <t>C.  Sign-off</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>Monitoring level the classification requires, and the level applied</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B57" s="15" t="n"/>
@@ -3363,7 +3388,7 @@
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Who accepts the gap, by name</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="B58" s="15" t="n"/>
@@ -3375,7 +3400,7 @@
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>The date by which it closes</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B59" s="15" t="n"/>
@@ -3387,7 +3412,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="10" t="inlineStr">
         <is>
-          <t>How many consecutive sign-offs have accepted this same gap</t>
+          <t>Version of the design document signed</t>
         </is>
       </c>
       <c r="B60" s="15" t="n"/>
@@ -3396,157 +3421,279 @@
       <c r="E60" s="36" t="n"/>
       <c r="F60" s="34" t="n"/>
     </row>
-    <row r="61" ht="26" customHeight="1">
-      <c r="A61" s="13" t="inlineStr">
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="10" t="inlineStr">
+        <is>
+          <t>Version of this record signed</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="n"/>
+      <c r="C61" s="35" t="n"/>
+      <c r="D61" s="36" t="n"/>
+      <c r="E61" s="36" t="n"/>
+      <c r="F61" s="34" t="n"/>
+    </row>
+    <row r="62" ht="56" customHeight="1">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>The risk that is left, stated in their words</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="n"/>
+      <c r="C62" s="35" t="n"/>
+      <c r="D62" s="36" t="n"/>
+      <c r="E62" s="36" t="n"/>
+      <c r="F62" s="34" t="n"/>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="10" t="inlineStr">
+        <is>
+          <t>Any classification floor lowered by a compensating control</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="n"/>
+      <c r="C63" s="35" t="n"/>
+      <c r="D63" s="36" t="n"/>
+      <c r="E63" s="36" t="n"/>
+      <c r="F63" s="34" t="n"/>
+    </row>
+    <row r="64" ht="13" customHeight="1">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>A floor lowered in the design document and not repeated here has not been accepted by anybody.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="56" customHeight="1">
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>Conditions on the sign-off, and when it must be looked at again</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="n"/>
+      <c r="C65" s="35" t="n"/>
+      <c r="D65" s="36" t="n"/>
+      <c r="E65" s="36" t="n"/>
+      <c r="F65" s="34" t="n"/>
+    </row>
+    <row r="66" ht="30" customHeight="1">
+      <c r="A66" s="24" t="inlineStr">
+        <is>
+          <t>THE LEVEL GAP.  The agent's classification names a platform control level and a monitoring level that an agent in it requires. Where the level applied is lower, the gap is accepted here, by name, or it is not accepted at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="30" customHeight="1">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>Platform control level the classification requires, and the level applied</t>
+        </is>
+      </c>
+      <c r="B67" s="15" t="n"/>
+      <c r="C67" s="35" t="n"/>
+      <c r="D67" s="36" t="n"/>
+      <c r="E67" s="36" t="n"/>
+      <c r="F67" s="34" t="n"/>
+    </row>
+    <row r="68" ht="30" customHeight="1">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>Monitoring level the classification requires, and the level applied</t>
+        </is>
+      </c>
+      <c r="B68" s="15" t="n"/>
+      <c r="C68" s="35" t="n"/>
+      <c r="D68" s="36" t="n"/>
+      <c r="E68" s="36" t="n"/>
+      <c r="F68" s="34" t="n"/>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>Who accepts the gap, by name</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="n"/>
+      <c r="C69" s="35" t="n"/>
+      <c r="D69" s="36" t="n"/>
+      <c r="E69" s="36" t="n"/>
+      <c r="F69" s="34" t="n"/>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="10" t="inlineStr">
+        <is>
+          <t>The date by which it closes</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="n"/>
+      <c r="C70" s="35" t="n"/>
+      <c r="D70" s="36" t="n"/>
+      <c r="E70" s="36" t="n"/>
+      <c r="F70" s="34" t="n"/>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="10" t="inlineStr">
+        <is>
+          <t>How many consecutive sign-offs have accepted this same gap</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="n"/>
+      <c r="C71" s="35" t="n"/>
+      <c r="D71" s="36" t="n"/>
+      <c r="E71" s="36" t="n"/>
+      <c r="F71" s="34" t="n"/>
+    </row>
+    <row r="72" ht="26" customHeight="1">
+      <c r="A72" s="13" t="inlineStr">
         <is>
           <t>Answer the last row honestly. A gap accepted once is a legitimate decision made under time pressure. A gap accepted three times in a row is a decision nobody is making, and this count is the only thing on any of these forms that would show it.</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="26" customHeight="1">
-      <c r="A62" s="32" t="n"/>
-      <c r="B62" s="32" t="n"/>
-      <c r="C62" s="32" t="n"/>
-      <c r="D62" s="32" t="n"/>
-      <c r="E62" s="32" t="n"/>
-      <c r="F62" s="32" t="n"/>
-    </row>
-    <row r="63" ht="26" customHeight="1">
-      <c r="A63" s="24" t="inlineStr">
+    <row r="73" ht="26" customHeight="1">
+      <c r="A73" s="32" t="n"/>
+      <c r="B73" s="32" t="n"/>
+      <c r="C73" s="32" t="n"/>
+      <c r="D73" s="32" t="n"/>
+      <c r="E73" s="32" t="n"/>
+      <c r="F73" s="32" t="n"/>
+    </row>
+    <row r="74" ht="26" customHeight="1">
+      <c r="A74" s="24" t="inlineStr">
         <is>
           <t>The sign-off is against the two versions named above. When live behavior stops matching the description it was granted against, it is void until somebody looks again.</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="26" customHeight="1">
-      <c r="A64" s="32" t="n"/>
-      <c r="B64" s="32" t="n"/>
-      <c r="C64" s="32" t="n"/>
-      <c r="D64" s="32" t="n"/>
-      <c r="E64" s="32" t="n"/>
-      <c r="F64" s="32" t="n"/>
-    </row>
-    <row r="65" ht="22" customHeight="1">
-      <c r="A65" s="9" t="inlineStr">
+    <row r="75" ht="26" customHeight="1">
+      <c r="A75" s="32" t="n"/>
+      <c r="B75" s="32" t="n"/>
+      <c r="C75" s="32" t="n"/>
+      <c r="D75" s="32" t="n"/>
+      <c r="E75" s="32" t="n"/>
+      <c r="F75" s="32" t="n"/>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="9" t="inlineStr">
         <is>
           <t>D.  Revision history</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="28" customHeight="1">
-      <c r="A66" s="14" t="inlineStr">
+    <row r="77" ht="28" customHeight="1">
+      <c r="A77" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B66" s="14" t="inlineStr">
+      <c r="B77" s="14" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="C66" s="14" t="inlineStr">
+      <c r="C77" s="14" t="inlineStr">
         <is>
           <t>What changed</t>
         </is>
       </c>
-      <c r="D66" s="14" t="inlineStr">
+      <c r="D77" s="14" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="E66" s="14" t="inlineStr">
+      <c r="E77" s="14" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="F66" s="14" t="inlineStr">
+      <c r="F77" s="14" t="inlineStr">
         <is>
           <t>Did it need a new sign-off</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="26" customHeight="1">
-      <c r="A67" s="35" t="n"/>
-      <c r="B67" s="35" t="n"/>
-      <c r="C67" s="35" t="n"/>
-      <c r="D67" s="35" t="n"/>
-      <c r="E67" s="35" t="n"/>
-      <c r="F67" s="35" t="n"/>
-    </row>
-    <row r="68" ht="26" customHeight="1">
-      <c r="A68" s="35" t="n"/>
-      <c r="B68" s="35" t="n"/>
-      <c r="C68" s="35" t="n"/>
-      <c r="D68" s="35" t="n"/>
-      <c r="E68" s="35" t="n"/>
-      <c r="F68" s="35" t="n"/>
-    </row>
-    <row r="69" ht="26" customHeight="1">
-      <c r="A69" s="35" t="n"/>
-      <c r="B69" s="35" t="n"/>
-      <c r="C69" s="35" t="n"/>
-      <c r="D69" s="35" t="n"/>
-      <c r="E69" s="35" t="n"/>
-      <c r="F69" s="35" t="n"/>
-    </row>
-    <row r="70" ht="26" customHeight="1">
-      <c r="A70" s="35" t="n"/>
-      <c r="B70" s="35" t="n"/>
-      <c r="C70" s="35" t="n"/>
-      <c r="D70" s="35" t="n"/>
-      <c r="E70" s="35" t="n"/>
-      <c r="F70" s="35" t="n"/>
-    </row>
-    <row r="71" ht="26" customHeight="1">
-      <c r="A71" s="35" t="n"/>
-      <c r="B71" s="35" t="n"/>
-      <c r="C71" s="35" t="n"/>
-      <c r="D71" s="35" t="n"/>
-      <c r="E71" s="35" t="n"/>
-      <c r="F71" s="35" t="n"/>
-    </row>
-    <row r="72" ht="26" customHeight="1">
-      <c r="A72" s="35" t="n"/>
-      <c r="B72" s="35" t="n"/>
-      <c r="C72" s="35" t="n"/>
-      <c r="D72" s="35" t="n"/>
-      <c r="E72" s="35" t="n"/>
-      <c r="F72" s="35" t="n"/>
-    </row>
-    <row r="73" ht="26" customHeight="1">
-      <c r="A73" s="35" t="n"/>
-      <c r="B73" s="35" t="n"/>
-      <c r="C73" s="35" t="n"/>
-      <c r="D73" s="35" t="n"/>
-      <c r="E73" s="35" t="n"/>
-      <c r="F73" s="35" t="n"/>
-    </row>
-    <row r="74" ht="26" customHeight="1">
-      <c r="A74" s="35" t="n"/>
-      <c r="B74" s="35" t="n"/>
-      <c r="C74" s="35" t="n"/>
-      <c r="D74" s="35" t="n"/>
-      <c r="E74" s="35" t="n"/>
-      <c r="F74" s="35" t="n"/>
-    </row>
-    <row r="75" ht="26" customHeight="1">
-      <c r="A75" s="35" t="n"/>
-      <c r="B75" s="35" t="n"/>
-      <c r="C75" s="35" t="n"/>
-      <c r="D75" s="35" t="n"/>
-      <c r="E75" s="35" t="n"/>
-      <c r="F75" s="35" t="n"/>
-    </row>
-    <row r="76" ht="26" customHeight="1">
-      <c r="A76" s="35" t="n"/>
-      <c r="B76" s="35" t="n"/>
-      <c r="C76" s="35" t="n"/>
-      <c r="D76" s="35" t="n"/>
-      <c r="E76" s="35" t="n"/>
-      <c r="F76" s="35" t="n"/>
-    </row>
-    <row r="77" ht="26" customHeight="1">
-      <c r="A77" s="13" t="inlineStr">
+    <row r="78" ht="26" customHeight="1">
+      <c r="A78" s="35" t="n"/>
+      <c r="B78" s="35" t="n"/>
+      <c r="C78" s="35" t="n"/>
+      <c r="D78" s="35" t="n"/>
+      <c r="E78" s="35" t="n"/>
+      <c r="F78" s="35" t="n"/>
+    </row>
+    <row r="79" ht="26" customHeight="1">
+      <c r="A79" s="35" t="n"/>
+      <c r="B79" s="35" t="n"/>
+      <c r="C79" s="35" t="n"/>
+      <c r="D79" s="35" t="n"/>
+      <c r="E79" s="35" t="n"/>
+      <c r="F79" s="35" t="n"/>
+    </row>
+    <row r="80" ht="26" customHeight="1">
+      <c r="A80" s="35" t="n"/>
+      <c r="B80" s="35" t="n"/>
+      <c r="C80" s="35" t="n"/>
+      <c r="D80" s="35" t="n"/>
+      <c r="E80" s="35" t="n"/>
+      <c r="F80" s="35" t="n"/>
+    </row>
+    <row r="81" ht="26" customHeight="1">
+      <c r="A81" s="35" t="n"/>
+      <c r="B81" s="35" t="n"/>
+      <c r="C81" s="35" t="n"/>
+      <c r="D81" s="35" t="n"/>
+      <c r="E81" s="35" t="n"/>
+      <c r="F81" s="35" t="n"/>
+    </row>
+    <row r="82" ht="26" customHeight="1">
+      <c r="A82" s="35" t="n"/>
+      <c r="B82" s="35" t="n"/>
+      <c r="C82" s="35" t="n"/>
+      <c r="D82" s="35" t="n"/>
+      <c r="E82" s="35" t="n"/>
+      <c r="F82" s="35" t="n"/>
+    </row>
+    <row r="83" ht="26" customHeight="1">
+      <c r="A83" s="35" t="n"/>
+      <c r="B83" s="35" t="n"/>
+      <c r="C83" s="35" t="n"/>
+      <c r="D83" s="35" t="n"/>
+      <c r="E83" s="35" t="n"/>
+      <c r="F83" s="35" t="n"/>
+    </row>
+    <row r="84" ht="26" customHeight="1">
+      <c r="A84" s="35" t="n"/>
+      <c r="B84" s="35" t="n"/>
+      <c r="C84" s="35" t="n"/>
+      <c r="D84" s="35" t="n"/>
+      <c r="E84" s="35" t="n"/>
+      <c r="F84" s="35" t="n"/>
+    </row>
+    <row r="85" ht="26" customHeight="1">
+      <c r="A85" s="35" t="n"/>
+      <c r="B85" s="35" t="n"/>
+      <c r="C85" s="35" t="n"/>
+      <c r="D85" s="35" t="n"/>
+      <c r="E85" s="35" t="n"/>
+      <c r="F85" s="35" t="n"/>
+    </row>
+    <row r="86" ht="26" customHeight="1">
+      <c r="A86" s="35" t="n"/>
+      <c r="B86" s="35" t="n"/>
+      <c r="C86" s="35" t="n"/>
+      <c r="D86" s="35" t="n"/>
+      <c r="E86" s="35" t="n"/>
+      <c r="F86" s="35" t="n"/>
+    </row>
+    <row r="87" ht="26" customHeight="1">
+      <c r="A87" s="35" t="n"/>
+      <c r="B87" s="35" t="n"/>
+      <c r="C87" s="35" t="n"/>
+      <c r="D87" s="35" t="n"/>
+      <c r="E87" s="35" t="n"/>
+      <c r="F87" s="35" t="n"/>
+    </row>
+    <row r="88" ht="26" customHeight="1">
+      <c r="A88" s="13" t="inlineStr">
         <is>
           <t>A model version bump, a framework upgrade, a new tool, or a change of host all produce a row. Answer the last column every time, because an auditor will ask which changes went live without a fresh sign-off.</t>
         </is>
@@ -3554,107 +3701,122 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="94">
+  <mergeCells count="109">
     <mergeCell ref="C52:F52"/>
+    <mergeCell ref="C61:F61"/>
     <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A66:F66"/>
     <mergeCell ref="A51:B51"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A70:B70"/>
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="A54:B54"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A41:B41"/>
     <mergeCell ref="A32:F32"/>
+    <mergeCell ref="C62:F62"/>
     <mergeCell ref="C15:F15"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A72:F72"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A31:F31"/>
     <mergeCell ref="C54:F54"/>
+    <mergeCell ref="C63:F63"/>
     <mergeCell ref="C10:F10"/>
-    <mergeCell ref="C41:F41"/>
-    <mergeCell ref="C50:F50"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C56:F56"/>
-    <mergeCell ref="C43:F43"/>
+    <mergeCell ref="A64:F64"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A62:B62"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="A28:B28"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A48:B48"/>
     <mergeCell ref="A59:B59"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="C67:F67"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C69:F69"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="C14:F14"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A71:B71"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="C40:F40"/>
     <mergeCell ref="A52:B52"/>
+    <mergeCell ref="A63:B63"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A61:F61"/>
-    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A88:F88"/>
+    <mergeCell ref="C71:F71"/>
+    <mergeCell ref="A46:F46"/>
     <mergeCell ref="C8:F8"/>
     <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A74:F74"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A26:F26"/>
     <mergeCell ref="C57:F57"/>
+    <mergeCell ref="A69:B69"/>
     <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="A76:F76"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="C68:F68"/>
     <mergeCell ref="A53:F53"/>
     <mergeCell ref="C58:F58"/>
+    <mergeCell ref="D33:F33"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A63:F63"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C45:F45"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A57:B57"/>
     <mergeCell ref="C20:F20"/>
-    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="D35:F35"/>
     <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C65:F65"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="C47:F47"/>
     <mergeCell ref="A39:F39"/>
-    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="C44:F44"/>
     <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A43:B43"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="C12:F12"/>
-    <mergeCell ref="A45:F45"/>
-    <mergeCell ref="C46:F46"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="D36:F36"/>
     <mergeCell ref="C51:F51"/>
     <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A67:B67"/>
     <mergeCell ref="C60:F60"/>
-    <mergeCell ref="A65:F65"/>
-    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="C70:F70"/>
     <mergeCell ref="C48:F48"/>
+    <mergeCell ref="C23:F23"/>
     <mergeCell ref="A60:B60"/>
+    <mergeCell ref="C7:F7"/>
     <mergeCell ref="C38:F38"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A25:B25"/>
     <mergeCell ref="C49:F49"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="C33:F33"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A43:F43"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="C16:F16"/>
-    <mergeCell ref="A77:F77"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="A20:B20"/>
     <mergeCell ref="C9:F9"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A29:B29"/>
     <mergeCell ref="C59:F59"/>
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="C11:F11"/>
     <mergeCell ref="A58:B58"/>
-    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C16 C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Level 1,Level 2,Level 3"</formula1>
     </dataValidation>
-    <dataValidation sqref="F67:F76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F78:F87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3677,7 +3839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3812,7 +3974,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Who owns this monitoring</t>
+          <t>Version of the Monitoring Levels this score was made against</t>
         </is>
       </c>
       <c r="B13" s="15" t="n"/>
@@ -3821,61 +3983,61 @@
       <c r="E13" s="36" t="n"/>
       <c r="F13" s="34" t="n"/>
     </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Who owns this monitoring</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="36" t="n"/>
+      <c r="E14" s="36" t="n"/>
+      <c r="F14" s="34" t="n"/>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Where the level applied is lower than the level the classification requires, the gap is accepted in section C of the Platform &amp; Sign-off sheet, not here. This sheet records what is true; that one records who accepted it.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="32" t="n"/>
-      <c r="B15" s="32" t="n"/>
-      <c r="C15" s="32" t="n"/>
-      <c r="D15" s="32" t="n"/>
-      <c r="E15" s="32" t="n"/>
-      <c r="F15" s="32" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="32" t="n"/>
+      <c r="B16" s="32" t="n"/>
+      <c r="C16" s="32" t="n"/>
+      <c r="D16" s="32" t="n"/>
+      <c r="E16" s="32" t="n"/>
+      <c r="F16" s="32" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>What you record</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>Do you record it</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>Where it goes</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>How long you keep it</t>
         </is>
       </c>
-      <c r="E16" s="16" t="n"/>
-      <c r="F16" s="15" t="n"/>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="25" t="inlineStr">
-        <is>
-          <t>Every tool call, and its arguments</t>
-        </is>
-      </c>
-      <c r="B17" s="35" t="n"/>
-      <c r="C17" s="35" t="n"/>
-      <c r="D17" s="35" t="n"/>
-      <c r="E17" s="36" t="n"/>
-      <c r="F17" s="34" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="15" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>Inputs to the run</t>
+          <t>Every tool call, and its arguments</t>
         </is>
       </c>
       <c r="B18" s="35" t="n"/>
@@ -3887,7 +4049,7 @@
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>Outputs of the run</t>
+          <t>Inputs to the run</t>
         </is>
       </c>
       <c r="B19" s="35" t="n"/>
@@ -3899,7 +4061,7 @@
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>The prompt and context as sent</t>
+          <t>Outputs of the run</t>
         </is>
       </c>
       <c r="B20" s="35" t="n"/>
@@ -3911,7 +4073,7 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>The agent's steps between the request and the answer</t>
+          <t>The prompt and context as sent</t>
         </is>
       </c>
       <c r="B21" s="35" t="n"/>
@@ -3923,7 +4085,7 @@
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>Escalations to a person, and the outcome</t>
+          <t>The agent's steps between the request and the answer</t>
         </is>
       </c>
       <c r="B22" s="35" t="n"/>
@@ -3935,7 +4097,7 @@
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>Enough of the run to replay it</t>
+          <t>Escalations to a person, and the outcome</t>
         </is>
       </c>
       <c r="B23" s="35" t="n"/>
@@ -3947,7 +4109,7 @@
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>Cost and token use per run</t>
+          <t>Enough of the run to replay it</t>
         </is>
       </c>
       <c r="B24" s="35" t="n"/>
@@ -3956,83 +4118,83 @@
       <c r="E24" s="36" t="n"/>
       <c r="F24" s="34" t="n"/>
     </row>
-    <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="32" t="n"/>
-      <c r="B25" s="32" t="n"/>
-      <c r="C25" s="32" t="n"/>
-      <c r="D25" s="32" t="n"/>
-      <c r="E25" s="32" t="n"/>
-      <c r="F25" s="32" t="n"/>
-    </row>
-    <row r="26" ht="56" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="25" t="inlineStr">
+        <is>
+          <t>Cost and token use per run</t>
+        </is>
+      </c>
+      <c r="B25" s="35" t="n"/>
+      <c r="C25" s="35" t="n"/>
+      <c r="D25" s="35" t="n"/>
+      <c r="E25" s="36" t="n"/>
+      <c r="F25" s="34" t="n"/>
+    </row>
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="32" t="n"/>
+      <c r="B26" s="32" t="n"/>
+      <c r="C26" s="32" t="n"/>
+      <c r="D26" s="32" t="n"/>
+      <c r="E26" s="32" t="n"/>
+      <c r="F26" s="32" t="n"/>
+    </row>
+    <row r="27" ht="56" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>What you deliberately do NOT record, and why</t>
         </is>
       </c>
-      <c r="B26" s="15" t="n"/>
-      <c r="C26" s="35" t="n"/>
-      <c r="D26" s="36" t="n"/>
-      <c r="E26" s="36" t="n"/>
-      <c r="F26" s="34" t="n"/>
-    </row>
-    <row r="27" ht="13" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="B27" s="15" t="n"/>
+      <c r="C27" s="35" t="n"/>
+      <c r="D27" s="36" t="n"/>
+      <c r="E27" s="36" t="n"/>
+      <c r="F27" s="34" t="n"/>
+    </row>
+    <row r="28" ht="13" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>Usually personal data you have no basis to retain. Say what you lose by not recording it.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="56" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
+    <row r="29" ht="56" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>Who can read these records, and who can change them</t>
         </is>
       </c>
-      <c r="B28" s="15" t="n"/>
-      <c r="C28" s="35" t="n"/>
-      <c r="D28" s="36" t="n"/>
-      <c r="E28" s="36" t="n"/>
-      <c r="F28" s="34" t="n"/>
-    </row>
-    <row r="29" ht="13" customHeight="1">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="B29" s="15" t="n"/>
+      <c r="C29" s="35" t="n"/>
+      <c r="D29" s="36" t="n"/>
+      <c r="E29" s="36" t="n"/>
+      <c r="F29" s="34" t="n"/>
+    </row>
+    <row r="30" ht="13" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>If the team that operates the agent can edit its own logs, say so here. Stage 5 needs records an auditor will accept.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="32" t="n"/>
-      <c r="B30" s="32" t="n"/>
-      <c r="C30" s="32" t="n"/>
-      <c r="D30" s="32" t="n"/>
-      <c r="E30" s="32" t="n"/>
-      <c r="F30" s="32" t="n"/>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="32" t="n"/>
+      <c r="B31" s="32" t="n"/>
+      <c r="C31" s="32" t="n"/>
+      <c r="D31" s="32" t="n"/>
+      <c r="E31" s="32" t="n"/>
+      <c r="F31" s="32" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>B.  The evals, and what runs them</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="56" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
+    <row r="33" ht="56" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>Which evals run against the live agent</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="n"/>
-      <c r="C32" s="35" t="n"/>
-      <c r="D32" s="36" t="n"/>
-      <c r="E32" s="36" t="n"/>
-      <c r="F32" s="34" t="n"/>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>What starts them</t>
         </is>
       </c>
       <c r="B33" s="15" t="n"/>
@@ -4041,29 +4203,29 @@
       <c r="E33" s="36" t="n"/>
       <c r="F33" s="34" t="n"/>
     </row>
-    <row r="34" ht="13" customHeight="1">
-      <c r="A34" s="13" t="inlineStr">
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>What starts them</t>
+        </is>
+      </c>
+      <c r="B34" s="15" t="n"/>
+      <c r="C34" s="35" t="n"/>
+      <c r="D34" s="36" t="n"/>
+      <c r="E34" s="36" t="n"/>
+      <c r="F34" s="34" t="n"/>
+    </row>
+    <row r="35" ht="13" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
         <is>
           <t>A schedule, a deployment, live traffic, or a person. An eval a person has to remember to run is not assurance.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="56" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
+    <row r="36" ht="56" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>How often, or what share of live traffic if they run continuously</t>
-        </is>
-      </c>
-      <c r="B35" s="15" t="n"/>
-      <c r="C35" s="35" t="n"/>
-      <c r="D35" s="36" t="n"/>
-      <c r="E35" s="36" t="n"/>
-      <c r="F35" s="34" t="n"/>
-    </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>Where the results go</t>
         </is>
       </c>
       <c r="B36" s="15" t="n"/>
@@ -4075,7 +4237,7 @@
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>Who is told when one fails</t>
+          <t>Where the results go</t>
         </is>
       </c>
       <c r="B37" s="15" t="n"/>
@@ -4087,7 +4249,7 @@
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>Who owns extending the eval set as the agent changes</t>
+          <t>Who is told when one fails</t>
         </is>
       </c>
       <c r="B38" s="15" t="n"/>
@@ -4096,10 +4258,10 @@
       <c r="E38" s="36" t="n"/>
       <c r="F38" s="34" t="n"/>
     </row>
-    <row r="39" ht="56" customHeight="1">
+    <row r="39" ht="30" customHeight="1">
       <c r="A39" s="10" t="inlineStr">
         <is>
-          <t>How you would know they had stopped running</t>
+          <t>Who owns extending the eval set as the agent changes</t>
         </is>
       </c>
       <c r="B39" s="15" t="n"/>
@@ -4108,91 +4270,91 @@
       <c r="E39" s="36" t="n"/>
       <c r="F39" s="34" t="n"/>
     </row>
-    <row r="40" ht="13" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
+    <row r="40" ht="56" customHeight="1">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>How you would know they had stopped running</t>
+        </is>
+      </c>
+      <c r="B40" s="15" t="n"/>
+      <c r="C40" s="35" t="n"/>
+      <c r="D40" s="36" t="n"/>
+      <c r="E40" s="36" t="n"/>
+      <c r="F40" s="34" t="n"/>
+    </row>
+    <row r="41" ht="13" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
         <is>
           <t>A dead scheduler and a continuous job that quietly stopped look the same from outside: everything is green because nothing is running.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="56" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
+    <row r="42" ht="56" customHeight="1">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>Which baseline the results are compared against</t>
         </is>
       </c>
-      <c r="B41" s="15" t="n"/>
-      <c r="C41" s="35" t="n"/>
-      <c r="D41" s="36" t="n"/>
-      <c r="E41" s="36" t="n"/>
-      <c r="F41" s="34" t="n"/>
-    </row>
-    <row r="42" ht="13" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="B42" s="15" t="n"/>
+      <c r="C42" s="35" t="n"/>
+      <c r="D42" s="36" t="n"/>
+      <c r="E42" s="36" t="n"/>
+      <c r="F42" s="34" t="n"/>
+    </row>
+    <row r="43" ht="13" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>Normally the eval results recorded at sign-off. Name the version.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="32" t="n"/>
-      <c r="B43" s="32" t="n"/>
-      <c r="C43" s="32" t="n"/>
-      <c r="D43" s="32" t="n"/>
-      <c r="E43" s="32" t="n"/>
-      <c r="F43" s="32" t="n"/>
-    </row>
-    <row r="44" ht="22" customHeight="1">
-      <c r="A44" s="9" t="inlineStr">
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="32" t="n"/>
+      <c r="B44" s="32" t="n"/>
+      <c r="C44" s="32" t="n"/>
+      <c r="D44" s="32" t="n"/>
+      <c r="E44" s="32" t="n"/>
+      <c r="F44" s="32" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="9" t="inlineStr">
         <is>
           <t>C.  What counts as normal, and what starts an alert</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="14" t="inlineStr">
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="B45" s="14" t="inlineStr">
+      <c r="B46" s="14" t="inlineStr">
         <is>
           <t>What normal looks like</t>
         </is>
       </c>
-      <c r="C45" s="14" t="inlineStr">
+      <c r="C46" s="14" t="inlineStr">
         <is>
           <t>What starts an alert</t>
         </is>
       </c>
-      <c r="D45" s="14" t="inlineStr">
+      <c r="D46" s="14" t="inlineStr">
         <is>
           <t>Who receives it</t>
         </is>
       </c>
-      <c r="E45" s="14" t="inlineStr">
+      <c r="E46" s="14" t="inlineStr">
         <is>
           <t>Implemented today</t>
         </is>
       </c>
-      <c r="F45" s="15" t="n"/>
-    </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="25" t="inlineStr">
-        <is>
-          <t>A call to a tool outside the declared set</t>
-        </is>
-      </c>
-      <c r="B46" s="35" t="n"/>
-      <c r="C46" s="35" t="n"/>
-      <c r="D46" s="35" t="n"/>
-      <c r="E46" s="35" t="n"/>
-      <c r="F46" s="34" t="n"/>
+      <c r="F46" s="15" t="n"/>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>Volume of runs</t>
+          <t>A call to a tool outside the declared set</t>
         </is>
       </c>
       <c r="B47" s="35" t="n"/>
@@ -4204,7 +4366,7 @@
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>Escalation rate to a person</t>
+          <t>Volume of runs</t>
         </is>
       </c>
       <c r="B48" s="35" t="n"/>
@@ -4216,7 +4378,7 @@
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>Eval failure</t>
+          <t>Escalation rate to a person</t>
         </is>
       </c>
       <c r="B49" s="35" t="n"/>
@@ -4228,7 +4390,7 @@
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>Cost per run or per day</t>
+          <t>Eval failure</t>
         </is>
       </c>
       <c r="B50" s="35" t="n"/>
@@ -4240,7 +4402,7 @@
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>Error or retry rate</t>
+          <t>Cost per run or per day</t>
         </is>
       </c>
       <c r="B51" s="35" t="n"/>
@@ -4252,7 +4414,7 @@
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>Drift from the design document</t>
+          <t>Error or retry rate</t>
         </is>
       </c>
       <c r="B52" s="35" t="n"/>
@@ -4262,75 +4424,75 @@
       <c r="F52" s="34" t="n"/>
     </row>
     <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="37" t="n"/>
+      <c r="A53" s="25" t="inlineStr">
+        <is>
+          <t>Drift from the design document</t>
+        </is>
+      </c>
       <c r="B53" s="35" t="n"/>
       <c r="C53" s="35" t="n"/>
       <c r="D53" s="35" t="n"/>
       <c r="E53" s="35" t="n"/>
       <c r="F53" s="34" t="n"/>
     </row>
-    <row r="54" ht="39" customHeight="1">
-      <c r="A54" s="13" t="inlineStr">
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="37" t="n"/>
+      <c r="B54" s="35" t="n"/>
+      <c r="C54" s="35" t="n"/>
+      <c r="D54" s="35" t="n"/>
+      <c r="E54" s="35" t="n"/>
+      <c r="F54" s="34" t="n"/>
+    </row>
+    <row r="55" ht="39" customHeight="1">
+      <c r="A55" s="13" t="inlineStr">
         <is>
           <t>Answer the last column for what is implemented today, not what is planned. A row with nothing behind it is a gap the sign-off has to carry. The first row needs the section 3 grant list in a form the monitor can read. It is the only machine-checkable claim in the framework, and naming where the monitor gets it is the difference between an alert you can build and one you intend to.</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="32" t="n"/>
-      <c r="B55" s="32" t="n"/>
-      <c r="C55" s="32" t="n"/>
-      <c r="D55" s="32" t="n"/>
-      <c r="E55" s="32" t="n"/>
-      <c r="F55" s="32" t="n"/>
-    </row>
-    <row r="56" ht="22" customHeight="1">
-      <c r="A56" s="9" t="inlineStr">
+    <row r="56" ht="26" customHeight="1">
+      <c r="A56" s="32" t="n"/>
+      <c r="B56" s="32" t="n"/>
+      <c r="C56" s="32" t="n"/>
+      <c r="D56" s="32" t="n"/>
+      <c r="E56" s="32" t="n"/>
+      <c r="F56" s="32" t="n"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="9" t="inlineStr">
         <is>
           <t>D.  What an alert starts</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="14" t="inlineStr">
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="B57" s="14" t="inlineStr">
+      <c r="B58" s="14" t="inlineStr">
         <is>
           <t>What happens</t>
         </is>
       </c>
-      <c r="C57" s="15" t="n"/>
-      <c r="D57" s="14" t="inlineStr">
+      <c r="C58" s="15" t="n"/>
+      <c r="D58" s="14" t="inlineStr">
         <is>
           <t>Who does it</t>
         </is>
       </c>
-      <c r="E57" s="14" t="inlineStr">
+      <c r="E58" s="14" t="inlineStr">
         <is>
           <t>Within what time</t>
         </is>
       </c>
-      <c r="F57" s="15" t="n"/>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="25" t="inlineStr">
-        <is>
-          <t>Triage: is this real</t>
-        </is>
-      </c>
-      <c r="B58" s="35" t="n"/>
-      <c r="C58" s="34" t="n"/>
-      <c r="D58" s="35" t="n"/>
-      <c r="E58" s="35" t="n"/>
-      <c r="F58" s="34" t="n"/>
+      <c r="F58" s="15" t="n"/>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>Contain: stop or narrow the agent</t>
+          <t>Triage: is this real</t>
         </is>
       </c>
       <c r="B59" s="35" t="n"/>
@@ -4342,7 +4504,7 @@
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>Review the run records</t>
+          <t>Contain: stop or narrow the agent</t>
         </is>
       </c>
       <c r="B60" s="35" t="n"/>
@@ -4354,7 +4516,7 @@
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Review the run records</t>
         </is>
       </c>
       <c r="B61" s="35" t="n"/>
@@ -4366,7 +4528,7 @@
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>Tell the people affected</t>
+          <t>Fix</t>
         </is>
       </c>
       <c r="B62" s="35" t="n"/>
@@ -4378,7 +4540,7 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>Decide whether anybody outside has to be told, and start that clock</t>
+          <t>Tell the people affected</t>
         </is>
       </c>
       <c r="B63" s="35" t="n"/>
@@ -4390,7 +4552,7 @@
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="25" t="inlineStr">
         <is>
-          <t>Review after the incident</t>
+          <t>Decide whether anybody outside has to be told, and start that clock</t>
         </is>
       </c>
       <c r="B64" s="35" t="n"/>
@@ -4402,7 +4564,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="25" t="inlineStr">
         <is>
-          <t>Decide whether the agent resumes, and whether the sign-off still holds</t>
+          <t>Review after the incident</t>
         </is>
       </c>
       <c r="B65" s="35" t="n"/>
@@ -4411,130 +4573,126 @@
       <c r="E65" s="35" t="n"/>
       <c r="F65" s="34" t="n"/>
     </row>
-    <row r="66" ht="26" customHeight="1">
-      <c r="A66" s="13" t="inlineStr">
-        <is>
-          <t>For an agent inside a regulated process, notifying a regulator or a data-protection authority runs on a clock that starts well before the fix is finished. Stage 2 classifies agents on whether a mistake is reportable, so somebody has to decide here whether this one is.</t>
-        </is>
-      </c>
+    <row r="66" ht="30" customHeight="1">
+      <c r="A66" s="25" t="inlineStr">
+        <is>
+          <t>Decide whether the agent resumes, and whether the sign-off still holds</t>
+        </is>
+      </c>
+      <c r="B66" s="35" t="n"/>
+      <c r="C66" s="34" t="n"/>
+      <c r="D66" s="35" t="n"/>
+      <c r="E66" s="35" t="n"/>
+      <c r="F66" s="34" t="n"/>
     </row>
     <row r="67" ht="26" customHeight="1">
       <c r="A67" s="13" t="inlineStr">
         <is>
+          <t>For an agent inside a regulated process, notifying a regulator or a data-protection authority runs on a clock that starts well before the fix is finished. Stage 2 classifies agents on whether a mistake is reportable, so somebody has to decide here whether this one is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="26" customHeight="1">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
           <t>The stage 3 sign-off is void once live behavior stops matching what it was granted against, and an incident is that moment. Name who re-confirms it, or re-issues it, before the agent runs again.</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="26" customHeight="1">
-      <c r="A68" s="32" t="n"/>
-      <c r="B68" s="32" t="n"/>
-      <c r="C68" s="32" t="n"/>
-      <c r="D68" s="32" t="n"/>
-      <c r="E68" s="32" t="n"/>
-      <c r="F68" s="32" t="n"/>
-    </row>
-    <row r="69" ht="56" customHeight="1">
-      <c r="A69" s="10" t="inlineStr">
+    <row r="69" ht="26" customHeight="1">
+      <c r="A69" s="32" t="n"/>
+      <c r="B69" s="32" t="n"/>
+      <c r="C69" s="32" t="n"/>
+      <c r="D69" s="32" t="n"/>
+      <c r="E69" s="32" t="n"/>
+      <c r="F69" s="32" t="n"/>
+    </row>
+    <row r="70" ht="56" customHeight="1">
+      <c r="A70" s="10" t="inlineStr">
         <is>
           <t>How the agent is stopped, and by whom</t>
         </is>
       </c>
-      <c r="B69" s="15" t="n"/>
-      <c r="C69" s="35" t="n"/>
-      <c r="D69" s="36" t="n"/>
-      <c r="E69" s="36" t="n"/>
-      <c r="F69" s="34" t="n"/>
-    </row>
-    <row r="70" ht="13" customHeight="1">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="B70" s="15" t="n"/>
+      <c r="C70" s="35" t="n"/>
+      <c r="D70" s="36" t="n"/>
+      <c r="E70" s="36" t="n"/>
+      <c r="F70" s="34" t="n"/>
+    </row>
+    <row r="71" ht="13" customHeight="1">
+      <c r="A71" s="13" t="inlineStr">
         <is>
           <t>Point at section 5 of the design document rather than restating it. Say who is on call.</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="56" customHeight="1">
-      <c r="A71" s="10" t="inlineStr">
+    <row r="72" ht="56" customHeight="1">
+      <c r="A72" s="10" t="inlineStr">
         <is>
           <t>What you tell a customer, and who decides</t>
         </is>
       </c>
-      <c r="B71" s="15" t="n"/>
-      <c r="C71" s="35" t="n"/>
-      <c r="D71" s="36" t="n"/>
-      <c r="E71" s="36" t="n"/>
-      <c r="F71" s="34" t="n"/>
-    </row>
-    <row r="72" ht="13" customHeight="1">
-      <c r="A72" s="13" t="inlineStr">
-        <is>
-          <t>For any agent where the person on the other end is not internal staff.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="26" customHeight="1">
-      <c r="A73" s="32" t="n"/>
-      <c r="B73" s="32" t="n"/>
-      <c r="C73" s="32" t="n"/>
-      <c r="D73" s="32" t="n"/>
-      <c r="E73" s="32" t="n"/>
-      <c r="F73" s="32" t="n"/>
-    </row>
-    <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="9" t="inlineStr">
+      <c r="B72" s="15" t="n"/>
+      <c r="C72" s="35" t="n"/>
+      <c r="D72" s="36" t="n"/>
+      <c r="E72" s="36" t="n"/>
+      <c r="F72" s="34" t="n"/>
+    </row>
+    <row r="73" ht="13" customHeight="1">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>For any agent where the person on the other end is not internal staff. Say also how that person challenges the outcome, pointing at section 5 of the design document rather than restating it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="26" customHeight="1">
+      <c r="A74" s="32" t="n"/>
+      <c r="B74" s="32" t="n"/>
+      <c r="C74" s="32" t="n"/>
+      <c r="D74" s="32" t="n"/>
+      <c r="E74" s="32" t="n"/>
+      <c r="F74" s="32" t="n"/>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="9" t="inlineStr">
         <is>
           <t>E.  What goes wrong, and what you do about it</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="38" customHeight="1">
-      <c r="A75" s="13" t="inlineStr">
+    <row r="76" ht="38" customHeight="1">
+      <c r="A76" s="13" t="inlineStr">
         <is>
           <t>Agents fail in ways ordinary software does not. Write what you would do, or write "not covered" and let the sign-off carry it. Where a row does not apply, write "the agent cannot do this" rather than leaving it blank. Drawn from the OWASP Top 10 for Agentic Applications; the OWASP column names the entry each row comes from.</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="30" customHeight="1">
-      <c r="A76" s="14" t="inlineStr">
+    <row r="77" ht="30" customHeight="1">
+      <c r="A77" s="14" t="inlineStr">
         <is>
           <t>What goes wrong</t>
         </is>
       </c>
-      <c r="B76" s="14" t="inlineStr">
+      <c r="B77" s="14" t="inlineStr">
         <is>
           <t>OWASP</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>What you do</t>
         </is>
       </c>
-    </row>
-    <row r="77" ht="30" customHeight="1">
-      <c r="A77" s="25" t="inlineStr">
-        <is>
-          <t>The agent calls a tool outside its declared set</t>
-        </is>
-      </c>
-      <c r="B77" s="25" t="inlineStr">
-        <is>
-          <t>ASI02, ASI03</t>
-        </is>
-      </c>
-      <c r="C77" s="32" t="n"/>
-      <c r="D77" s="32" t="n"/>
-      <c r="E77" s="32" t="n"/>
-      <c r="F77" s="32" t="n"/>
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="25" t="inlineStr">
         <is>
-          <t>A chain of tool calls each succeeds but the outcome is wrong</t>
+          <t>The agent calls a tool outside its declared set</t>
         </is>
       </c>
       <c r="B78" s="25" t="inlineStr">
         <is>
-          <t>ASI08</t>
+          <t>ASI02, ASI03</t>
         </is>
       </c>
       <c r="C78" s="32" t="n"/>
@@ -4545,12 +4703,12 @@
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="25" t="inlineStr">
         <is>
-          <t>Prompt injection through content the agent reads</t>
+          <t>A chain of tool calls each succeeds but the outcome is wrong</t>
         </is>
       </c>
       <c r="B79" s="25" t="inlineStr">
         <is>
-          <t>ASI01</t>
+          <t>ASI08</t>
         </is>
       </c>
       <c r="C79" s="32" t="n"/>
@@ -4561,12 +4719,12 @@
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="25" t="inlineStr">
         <is>
-          <t>Scope creep: used for work it was not designed for</t>
+          <t>Prompt injection through content the agent reads</t>
         </is>
       </c>
       <c r="B80" s="25" t="inlineStr">
         <is>
-          <t>ASI09</t>
+          <t>ASI01</t>
         </is>
       </c>
       <c r="C80" s="32" t="n"/>
@@ -4577,12 +4735,12 @@
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="25" t="inlineStr">
         <is>
-          <t>The agent loops, or runs away on cost</t>
+          <t>Scope creep: used for work it was not designed for</t>
         </is>
       </c>
       <c r="B81" s="25" t="inlineStr">
         <is>
-          <t>ASI08</t>
+          <t>ASI09</t>
         </is>
       </c>
       <c r="C81" s="32" t="n"/>
@@ -4593,12 +4751,12 @@
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="25" t="inlineStr">
         <is>
-          <t>A model or framework update changes behavior with no code change</t>
+          <t>The agent loops, or runs away on cost</t>
         </is>
       </c>
       <c r="B82" s="25" t="inlineStr">
         <is>
-          <t>ASI04</t>
+          <t>ASI08</t>
         </is>
       </c>
       <c r="C82" s="32" t="n"/>
@@ -4609,12 +4767,12 @@
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="25" t="inlineStr">
         <is>
-          <t>Memory or retrieved context has been poisoned</t>
+          <t>A model or framework update changes behavior with no code change</t>
         </is>
       </c>
       <c r="B83" s="25" t="inlineStr">
         <is>
-          <t>ASI06</t>
+          <t>ASI04</t>
         </is>
       </c>
       <c r="C83" s="32" t="n"/>
@@ -4625,12 +4783,12 @@
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="25" t="inlineStr">
         <is>
-          <t>The agent is confidently wrong and a person acts on it</t>
+          <t>Memory or retrieved context has been poisoned</t>
         </is>
       </c>
       <c r="B84" s="25" t="inlineStr">
         <is>
-          <t>ASI09</t>
+          <t>ASI06</t>
         </is>
       </c>
       <c r="C84" s="32" t="n"/>
@@ -4641,7 +4799,7 @@
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="25" t="inlineStr">
         <is>
-          <t>The agent stops escalating when it should</t>
+          <t>The agent is confidently wrong and a person acts on it</t>
         </is>
       </c>
       <c r="B85" s="25" t="inlineStr">
@@ -4657,12 +4815,12 @@
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="25" t="inlineStr">
         <is>
-          <t>The agent runs code or shell commands it composed itself</t>
+          <t>The agent stops escalating when it should</t>
         </is>
       </c>
       <c r="B86" s="25" t="inlineStr">
         <is>
-          <t>ASI05</t>
+          <t>ASI09</t>
         </is>
       </c>
       <c r="C86" s="32" t="n"/>
@@ -4673,12 +4831,12 @@
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="25" t="inlineStr">
         <is>
-          <t>A supervising agent fails, or supervises wrongly</t>
+          <t>The agent runs code or shell commands it composed itself</t>
         </is>
       </c>
       <c r="B87" s="25" t="inlineStr">
         <is>
-          <t>ASI07, ASI10</t>
+          <t>ASI05</t>
         </is>
       </c>
       <c r="C87" s="32" t="n"/>
@@ -4686,56 +4844,64 @@
       <c r="E87" s="32" t="n"/>
       <c r="F87" s="32" t="n"/>
     </row>
-    <row r="88" ht="26" customHeight="1">
-      <c r="A88" s="32" t="n"/>
-      <c r="B88" s="32" t="n"/>
+    <row r="88" ht="30" customHeight="1">
+      <c r="A88" s="25" t="inlineStr">
+        <is>
+          <t>A supervising agent fails, or supervises wrongly</t>
+        </is>
+      </c>
+      <c r="B88" s="25" t="inlineStr">
+        <is>
+          <t>ASI07, ASI10</t>
+        </is>
+      </c>
       <c r="C88" s="32" t="n"/>
       <c r="D88" s="32" t="n"/>
       <c r="E88" s="32" t="n"/>
       <c r="F88" s="32" t="n"/>
     </row>
-    <row r="89" ht="22" customHeight="1">
-      <c r="A89" s="9" t="inlineStr">
+    <row r="89" ht="26" customHeight="1">
+      <c r="A89" s="32" t="n"/>
+      <c r="B89" s="32" t="n"/>
+      <c r="C89" s="32" t="n"/>
+      <c r="D89" s="32" t="n"/>
+      <c r="E89" s="32" t="n"/>
+      <c r="F89" s="32" t="n"/>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="9" t="inlineStr">
         <is>
           <t>F.  Revision history</t>
         </is>
       </c>
     </row>
-    <row r="90" ht="30" customHeight="1">
-      <c r="A90" s="14" t="inlineStr">
+    <row r="91" ht="30" customHeight="1">
+      <c r="A91" s="14" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B90" s="14" t="inlineStr">
+      <c r="B91" s="14" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="C90" s="14" t="inlineStr">
+      <c r="C91" s="14" t="inlineStr">
         <is>
           <t>What changed</t>
         </is>
       </c>
-      <c r="D90" s="14" t="inlineStr">
+      <c r="D91" s="14" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="E90" s="14" t="inlineStr">
+      <c r="E91" s="14" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="F90" s="15" t="n"/>
-    </row>
-    <row r="91" ht="30" customHeight="1">
-      <c r="A91" s="35" t="n"/>
-      <c r="B91" s="35" t="n"/>
-      <c r="C91" s="35" t="n"/>
-      <c r="D91" s="35" t="n"/>
-      <c r="E91" s="35" t="n"/>
-      <c r="F91" s="34" t="n"/>
+      <c r="F91" s="15" t="n"/>
     </row>
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="35" t="n"/>
@@ -4793,129 +4959,139 @@
       <c r="E98" s="35" t="n"/>
       <c r="F98" s="34" t="n"/>
     </row>
+    <row r="99" ht="30" customHeight="1">
+      <c r="A99" s="35" t="n"/>
+      <c r="B99" s="35" t="n"/>
+      <c r="C99" s="35" t="n"/>
+      <c r="D99" s="35" t="n"/>
+      <c r="E99" s="35" t="n"/>
+      <c r="F99" s="34" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
-  <mergeCells count="114">
+  <mergeCells count="116">
+    <mergeCell ref="C39:F39"/>
+    <mergeCell ref="E62:F62"/>
+    <mergeCell ref="A75:F75"/>
+    <mergeCell ref="C72:F72"/>
+    <mergeCell ref="C81:F81"/>
+    <mergeCell ref="A70:B70"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="E64:F64"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="C78:F78"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C87:F87"/>
     <mergeCell ref="E63:F63"/>
-    <mergeCell ref="A67:F67"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="C82:F82"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="C38:F38"/>
-    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="A27:B27"/>
     <mergeCell ref="E65:F65"/>
-    <mergeCell ref="C13:F13"/>
-    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="E99:F99"/>
     <mergeCell ref="C79:F79"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="E64:F64"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C80:F80"/>
-    <mergeCell ref="D24:F24"/>
-    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="C88:F88"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="A42:B42"/>
     <mergeCell ref="C10:F10"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A74:F74"/>
-    <mergeCell ref="E92:F92"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="E94:F94"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A73:F73"/>
+    <mergeCell ref="E91:F91"/>
     <mergeCell ref="B64:C64"/>
+    <mergeCell ref="E53:F53"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="E93:F93"/>
+    <mergeCell ref="C27:F27"/>
     <mergeCell ref="A9:B9"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A41:F41"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="D17:F17"/>
-    <mergeCell ref="E49:F49"/>
-    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="C83:F83"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C40:F40"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="E66:F66"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="A90:F90"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="C82:F82"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="E52:F52"/>
+    <mergeCell ref="E92:F92"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="A71:F71"/>
+    <mergeCell ref="A76:F76"/>
+    <mergeCell ref="C77:F77"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="E94:F94"/>
+    <mergeCell ref="C86:F86"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="A68:F68"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="E95:F95"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="D20:F20"/>
     <mergeCell ref="C84:F84"/>
     <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="E91:F91"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C41:F41"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A89:F89"/>
-    <mergeCell ref="D22:F22"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="C77:F77"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C83:F83"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A75:F75"/>
-    <mergeCell ref="E53:F53"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="E93:F93"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="C80:F80"/>
+    <mergeCell ref="E54:F54"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="E96:F96"/>
+    <mergeCell ref="C70:F70"/>
+    <mergeCell ref="B62:C62"/>
     <mergeCell ref="B59:C59"/>
-    <mergeCell ref="A72:F72"/>
-    <mergeCell ref="C78:F78"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="E95:F95"/>
-    <mergeCell ref="C87:F87"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="C69:F69"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="A54:F54"/>
-    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="E98:F98"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="C38:F38"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="A4:F4"/>
     <mergeCell ref="E60:F60"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="E96:F96"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="E90:F90"/>
-    <mergeCell ref="E62:F62"/>
-    <mergeCell ref="D20:F20"/>
-    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="C42:F42"/>
+    <mergeCell ref="D24:F24"/>
+    <mergeCell ref="A43:F43"/>
+    <mergeCell ref="A67:F67"/>
     <mergeCell ref="C85:F85"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="C81:F81"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="E57:F57"/>
-    <mergeCell ref="E97:F97"/>
-    <mergeCell ref="A66:F66"/>
-    <mergeCell ref="C71:F71"/>
-    <mergeCell ref="B63:C63"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="C39:F39"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="C86:F86"/>
+    <mergeCell ref="B65:C65"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="D19:F19"/>
-    <mergeCell ref="C76:F76"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="A29:B29"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="E98:F98"/>
+    <mergeCell ref="E97:F97"/>
     <mergeCell ref="C11:F11"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A70:F70"/>
-    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="E47:F47"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C10 C11 C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Level 1,Level 2,Level 3"</formula1>
     </dataValidation>
-    <dataValidation sqref="B17:B24 E46:E53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B18:B25 E47:E54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Partly"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>